<commit_message>
Funding model: one regional funded 12M with coach, one unfunded
- Compare: B5 = 12M (4 ppl, funded), new B12 = 0 (3 ppl, unfunded); plan sheets use B12 for the 3-ppl column
- New "Fits 12M?" column, regenerated picks for unfunded / funded scenarios
- details.md: funding model and funded-vs-unfunded table

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ICPC_Single_Contest_Plans.xlsx
+++ b/ICPC_Single_Contest_Plans.xlsx
@@ -275,7 +275,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="123">
+  <cellXfs count="124">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -637,6 +637,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -890,11 +893,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="55" min="1" max="1"/>
     <col width="17" customWidth="1" style="55" min="2" max="11"/>
+    <col width="22" customWidth="1" style="56" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.35" customHeight="1" s="56">
@@ -907,7 +911,7 @@
     <row r="2" ht="42" customHeight="1" s="56">
       <c r="A2" s="58" t="inlineStr">
         <is>
-          <t>Each trip planned as if it is the only contest attended. Two to three variants per contest, costed for 3 people (contestants, 1 room) and 4 people (3 contestants + coach). University pays flights, trains, hotels, meals &amp; local transport; contest fees and 'Other' are personal. Prices checked 30 Sep 2026; flights re-priced on Trip.com 30 Sep – 1 Oct 2026; trains (Ctrip) and hotels (Trip.com) re-checked 1 Oct; official train fares and sale times from 12306 on 3 Oct; 10 Oct: Shanghai and Nanchang added, trains re-checked on 12306 / ChinaTicketOnline, flights and hotels on Trip.com (built-in browser) and SlickTrip. Blue = inputs; yellow = key assumptions; green = links.</t>
+          <t>Each trip planned as if it is the only contest attended. Two to three variants per contest. Two scenarios: the UNFUNDED regional (3 contestants pay everything) and the FUNDED regional (₮12M from the university, coach travels: 4 people). University funding covers flights, trains, hotels, meals &amp; local transport; contest fees and 'Other' are personal. Prices: Trip.com / 12306 / ChinaTicketOnline / SlickTrip / Booking.com checked 30 Sep – 10 Oct 2026. Blue = inputs; yellow = key assumptions; green = links.</t>
         </is>
       </c>
     </row>
@@ -921,22 +925,22 @@
     <row r="5" ht="15" customHeight="1" s="56">
       <c r="A5" s="60" t="inlineStr">
         <is>
-          <t>University funding per regional (MNT)</t>
+          <t>University funding – funded regional (MNT)</t>
         </is>
       </c>
       <c r="B5" s="61" t="n">
-        <v>15000000</v>
+        <v>12000000</v>
       </c>
       <c r="C5" s="62" t="inlineStr">
         <is>
-          <t>Team: ₮15M for each regional; two separate trips with home in between</t>
+          <t>One regional is funded with ₮12M and the coach travels (4 people: 3 contestants + coach); used in every "4 ppl" column</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="56">
       <c r="A6" s="60" t="inlineStr">
         <is>
-          <t>Travelers – small team</t>
+          <t>Travelers – unfunded regional</t>
         </is>
       </c>
       <c r="B6" s="63" t="n">
@@ -944,14 +948,14 @@
       </c>
       <c r="C6" s="62" t="inlineStr">
         <is>
-          <t>3 contestants, one room</t>
+          <t>3 contestants, one room, everyone pays</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="56">
       <c r="A7" s="60" t="inlineStr">
         <is>
-          <t>Travelers – with coach</t>
+          <t>Travelers – funded regional (with coach)</t>
         </is>
       </c>
       <c r="B7" s="63" t="n">
@@ -959,7 +963,7 @@
       </c>
       <c r="C7" s="62" t="inlineStr">
         <is>
-          <t>3 contestants + coach, two rooms</t>
+          <t>3 contestants + coach, two rooms (or one family room for 4)</t>
         </is>
       </c>
     </row>
@@ -1023,10 +1027,25 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="60" t="inlineStr">
+        <is>
+          <t>University funding – unfunded regional (MNT)</t>
+        </is>
+      </c>
+      <c r="B12" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="62" t="inlineStr">
+        <is>
+          <t>The other regional is unfunded: the 3 contestants pay everything themselves; used in every "3 ppl" column</t>
+        </is>
+      </c>
+    </row>
     <row r="13" ht="15" customHeight="1" s="56">
       <c r="A13" s="59" t="inlineStr">
         <is>
-          <t>Side-by-side (all figures incl. 10% contingency on the university part)</t>
+          <t>Side-by-side (all figures incl. 10% contingency on the travel + stay part). 3 ppl = the UNFUNDED regional, 4 ppl = the FUNDED regional (₮12M, coach travels)</t>
         </is>
       </c>
     </row>
@@ -1038,32 +1057,32 @@
       </c>
       <c r="B14" s="66" t="inlineStr">
         <is>
-          <t>Univ.-paid total – 3 ppl</t>
+          <t>Travel + stay total – 3 ppl (unfunded: paid by the contestants)</t>
         </is>
       </c>
       <c r="C14" s="66" t="inlineStr">
         <is>
-          <t>Funding left – 3 ppl</t>
+          <t>Funding left – 3 ppl (funding ₮0)</t>
         </is>
       </c>
       <c r="D14" s="66" t="inlineStr">
         <is>
-          <t>Out-of-pocket per person – 3 ppl</t>
+          <t>Cost per person – 3 ppl (everything incl. fee)</t>
         </is>
       </c>
       <c r="E14" s="66" t="inlineStr">
         <is>
-          <t>Univ.-paid total – 4 ppl</t>
+          <t>Travel + stay total – 4 ppl (funded)</t>
         </is>
       </c>
       <c r="F14" s="66" t="inlineStr">
         <is>
-          <t>Funding left – 4 ppl</t>
+          <t>Left of the ₮12M – 4 ppl (negative = over)</t>
         </is>
       </c>
       <c r="G14" s="66" t="inlineStr">
         <is>
-          <t>Out-of-pocket per person – 4 ppl</t>
+          <t>Out-of-pocket per person – 4 ppl (fee, UB taxi, insurance, eSIM)</t>
         </is>
       </c>
       <c r="H14" s="66" t="inlineStr">
@@ -1084,6 +1103,11 @@
       <c r="K14" s="66" t="inlineStr">
         <is>
           <t>Door-to-door</t>
+        </is>
+      </c>
+      <c r="L14" s="66" t="inlineStr">
+        <is>
+          <t>Fits ₮12M with the coach?</t>
         </is>
       </c>
     </row>
@@ -1133,6 +1157,10 @@
         <f>'Shenyang – Budget'!D69</f>
         <v/>
       </c>
+      <c r="L15" s="123">
+        <f>IF(F15&gt;=0,"yes","over by "&amp;TEXT(-F15,"#,##0")&amp;" ₮")</f>
+        <v/>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="56">
       <c r="A16" s="67" t="inlineStr">
@@ -1180,6 +1208,10 @@
         <f>'Shenyang – Comfort'!D68</f>
         <v/>
       </c>
+      <c r="L16" s="123">
+        <f>IF(F16&gt;=0,"yes","over by "&amp;TEXT(-F16,"#,##0")&amp;" ₮")</f>
+        <v/>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="56">
       <c r="A17" s="67" t="inlineStr">
@@ -1227,6 +1259,10 @@
         <f>'Shenyang – Budget (G-train)'!D70</f>
         <v/>
       </c>
+      <c r="L17" s="123">
+        <f>IF(F17&gt;=0,"yes","over by "&amp;TEXT(-F17,"#,##0")&amp;" ₮")</f>
+        <v/>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="56">
       <c r="A18" s="67" t="inlineStr">
@@ -1274,6 +1310,10 @@
         <f>'Shenyang – Comfort (G-train)'!D71</f>
         <v/>
       </c>
+      <c r="L18" s="123">
+        <f>IF(F18&gt;=0,"yes","over by "&amp;TEXT(-F18,"#,##0")&amp;" ₮")</f>
+        <v/>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="56">
       <c r="A19" s="67" t="inlineStr">
@@ -1321,6 +1361,10 @@
         <f>'Shanghai – Sleeper'!D71</f>
         <v/>
       </c>
+      <c r="L19" s="123">
+        <f>IF(F19&gt;=0,"yes","over by "&amp;TEXT(-F19,"#,##0")&amp;" ₮")</f>
+        <v/>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="56">
       <c r="A20" s="67" t="inlineStr">
@@ -1368,6 +1412,10 @@
         <f>'Shanghai – Spring nonstop'!D65</f>
         <v/>
       </c>
+      <c r="L20" s="123">
+        <f>IF(F20&gt;=0,"yes","over by "&amp;TEXT(-F20,"#,##0")&amp;" ₮")</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="67" t="inlineStr">
@@ -1415,6 +1463,10 @@
         <f>'Shanghai – Train (no sleeper)'!D74</f>
         <v/>
       </c>
+      <c r="L21" s="123">
+        <f>IF(F21&gt;=0,"yes","over by "&amp;TEXT(-F21,"#,##0")&amp;" ₮")</f>
+        <v/>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="56">
       <c r="A22" s="67" t="inlineStr">
@@ -1462,6 +1514,10 @@
         <f>'Nanchang – Sleeper'!D70</f>
         <v/>
       </c>
+      <c r="L22" s="123">
+        <f>IF(F22&gt;=0,"yes","over by "&amp;TEXT(-F22,"#,##0")&amp;" ₮")</f>
+        <v/>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1" s="56">
       <c r="A23" s="67" t="inlineStr">
@@ -1509,6 +1565,10 @@
         <f>'Nanchang – Comfort'!D72</f>
         <v/>
       </c>
+      <c r="L23" s="123">
+        <f>IF(F23&gt;=0,"yes","over by "&amp;TEXT(-F23,"#,##0")&amp;" ₮")</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1" s="56">
       <c r="A24" s="67" t="inlineStr">
@@ -1556,6 +1616,10 @@
         <f>'Nanchang – Fly in (Air China)'!D68</f>
         <v/>
       </c>
+      <c r="L24" s="123">
+        <f>IF(F24&gt;=0,"yes","over by "&amp;TEXT(-F24,"#,##0")&amp;" ₮")</f>
+        <v/>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1" s="56">
       <c r="A25" s="67" t="inlineStr">
@@ -1603,6 +1667,10 @@
         <f>'Hong Kong – Budget'!D60</f>
         <v/>
       </c>
+      <c r="L25" s="123">
+        <f>IF(F25&gt;=0,"yes","over by "&amp;TEXT(-F25,"#,##0")&amp;" ₮")</f>
+        <v/>
+      </c>
     </row>
     <row r="26" s="56">
       <c r="A26" s="67" t="inlineStr">
@@ -1650,6 +1718,10 @@
         <f>'Hong Kong – Comfort'!D60</f>
         <v/>
       </c>
+      <c r="L26" s="123">
+        <f>IF(F26&gt;=0,"yes","over by "&amp;TEXT(-F26,"#,##0")&amp;" ₮")</f>
+        <v/>
+      </c>
     </row>
     <row r="27" ht="30" customHeight="1" s="56">
       <c r="A27" s="67" t="inlineStr">
@@ -1697,6 +1769,10 @@
         <f>'Hong Kong – Value'!D60</f>
         <v/>
       </c>
+      <c r="L27" s="123">
+        <f>IF(F27&gt;=0,"yes","over by "&amp;TEXT(-F27,"#,##0")&amp;" ₮")</f>
+        <v/>
+      </c>
     </row>
     <row r="28" s="56">
       <c r="A28" s="67" t="inlineStr">
@@ -1744,6 +1820,10 @@
         <f>'Hong Kong – Sleep first'!D60</f>
         <v/>
       </c>
+      <c r="L28" s="123">
+        <f>IF(F28&gt;=0,"yes","over by "&amp;TEXT(-F28,"#,##0")&amp;" ₮")</f>
+        <v/>
+      </c>
     </row>
     <row r="29" ht="30" customHeight="1" s="56">
       <c r="A29" s="67" t="inlineStr">
@@ -1791,6 +1871,10 @@
         <f>'EC Final Hangzhou – Train'!D70</f>
         <v/>
       </c>
+      <c r="L29" s="123">
+        <f>IF(F29&gt;=0,"yes","over by "&amp;TEXT(-F29,"#,##0")&amp;" ₮")</f>
+        <v/>
+      </c>
     </row>
     <row r="30" ht="30" customHeight="1" s="56">
       <c r="A30" s="67" t="inlineStr">
@@ -1836,6 +1920,10 @@
       </c>
       <c r="K30" s="71">
         <f>'EC Final Hangzhou – Fly'!D70</f>
+        <v/>
+      </c>
+      <c r="L30" s="123">
+        <f>IF(F30&gt;=0,"yes","over by "&amp;TEXT(-F30,"#,##0")&amp;" ₮")</f>
         <v/>
       </c>
     </row>
@@ -1853,88 +1941,88 @@
     <row r="33" ht="62" customHeight="1" s="56">
       <c r="A33" s="73" t="inlineStr">
         <is>
-          <t>Regional – Shenyang (14–15 Nov)</t>
+          <t>Unfunded regional (3 ppl pay)</t>
         </is>
       </c>
       <c r="B33" s="74" t="inlineStr">
         <is>
-          <t>Shenyang – Comfort: rest day, RiCH family room 1.3 km from NEU, hard sleeper home after the contest: ~₮6.2M (3 ppl) / ~₮8.0M (with coach). Shenyang – Budget (soft sleeper before day 1, hard after): ~₮5.2M (3 ppl) / ~₮7.0M (with coach). No sleepers at all: G-train Comfort ₮6.7M / ₮8.8M, G-train Budget ₮6.0M / ₮8.3M. Fly home on Air China 12:55 ($171).</t>
+          <t>Cheapest sleep-safe plans per person incl. fee, taxi, insurance, eSIM and 10% contingency: Shenyang – Budget ₮2.14M per person (soft sleeper before day 1); Shenyang – Comfort ₮2.46M per person; Nanchang – Sleeper ₮2.50M per person; Shanghai – Sleeper ₮2.89M per person; Hong Kong – Budget ₮3.43M per person; EC Final – Train ₮3.14M per person. Shenyang and Nanchang are the cheap ones to pay yourselves.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="62" customHeight="1" s="56">
       <c r="A34" s="73" t="inlineStr">
         <is>
-          <t>Regional – Shanghai (5–6 Dec)</t>
+          <t>Funded regional (₮12M, coach)</t>
         </is>
       </c>
       <c r="B34" s="74" t="inlineStr">
         <is>
-          <t>Shanghai – Sleeper: MIAT $151 + G17 out on 3 Dec, Jenny's Apartment 3 nights (1 km), D8 overnight seat back, Air China 12:55 $172 on 7 Dec: ~₮7.5M (3 ppl) / ~₮9.8M (with coach). Spring nonstop (Tue 1 → Tue 8 Dec, 7 nights): ~₮8.2M (3 ppl) / ~₮10.7M (with coach); day train home with a Beijing night ~₮8.1M (3 ppl) / ~₮10.8M (with coach). A Mongolian team needs a wildcard: email shu_icpc@163.com now.</t>
+          <t>Fits ₮12M: Shenyang – Comfort ₮8.04M (fits, ₮3.96M left); Shanghai – Sleeper ₮9.83M (fits, ₮2.17M left); Nanchang – Sleeper ₮8.19M (fits, ₮3.81M left); EC Final – Train ₮11.12M (fits, ₮0.88M left). Hong Kong – Budget ₮12.12M (over by ₮0.12M) only works without the 10% contingency (subtotal ~₮11.0M); Hong Kong Value / Comfort / Sleep first and EC Final – Fly do not fit. Use the funded trip for the dearest contest you must attend (Shanghai, Hong Kong, EC Final) and pay the cheap one yourselves.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="47" customHeight="1" s="56">
       <c r="A35" s="73" t="inlineStr">
         <is>
+          <t>Regional – Shenyang (14–15 Nov)</t>
+        </is>
+      </c>
+      <c r="B35" s="74" t="inlineStr">
+        <is>
+          <t>Comfort: rest day, RiCH family room 1.3 km from NEU, hard sleeper home after the contest. No sleepers at all: G-train Comfort ₮6.72M / ₮8.84M, G-train Budget ₮6.05M / ₮8.27M (3 / 4 ppl). Fly home on Air China 12:55 ($171).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="47" customHeight="1" s="56">
+      <c r="A36" s="73" t="inlineStr">
+        <is>
+          <t>Regional – Shanghai (5–6 Dec)</t>
+        </is>
+      </c>
+      <c r="B36" s="74" t="inlineStr">
+        <is>
+          <t>Sleeper: MIAT $151 + G17 out on 3 Dec, Jenny's Apartment 3 nights (1 km), D8 overnight seat back, Air China 12:55 $172 on 7 Dec. Spring nonstop (Tue 1 → Tue 8 Dec, 7 nights) ₮8.21M / ₮10.73M; day train home with a Beijing night ₮8.11M / ₮10.78M. Wildcard: email shu_icpc@163.com now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="47" customHeight="1" s="56">
+      <c r="A37" s="73" t="inlineStr">
+        <is>
           <t>Regional – Nanchang (19–20 Dec)</t>
         </is>
       </c>
-      <c r="B35" s="74" t="inlineStr">
-        <is>
-          <t>Nanchang – Sleeper: Air China $157 + Z111 hard sleeper (arrive 11:52 on 18 Dec), Orange Hotel 2 nights, D136 seat back, Air China 12:55 $172: ~₮6.3M (3 ppl) / ~₮8.2M (with coach). Comfort (daytime G-train, 3 hotel nights) ₮8.0M / ₮10.3M; Fly in (Air China through ticket $356) ₮8.4M / ₮11.0M.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="62" customHeight="1" s="56">
-      <c r="A36" s="73" t="inlineStr">
+      <c r="B37" s="74" t="inlineStr">
+        <is>
+          <t>Sleeper: Air China $157 + Z111 hard sleeper (arrive 11:52 on 18 Dec), Orange Hotel 2 nights, D136 seat back, Air China 12:55 $172. Comfort (daytime G-train, 3 hotel nights) ₮7.96M / ₮10.32M; Fly in (Air China through ticket $356) ₮8.41M / ₮10.95M.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="47" customHeight="1" s="56">
+      <c r="A38" s="73" t="inlineStr">
         <is>
           <t>Regional – Hong Kong (9–10 Jan)</t>
         </is>
       </c>
-      <c r="B36" s="74" t="inlineStr">
-        <is>
-          <t>Hong Kong – Sleep first (recommended for sleep): MIAT nonstop ($586 return on Trip.com, low against the usual $708–900), two rooms in iclub AMTD Sheung Wan 2 MTR stops from HKU: ~₮11.6M (3 ppl) / ~₮14.5M (with coach). Budget (Chungking Mansion guesthouse) ₮9.1M / ₮12.1M; Value (Kusa Inn 9.6) ₮9.1M / ₮12.4M; Comfort ₮9.6M / ₮13.2M. No route or date is cheaper: Beijing, Hohhot, Shenzhen and Seoul combinations all cost more (checked 10 Oct).</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="62" customHeight="1" s="56">
-      <c r="A37" s="73" t="inlineStr">
+      <c r="B38" s="74" t="inlineStr">
+        <is>
+          <t>MIAT nonstop ($586 return on Trip.com, low against the usual $708–900) is the cheapest way in. Budget guesthouse ₮9.08M / ₮12.12M; Value (Kusa Inn 9.6) ₮9.08M / ₮12.38M; Sleep first (2 rooms near HKU) ₮11.63M / ₮14.45M. No route or date is cheaper (checked 10 Oct).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="47" customHeight="1" s="56">
+      <c r="A39" s="73" t="inlineStr">
         <is>
           <t>EC Final (only if qualified)</t>
         </is>
       </c>
-      <c r="B37" s="74" t="inlineStr">
-        <is>
-          <t>Train is cheapest (~₮8.2M / ~₮11.1M with coach): MIAT to Beijing, D17 overnight sleeper Beijing 19:10 → Hangzhou 09:15 (¥491, saves the 25 Jan hotel night), Air China through ticket Hangzhou → UB home on 29 Jan. Fly is ~₮11.0M / ~₮14.8M with the coach (just inside ₮15M): Aero Mongolia UB → Hohhot 06:30 + Xiamen Airlines → Hangzhou 13:40 (¥2,752, separate tickets), Air China through ticket home. Buy D17 on 12306 at 10:00 on 11 Jan, the day sales open.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="30" customHeight="1" s="56"/>
-    <row r="39" ht="32" customHeight="1" s="56">
-      <c r="A39" s="75" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
       <c r="B39" s="74" t="inlineStr">
         <is>
-          <t>Dates are provisional (ICPC Beijing HQ summary, 5 Aug 2026). Hong Kong host (HKU) and EC Final venue (HZNU Cangqian) are from secondary sources; Shanghai (Shanghai University Baoshan) follows the 2025 invitation and Nanchang (Jiangxi Normal University Yaohu campus) the 2019 handbook – confirm each invitation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="18" customHeight="1" s="56">
-      <c r="A40" s="75" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B40" s="74" t="inlineStr">
-        <is>
-          <t>EC Final is qualification-only: plan it only once the team has earned a slot at a regional.</t>
-        </is>
-      </c>
-    </row>
+          <t>Train: MIAT to Beijing, D17 overnight sleeper Beijing 19:10 → Hangzhou 09:15 (¥491), Air China through ticket Hangzhou → UB on 29 Jan: ₮11.12M (fits, ₮0.88M left) for 4 ppl, ₮3.14M per person for 3. Fly (Aero Mongolia + Xiamen via Hohhot) is ₮14.82M (over by ₮2.82M) – does not fit ₮12M. Buy D17 on 12306 at 10:00 on 11 Jan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1" s="56"/>
     <row r="41" ht="32" customHeight="1" s="56">
       <c r="A41" s="75" t="inlineStr">
         <is>
@@ -1943,11 +2031,11 @@
       </c>
       <c r="B41" s="74" t="inlineStr">
         <is>
-          <t>4-person plans use whatever split is cheapest on Trip.com/Booking.com: one family room for 4 (Shenyang RiCH, Nanchang Orange Hotel), or two rooms. Taxi costs assume one car; with luggage 4 people may need an XL car.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="47" customHeight="1" s="56">
+          <t>Dates are provisional (ICPC Beijing HQ summary, 5 Aug 2026). Hong Kong host (HKU) and EC Final venue (HZNU Cangqian) are from secondary sources; Shanghai (Shanghai University Baoshan) follows the 2025 invitation and Nanchang (Jiangxi Normal University Yaohu campus) the 2019 handbook – confirm each invitation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1" s="56">
       <c r="A42" s="75" t="inlineStr">
         <is>
           <t>Note</t>
@@ -1955,7 +2043,7 @@
       </c>
       <c r="B42" s="74" t="inlineStr">
         <is>
-          <t>Sleep rule (see the 'Sleep check' sheet): the two nights before each contest day are in a quiet bed near the venue; sleepers, early flights and red-eyes are only used before day 1 (soft sleeper) or after the contest (anything goes). Sleeper trains replace hotel nights in the Shenyang, Shanghai (D8 seat), Nanchang (Z111 / D136 seat) and EC Final (D17) plans; the 'G-train' / 'no sleeper' variants cost more per trip. Chinese train tickets go on sale 14 days ahead – dates are in the '12306 &amp; ChinaTicketOnline' and '10 Oct' sheets of the fares workbook.</t>
+          <t>EC Final is qualification-only: plan it only once the team has earned a slot at a regional.</t>
         </is>
       </c>
     </row>
@@ -1967,18 +2055,69 @@
       </c>
       <c r="B43" s="74" t="inlineStr">
         <is>
+          <t>4-person plans use whatever split is cheapest on Trip.com/Booking.com: one family room for 4 (Shenyang RiCH, Nanchang Orange Hotel), or two rooms. Taxi costs assume one car; with luggage 4 people may need an XL car.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="47" customHeight="1" s="56">
+      <c r="A44" s="75" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B44" s="74" t="inlineStr">
+        <is>
+          <t>Sleep rule (see the 'Sleep check' sheet): the two nights before each contest day are in a quiet bed near the venue; sleepers, early flights and red-eyes are only used before day 1 (soft sleeper) or after the contest (anything goes). Sleeper trains replace hotel nights in the Shenyang, Shanghai (D8 seat), Nanchang (Z111 / D136 seat) and EC Final (D17) plans; the 'G-train' / 'no sleeper' variants cost more per trip. Chinese train tickets go on sale 14 days ahead – dates are in the '12306 &amp; ChinaTicketOnline' and '10 Oct' sheets of the fares workbook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="32" customHeight="1" s="56">
+      <c r="A45" s="75" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B45" s="74" t="inlineStr">
+        <is>
           <t>Sources (10 Oct): Trip.com (flights and hotels, built-in browser), 12306 (official train fares), ChinaTicketOnline (timetable and sale-date check; 30–70% dearer than 12306, not used for booking), SlickTrip (MIAT / Spring fares; Air China is unpriced there).</t>
         </is>
       </c>
     </row>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="72"/>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="13">
+    <mergeCell ref="B45:K45"/>
     <mergeCell ref="B41:K41"/>
-    <mergeCell ref="B40:K40"/>
     <mergeCell ref="B35:K35"/>
+    <mergeCell ref="B44:K44"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B43:K43"/>
     <mergeCell ref="B39:K39"/>
+    <mergeCell ref="B38:K38"/>
     <mergeCell ref="B34:K34"/>
     <mergeCell ref="B33:K33"/>
     <mergeCell ref="B42:K42"/>
@@ -2027,6 +2166,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -2049,6 +2189,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -2900,16 +3041,17 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31" ht="15" customHeight="1" s="56">
       <c r="G31" s="60" t="n"/>
       <c r="H31" s="96" t="inlineStr">
         <is>
-          <t>3 people</t>
+          <t>3 people – UNFUNDED</t>
         </is>
       </c>
       <c r="K31" s="96" t="inlineStr">
         <is>
-          <t>4 people</t>
+          <t>4 people – FUNDED ₮12M</t>
         </is>
       </c>
     </row>
@@ -2965,7 +3107,7 @@
         </is>
       </c>
       <c r="H35" s="101">
-        <f>Compare!$B$5-H34</f>
+        <f>Compare!$B$12-H34</f>
         <v/>
       </c>
       <c r="K35" s="101">
@@ -3033,6 +3175,7 @@
         <v/>
       </c>
     </row>
+    <row r="40"/>
     <row r="41" ht="15" customHeight="1" s="56">
       <c r="A41" s="72" t="inlineStr">
         <is>
@@ -3088,6 +3231,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47" ht="15" customHeight="1" s="56">
       <c r="A47" s="72" t="inlineStr">
         <is>
@@ -3197,6 +3341,7 @@
         </is>
       </c>
     </row>
+    <row r="54"/>
     <row r="55" ht="15" customHeight="1" s="56">
       <c r="A55" s="72" t="inlineStr">
         <is>
@@ -3601,6 +3746,7 @@
       <c r="K68" s="107" t="n"/>
       <c r="L68" s="107" t="n"/>
     </row>
+    <row r="69"/>
     <row r="70" ht="15" customHeight="1" s="56">
       <c r="C70" s="59" t="inlineStr">
         <is>
@@ -3676,6 +3822,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -3698,6 +3845,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -4639,16 +4787,17 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
     <row r="33" ht="15" customHeight="1" s="56">
       <c r="G33" s="60" t="n"/>
       <c r="H33" s="96" t="inlineStr">
         <is>
-          <t>3 people</t>
+          <t>3 people – UNFUNDED</t>
         </is>
       </c>
       <c r="K33" s="96" t="inlineStr">
         <is>
-          <t>4 people</t>
+          <t>4 people – FUNDED ₮12M</t>
         </is>
       </c>
     </row>
@@ -4704,7 +4853,7 @@
         </is>
       </c>
       <c r="H37" s="101">
-        <f>Compare!$B$5-H36</f>
+        <f>Compare!$B$12-H36</f>
         <v/>
       </c>
       <c r="K37" s="101">
@@ -4772,6 +4921,7 @@
         <v/>
       </c>
     </row>
+    <row r="42"/>
     <row r="43" ht="15" customHeight="1" s="56">
       <c r="A43" s="72" t="inlineStr">
         <is>
@@ -4827,6 +4977,7 @@
         </is>
       </c>
     </row>
+    <row r="48"/>
     <row r="49" ht="15" customHeight="1" s="56">
       <c r="A49" s="72" t="inlineStr">
         <is>
@@ -4936,6 +5087,7 @@
         </is>
       </c>
     </row>
+    <row r="56"/>
     <row r="57" ht="15" customHeight="1" s="56">
       <c r="A57" s="72" t="inlineStr">
         <is>
@@ -5340,6 +5492,7 @@
       <c r="K70" s="107" t="n"/>
       <c r="L70" s="107" t="n"/>
     </row>
+    <row r="71"/>
     <row r="72" ht="15" customHeight="1" s="56">
       <c r="C72" s="59" t="inlineStr">
         <is>
@@ -5415,6 +5568,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -5437,6 +5591,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -6284,16 +6439,17 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31" ht="15" customHeight="1" s="56">
       <c r="G31" s="60" t="n"/>
       <c r="H31" s="96" t="inlineStr">
         <is>
-          <t>3 people</t>
+          <t>3 people – UNFUNDED</t>
         </is>
       </c>
       <c r="K31" s="96" t="inlineStr">
         <is>
-          <t>4 people</t>
+          <t>4 people – FUNDED ₮12M</t>
         </is>
       </c>
     </row>
@@ -6349,7 +6505,7 @@
         </is>
       </c>
       <c r="H35" s="101">
-        <f>Compare!$B$5-H34</f>
+        <f>Compare!$B$12-H34</f>
         <v/>
       </c>
       <c r="K35" s="101">
@@ -6417,6 +6573,7 @@
         <v/>
       </c>
     </row>
+    <row r="40"/>
     <row r="41" ht="15" customHeight="1" s="56">
       <c r="A41" s="72" t="inlineStr">
         <is>
@@ -6472,6 +6629,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47" ht="15" customHeight="1" s="56">
       <c r="A47" s="72" t="inlineStr">
         <is>
@@ -6581,6 +6739,7 @@
         </is>
       </c>
     </row>
+    <row r="54"/>
     <row r="55" ht="15" customHeight="1" s="56">
       <c r="A55" s="72" t="inlineStr">
         <is>
@@ -6929,6 +7088,7 @@
       <c r="K66" s="107" t="n"/>
       <c r="L66" s="107" t="n"/>
     </row>
+    <row r="67"/>
     <row r="68" ht="15" customHeight="1" s="56">
       <c r="C68" s="59" t="inlineStr">
         <is>
@@ -7002,6 +7162,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -7024,6 +7185,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -7716,16 +7878,17 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27" ht="15" customHeight="1" s="56">
       <c r="G27" s="60" t="n"/>
       <c r="H27" s="96" t="inlineStr">
         <is>
-          <t>3 people</t>
+          <t>3 people – UNFUNDED</t>
         </is>
       </c>
       <c r="K27" s="96" t="inlineStr">
         <is>
-          <t>4 people</t>
+          <t>4 people – FUNDED ₮12M</t>
         </is>
       </c>
     </row>
@@ -7781,7 +7944,7 @@
         </is>
       </c>
       <c r="H31" s="101">
-        <f>Compare!$B$5-H30</f>
+        <f>Compare!$B$12-H30</f>
         <v/>
       </c>
       <c r="K31" s="101">
@@ -7849,6 +8012,7 @@
         <v/>
       </c>
     </row>
+    <row r="36"/>
     <row r="37" ht="15" customHeight="1" s="56">
       <c r="A37" s="72" t="inlineStr">
         <is>
@@ -7904,6 +8068,7 @@
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43" ht="15" customHeight="1" s="56">
       <c r="A43" s="72" t="inlineStr">
         <is>
@@ -7996,6 +8161,7 @@
         </is>
       </c>
     </row>
+    <row r="49"/>
     <row r="50" ht="15" customHeight="1" s="56">
       <c r="A50" s="72" t="inlineStr">
         <is>
@@ -8298,19 +8464,19 @@
     <mergeCell ref="E58:L58"/>
     <mergeCell ref="C45:L45"/>
     <mergeCell ref="B38:L38"/>
-    <mergeCell ref="E53:L53"/>
     <mergeCell ref="E59:L59"/>
     <mergeCell ref="E51:L51"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="E54:L54"/>
+    <mergeCell ref="C44:L44"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
+    <mergeCell ref="E53:L53"/>
+    <mergeCell ref="B41:L41"/>
     <mergeCell ref="B40:L40"/>
-    <mergeCell ref="B41:L41"/>
-    <mergeCell ref="C44:L44"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -8354,6 +8520,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -8376,6 +8543,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -9068,16 +9236,17 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27" ht="15" customHeight="1" s="56">
       <c r="G27" s="60" t="n"/>
       <c r="H27" s="96" t="inlineStr">
         <is>
-          <t>3 people</t>
+          <t>3 people – UNFUNDED</t>
         </is>
       </c>
       <c r="K27" s="96" t="inlineStr">
         <is>
-          <t>4 people</t>
+          <t>4 people – FUNDED ₮12M</t>
         </is>
       </c>
     </row>
@@ -9133,7 +9302,7 @@
         </is>
       </c>
       <c r="H31" s="101">
-        <f>Compare!$B$5-H30</f>
+        <f>Compare!$B$12-H30</f>
         <v/>
       </c>
       <c r="K31" s="101">
@@ -9201,6 +9370,7 @@
         <v/>
       </c>
     </row>
+    <row r="36"/>
     <row r="37" ht="15" customHeight="1" s="56">
       <c r="A37" s="72" t="inlineStr">
         <is>
@@ -9256,6 +9426,7 @@
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43" ht="15" customHeight="1" s="56">
       <c r="A43" s="72" t="inlineStr">
         <is>
@@ -9348,6 +9519,7 @@
         </is>
       </c>
     </row>
+    <row r="49"/>
     <row r="50" ht="15" customHeight="1" s="56">
       <c r="A50" s="72" t="inlineStr">
         <is>
@@ -9650,19 +9822,19 @@
     <mergeCell ref="E58:L58"/>
     <mergeCell ref="C45:L45"/>
     <mergeCell ref="B38:L38"/>
-    <mergeCell ref="E53:L53"/>
     <mergeCell ref="E59:L59"/>
     <mergeCell ref="E51:L51"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="E54:L54"/>
+    <mergeCell ref="C44:L44"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
+    <mergeCell ref="E53:L53"/>
+    <mergeCell ref="B41:L41"/>
     <mergeCell ref="B40:L40"/>
-    <mergeCell ref="B41:L41"/>
-    <mergeCell ref="C44:L44"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -9706,6 +9878,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -9728,6 +9901,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -10420,16 +10594,17 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27" ht="15" customHeight="1" s="56">
       <c r="G27" s="60" t="n"/>
       <c r="H27" s="96" t="inlineStr">
         <is>
-          <t>3 people</t>
+          <t>3 people – UNFUNDED</t>
         </is>
       </c>
       <c r="K27" s="96" t="inlineStr">
         <is>
-          <t>4 people</t>
+          <t>4 people – FUNDED ₮12M</t>
         </is>
       </c>
     </row>
@@ -10485,7 +10660,7 @@
         </is>
       </c>
       <c r="H31" s="101">
-        <f>Compare!$B$5-H30</f>
+        <f>Compare!$B$12-H30</f>
         <v/>
       </c>
       <c r="K31" s="101">
@@ -10553,6 +10728,7 @@
         <v/>
       </c>
     </row>
+    <row r="36"/>
     <row r="37" ht="15" customHeight="1" s="56">
       <c r="A37" s="72" t="inlineStr">
         <is>
@@ -10608,6 +10784,7 @@
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43" ht="15" customHeight="1" s="56">
       <c r="A43" s="72" t="inlineStr">
         <is>
@@ -10700,6 +10877,7 @@
         </is>
       </c>
     </row>
+    <row r="49"/>
     <row r="50" ht="15" customHeight="1" s="56">
       <c r="A50" s="72" t="inlineStr">
         <is>
@@ -11002,17 +11180,17 @@
     <mergeCell ref="E58:L58"/>
     <mergeCell ref="C45:L45"/>
     <mergeCell ref="B38:L38"/>
+    <mergeCell ref="E53:L53"/>
     <mergeCell ref="E59:L59"/>
     <mergeCell ref="E51:L51"/>
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="E54:L54"/>
-    <mergeCell ref="B40:L40"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
-    <mergeCell ref="E53:L53"/>
+    <mergeCell ref="B40:L40"/>
     <mergeCell ref="B41:L41"/>
     <mergeCell ref="C44:L44"/>
   </mergeCells>
@@ -11058,6 +11236,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -11080,6 +11259,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -11772,16 +11952,17 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27" ht="15" customHeight="1" s="56">
       <c r="G27" s="60" t="n"/>
       <c r="H27" s="96" t="inlineStr">
         <is>
-          <t>3 people</t>
+          <t>3 people – UNFUNDED</t>
         </is>
       </c>
       <c r="K27" s="96" t="inlineStr">
         <is>
-          <t>4 people</t>
+          <t>4 people – FUNDED ₮12M</t>
         </is>
       </c>
     </row>
@@ -11837,7 +12018,7 @@
         </is>
       </c>
       <c r="H31" s="101">
-        <f>Compare!$B$5-H30</f>
+        <f>Compare!$B$12-H30</f>
         <v/>
       </c>
       <c r="K31" s="101">
@@ -11905,6 +12086,7 @@
         <v/>
       </c>
     </row>
+    <row r="36"/>
     <row r="37" ht="15" customHeight="1" s="56">
       <c r="A37" s="72" t="inlineStr">
         <is>
@@ -11956,10 +12138,11 @@
       </c>
       <c r="B41" s="74" t="inlineStr">
         <is>
-          <t>About ₮2.6M dearer than the guesthouse plan for 3 people (HK$6,206 vs HK$1,177 for the rooms); still below the ₮15M funding even with the coach.</t>
-        </is>
-      </c>
-    </row>
+          <t>About ₮2.6M dearer than the guesthouse plan for 3 people (HK$6,206 vs HK$1,177 for the rooms). With the coach it is ₮14.45M, over the ₮12M funding – so use it only for the unfunded trip if the team wants to pay for sleep, or drop to Value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42"/>
     <row r="43" ht="15" customHeight="1" s="56">
       <c r="A43" s="72" t="inlineStr">
         <is>
@@ -12052,6 +12235,7 @@
         </is>
       </c>
     </row>
+    <row r="49"/>
     <row r="50" ht="15" customHeight="1" s="56">
       <c r="A50" s="72" t="inlineStr">
         <is>
@@ -12359,14 +12543,14 @@
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="E54:L54"/>
-    <mergeCell ref="C44:L44"/>
+    <mergeCell ref="B40:L40"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
     <mergeCell ref="E53:L53"/>
     <mergeCell ref="B41:L41"/>
-    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="C44:L44"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -12410,6 +12594,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -12432,6 +12617,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -13248,16 +13434,17 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31" ht="15" customHeight="1" s="56">
       <c r="G31" s="60" t="n"/>
       <c r="H31" s="96" t="inlineStr">
         <is>
-          <t>3 people</t>
+          <t>3 people – UNFUNDED</t>
         </is>
       </c>
       <c r="K31" s="96" t="inlineStr">
         <is>
-          <t>4 people</t>
+          <t>4 people – FUNDED ₮12M</t>
         </is>
       </c>
     </row>
@@ -13313,7 +13500,7 @@
         </is>
       </c>
       <c r="H35" s="101">
-        <f>Compare!$B$5-H34</f>
+        <f>Compare!$B$12-H34</f>
         <v/>
       </c>
       <c r="K35" s="101">
@@ -13381,6 +13568,7 @@
         <v/>
       </c>
     </row>
+    <row r="40"/>
     <row r="41" ht="15" customHeight="1" s="56">
       <c r="A41" s="72" t="inlineStr">
         <is>
@@ -13424,6 +13612,7 @@
         </is>
       </c>
     </row>
+    <row r="45"/>
     <row r="46" ht="15" customHeight="1" s="56">
       <c r="A46" s="72" t="inlineStr">
         <is>
@@ -13538,6 +13727,7 @@
       <c r="B53" s="74" t="n"/>
       <c r="C53" s="74" t="n"/>
     </row>
+    <row r="54"/>
     <row r="55" ht="15" customHeight="1" s="56">
       <c r="A55" s="72" t="inlineStr">
         <is>
@@ -14046,6 +14236,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -14068,6 +14259,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -14835,16 +15027,17 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30" ht="15" customHeight="1" s="56">
       <c r="G30" s="60" t="n"/>
       <c r="H30" s="96" t="inlineStr">
         <is>
-          <t>3 people</t>
+          <t>3 people – UNFUNDED</t>
         </is>
       </c>
       <c r="K30" s="96" t="inlineStr">
         <is>
-          <t>4 people</t>
+          <t>4 people – FUNDED ₮12M</t>
         </is>
       </c>
     </row>
@@ -14900,7 +15093,7 @@
         </is>
       </c>
       <c r="H34" s="101">
-        <f>Compare!$B$5-H33</f>
+        <f>Compare!$B$12-H33</f>
         <v/>
       </c>
       <c r="K34" s="101">
@@ -14968,6 +15161,7 @@
         <v/>
       </c>
     </row>
+    <row r="39"/>
     <row r="40" ht="15" customHeight="1" s="56">
       <c r="A40" s="72" t="inlineStr">
         <is>
@@ -15011,6 +15205,7 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45" ht="15" customHeight="1" s="56">
       <c r="A45" s="72" t="inlineStr">
         <is>
@@ -15125,6 +15320,7 @@
       <c r="B52" s="74" t="n"/>
       <c r="C52" s="74" t="n"/>
     </row>
+    <row r="53"/>
     <row r="54" ht="15" customHeight="1" s="56">
       <c r="A54" s="72" t="inlineStr">
         <is>
@@ -16249,7 +16445,7 @@
       </c>
       <c r="H18" s="116" t="inlineStr">
         <is>
-          <t>Two rooms in an 8.6-rated hotel: +2.6M (3 ppl) / +2.3M (4 ppl) vs Budget (₮11.6M / ₮14.5M total, funding ₮15M).</t>
+          <t>Two rooms in an 8.6-rated hotel: ₮2.55M (3 ppl) / ₮2.33M (4 ppl) vs Budget (₮11.63M / ₮14.45M total). Over the ₮12M with the coach.</t>
         </is>
       </c>
     </row>
@@ -16389,7 +16585,7 @@
     <row r="24" ht="36" customHeight="1" s="56">
       <c r="A24" s="116" t="inlineStr">
         <is>
-          <t>Funding is ₮15M per regional and the recommended plans use ₮6–9M, so there is room for quiet rooms, 2 rooms instead of 1, and an extra rest day before every contest.</t>
+          <t>One regional is funded with ₮12M (coach travels, 4 people); the other is unfunded (3 contestants pay). The funded trip has little headroom (Hong Kong does not fit), and the unfunded trip pays for every hotel night, so protect sleep with timing and location first: arrive a day early only where it is cheap (Shenyang, Nanchang), pick the hotel closest to the venue, and take the cheap-but-bad options only after the contest.</t>
         </is>
       </c>
     </row>
@@ -16462,6 +16658,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -16484,6 +16681,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -17273,16 +17471,17 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31" ht="15" customHeight="1" s="56">
       <c r="G31" s="60" t="n"/>
       <c r="H31" s="96" t="inlineStr">
         <is>
-          <t>3 people</t>
+          <t>3 people – UNFUNDED</t>
         </is>
       </c>
       <c r="K31" s="96" t="inlineStr">
         <is>
-          <t>4 people</t>
+          <t>4 people – FUNDED ₮12M</t>
         </is>
       </c>
     </row>
@@ -17338,7 +17537,7 @@
         </is>
       </c>
       <c r="H35" s="101">
-        <f>Compare!$B$5-H34</f>
+        <f>Compare!$B$12-H34</f>
         <v/>
       </c>
       <c r="K35" s="101">
@@ -17406,6 +17605,7 @@
         <v/>
       </c>
     </row>
+    <row r="40"/>
     <row r="41" ht="15" customHeight="1" s="56">
       <c r="A41" s="72" t="inlineStr">
         <is>
@@ -17449,6 +17649,7 @@
         </is>
       </c>
     </row>
+    <row r="45"/>
     <row r="46" ht="15" customHeight="1" s="56">
       <c r="A46" s="72" t="inlineStr">
         <is>
@@ -17541,6 +17742,7 @@
         </is>
       </c>
     </row>
+    <row r="52"/>
     <row r="53" ht="15" customHeight="1" s="56">
       <c r="A53" s="72" t="inlineStr">
         <is>
@@ -18056,6 +18258,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -18078,6 +18281,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -18853,16 +19057,17 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30" ht="15" customHeight="1" s="56">
       <c r="G30" s="60" t="n"/>
       <c r="H30" s="96" t="inlineStr">
         <is>
-          <t>3 people</t>
+          <t>3 people – UNFUNDED</t>
         </is>
       </c>
       <c r="K30" s="96" t="inlineStr">
         <is>
-          <t>4 people</t>
+          <t>4 people – FUNDED ₮12M</t>
         </is>
       </c>
     </row>
@@ -18918,7 +19123,7 @@
         </is>
       </c>
       <c r="H34" s="101">
-        <f>Compare!$B$5-H33</f>
+        <f>Compare!$B$12-H33</f>
         <v/>
       </c>
       <c r="K34" s="101">
@@ -18986,6 +19191,7 @@
         <v/>
       </c>
     </row>
+    <row r="39"/>
     <row r="40" ht="15" customHeight="1" s="56">
       <c r="A40" s="72" t="inlineStr">
         <is>
@@ -19029,6 +19235,7 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45" ht="15" customHeight="1" s="56">
       <c r="A45" s="72" t="inlineStr">
         <is>
@@ -19138,6 +19345,7 @@
         </is>
       </c>
     </row>
+    <row r="52"/>
     <row r="53" ht="15" customHeight="1" s="56">
       <c r="A53" s="72" t="inlineStr">
         <is>
@@ -20555,12 +20763,12 @@
       <c r="G32" s="60" t="n"/>
       <c r="H32" s="96" t="inlineStr">
         <is>
-          <t>3 people</t>
+          <t>3 people – UNFUNDED</t>
         </is>
       </c>
       <c r="K32" s="96" t="inlineStr">
         <is>
-          <t>4 people</t>
+          <t>4 people – FUNDED ₮12M</t>
         </is>
       </c>
     </row>
@@ -20616,7 +20824,7 @@
         </is>
       </c>
       <c r="H36" s="101">
-        <f>Compare!$B$5-H35</f>
+        <f>Compare!$B$12-H35</f>
         <v/>
       </c>
       <c r="K36" s="101">
@@ -22249,12 +22457,12 @@
       <c r="G32" s="60" t="n"/>
       <c r="H32" s="96" t="inlineStr">
         <is>
-          <t>3 people</t>
+          <t>3 people – UNFUNDED</t>
         </is>
       </c>
       <c r="K32" s="96" t="inlineStr">
         <is>
-          <t>4 people</t>
+          <t>4 people – FUNDED ₮12M</t>
         </is>
       </c>
     </row>
@@ -22310,7 +22518,7 @@
         </is>
       </c>
       <c r="H36" s="101">
-        <f>Compare!$B$5-H35</f>
+        <f>Compare!$B$12-H35</f>
         <v/>
       </c>
       <c r="K36" s="101">
@@ -23037,6 +23245,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -23059,6 +23268,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -23955,16 +24165,17 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32" ht="15" customHeight="1" s="56">
       <c r="G32" s="60" t="n"/>
       <c r="H32" s="96" t="inlineStr">
         <is>
-          <t>3 people</t>
+          <t>3 people – UNFUNDED</t>
         </is>
       </c>
       <c r="K32" s="96" t="inlineStr">
         <is>
-          <t>4 people</t>
+          <t>4 people – FUNDED ₮12M</t>
         </is>
       </c>
     </row>
@@ -24020,7 +24231,7 @@
         </is>
       </c>
       <c r="H36" s="101">
-        <f>Compare!$B$5-H35</f>
+        <f>Compare!$B$12-H35</f>
         <v/>
       </c>
       <c r="K36" s="101">
@@ -24088,6 +24299,7 @@
         <v/>
       </c>
     </row>
+    <row r="41"/>
     <row r="42" ht="15" customHeight="1" s="56">
       <c r="A42" s="72" t="inlineStr">
         <is>
@@ -24143,6 +24355,7 @@
         </is>
       </c>
     </row>
+    <row r="47"/>
     <row r="48" ht="15" customHeight="1" s="56">
       <c r="A48" s="72" t="inlineStr">
         <is>
@@ -24252,6 +24465,7 @@
         </is>
       </c>
     </row>
+    <row r="55"/>
     <row r="56" ht="15" customHeight="1" s="56">
       <c r="A56" s="72" t="inlineStr">
         <is>
@@ -24656,6 +24870,7 @@
       <c r="K69" s="107" t="n"/>
       <c r="L69" s="107" t="n"/>
     </row>
+    <row r="70"/>
     <row r="71" ht="15" customHeight="1" s="56">
       <c r="C71" s="59" t="inlineStr">
         <is>
@@ -24731,6 +24946,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -24753,6 +24969,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -25490,16 +25707,17 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28" ht="15" customHeight="1" s="56">
       <c r="G28" s="60" t="n"/>
       <c r="H28" s="96" t="inlineStr">
         <is>
-          <t>3 people</t>
+          <t>3 people – UNFUNDED</t>
         </is>
       </c>
       <c r="K28" s="96" t="inlineStr">
         <is>
-          <t>4 people</t>
+          <t>4 people – FUNDED ₮12M</t>
         </is>
       </c>
     </row>
@@ -25555,7 +25773,7 @@
         </is>
       </c>
       <c r="H32" s="101">
-        <f>Compare!$B$5-H31</f>
+        <f>Compare!$B$12-H31</f>
         <v/>
       </c>
       <c r="K32" s="101">
@@ -25623,6 +25841,7 @@
         <v/>
       </c>
     </row>
+    <row r="37"/>
     <row r="38" ht="15" customHeight="1" s="56">
       <c r="A38" s="72" t="inlineStr">
         <is>
@@ -25678,6 +25897,7 @@
         </is>
       </c>
     </row>
+    <row r="43"/>
     <row r="44" ht="15" customHeight="1" s="56">
       <c r="A44" s="72" t="inlineStr">
         <is>
@@ -25804,6 +26024,7 @@
         </is>
       </c>
     </row>
+    <row r="52"/>
     <row r="53" ht="15" customHeight="1" s="56">
       <c r="A53" s="72" t="inlineStr">
         <is>
@@ -26116,6 +26337,7 @@
       <c r="K63" s="107" t="n"/>
       <c r="L63" s="107" t="n"/>
     </row>
+    <row r="64"/>
     <row r="65" ht="15" customHeight="1" s="56">
       <c r="C65" s="59" t="inlineStr">
         <is>
@@ -27203,12 +27425,12 @@
       <c r="G34" s="60" t="n"/>
       <c r="H34" s="96" t="inlineStr">
         <is>
-          <t>3 people</t>
+          <t>3 people – UNFUNDED</t>
         </is>
       </c>
       <c r="K34" s="96" t="inlineStr">
         <is>
-          <t>4 people</t>
+          <t>4 people – FUNDED ₮12M</t>
         </is>
       </c>
     </row>
@@ -27264,7 +27486,7 @@
         </is>
       </c>
       <c r="H38" s="101">
-        <f>Compare!$B$5-H37</f>
+        <f>Compare!$B$12-H37</f>
         <v/>
       </c>
       <c r="K38" s="101">

</xml_diff>

<commit_message>
Hong Kong funded plan for 12M, likely pairing HK funded + Shenyang unfunded
- New Hong Kong - Funded 12M sheet (BW Plus 2 rooms, airport bus), Sleep check row
- Compare: left of 12M before contingency column, picks with the likely pairing
- details.md: funded/unfunded table, HK flight structure, Hunnu Air note

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ICPC_Single_Contest_Plans.xlsx
+++ b/ICPC_Single_Contest_Plans.xlsx
@@ -23,8 +23,9 @@
     <sheet name="Hong Kong – Comfort" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="Hong Kong – Value" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="Hong Kong – Sleep first" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="EC Final Hangzhou – Train" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="EC Final Hangzhou – Fly" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Hong Kong – Funded 12M" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="EC Final Hangzhou – Train" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="EC Final Hangzhou – Fly" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -893,12 +894,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:M47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="55" min="1" max="1"/>
     <col width="17" customWidth="1" style="55" min="2" max="11"/>
     <col width="22" customWidth="1" style="56" min="12" max="12"/>
+    <col width="24" customWidth="1" style="56" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.35" customHeight="1" s="56">
@@ -1107,7 +1109,12 @@
       </c>
       <c r="L14" s="66" t="inlineStr">
         <is>
-          <t>Fits ₮12M with the coach?</t>
+          <t>Fits ₮12M incl. 10% contingency?</t>
+        </is>
+      </c>
+      <c r="M14" s="66" t="inlineStr">
+        <is>
+          <t>Left of ₮12M before contingency (4 ppl)</t>
         </is>
       </c>
     </row>
@@ -1161,6 +1168,10 @@
         <f>IF(F15&gt;=0,"yes","over by "&amp;TEXT(-F15,"#,##0")&amp;" ₮")</f>
         <v/>
       </c>
+      <c r="M15" s="68">
+        <f>Compare!$B$5-E15/(1+Compare!$B$11)</f>
+        <v/>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="56">
       <c r="A16" s="67" t="inlineStr">
@@ -1212,6 +1223,10 @@
         <f>IF(F16&gt;=0,"yes","over by "&amp;TEXT(-F16,"#,##0")&amp;" ₮")</f>
         <v/>
       </c>
+      <c r="M16" s="68">
+        <f>Compare!$B$5-E16/(1+Compare!$B$11)</f>
+        <v/>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="56">
       <c r="A17" s="67" t="inlineStr">
@@ -1263,6 +1278,10 @@
         <f>IF(F17&gt;=0,"yes","over by "&amp;TEXT(-F17,"#,##0")&amp;" ₮")</f>
         <v/>
       </c>
+      <c r="M17" s="68">
+        <f>Compare!$B$5-E17/(1+Compare!$B$11)</f>
+        <v/>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="56">
       <c r="A18" s="67" t="inlineStr">
@@ -1314,6 +1333,10 @@
         <f>IF(F18&gt;=0,"yes","over by "&amp;TEXT(-F18,"#,##0")&amp;" ₮")</f>
         <v/>
       </c>
+      <c r="M18" s="68">
+        <f>Compare!$B$5-E18/(1+Compare!$B$11)</f>
+        <v/>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="56">
       <c r="A19" s="67" t="inlineStr">
@@ -1365,6 +1388,10 @@
         <f>IF(F19&gt;=0,"yes","over by "&amp;TEXT(-F19,"#,##0")&amp;" ₮")</f>
         <v/>
       </c>
+      <c r="M19" s="68">
+        <f>Compare!$B$5-E19/(1+Compare!$B$11)</f>
+        <v/>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="56">
       <c r="A20" s="67" t="inlineStr">
@@ -1416,6 +1443,10 @@
         <f>IF(F20&gt;=0,"yes","over by "&amp;TEXT(-F20,"#,##0")&amp;" ₮")</f>
         <v/>
       </c>
+      <c r="M20" s="68">
+        <f>Compare!$B$5-E20/(1+Compare!$B$11)</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="67" t="inlineStr">
@@ -1467,6 +1498,10 @@
         <f>IF(F21&gt;=0,"yes","over by "&amp;TEXT(-F21,"#,##0")&amp;" ₮")</f>
         <v/>
       </c>
+      <c r="M21" s="68">
+        <f>Compare!$B$5-E21/(1+Compare!$B$11)</f>
+        <v/>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="56">
       <c r="A22" s="67" t="inlineStr">
@@ -1518,6 +1553,10 @@
         <f>IF(F22&gt;=0,"yes","over by "&amp;TEXT(-F22,"#,##0")&amp;" ₮")</f>
         <v/>
       </c>
+      <c r="M22" s="68">
+        <f>Compare!$B$5-E22/(1+Compare!$B$11)</f>
+        <v/>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1" s="56">
       <c r="A23" s="67" t="inlineStr">
@@ -1569,6 +1608,10 @@
         <f>IF(F23&gt;=0,"yes","over by "&amp;TEXT(-F23,"#,##0")&amp;" ₮")</f>
         <v/>
       </c>
+      <c r="M23" s="68">
+        <f>Compare!$B$5-E23/(1+Compare!$B$11)</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1" s="56">
       <c r="A24" s="67" t="inlineStr">
@@ -1620,6 +1663,10 @@
         <f>IF(F24&gt;=0,"yes","over by "&amp;TEXT(-F24,"#,##0")&amp;" ₮")</f>
         <v/>
       </c>
+      <c r="M24" s="68">
+        <f>Compare!$B$5-E24/(1+Compare!$B$11)</f>
+        <v/>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1" s="56">
       <c r="A25" s="67" t="inlineStr">
@@ -1671,6 +1718,10 @@
         <f>IF(F25&gt;=0,"yes","over by "&amp;TEXT(-F25,"#,##0")&amp;" ₮")</f>
         <v/>
       </c>
+      <c r="M25" s="68">
+        <f>Compare!$B$5-E25/(1+Compare!$B$11)</f>
+        <v/>
+      </c>
     </row>
     <row r="26" s="56">
       <c r="A26" s="67" t="inlineStr">
@@ -1722,6 +1773,10 @@
         <f>IF(F26&gt;=0,"yes","over by "&amp;TEXT(-F26,"#,##0")&amp;" ₮")</f>
         <v/>
       </c>
+      <c r="M26" s="68">
+        <f>Compare!$B$5-E26/(1+Compare!$B$11)</f>
+        <v/>
+      </c>
     </row>
     <row r="27" ht="30" customHeight="1" s="56">
       <c r="A27" s="67" t="inlineStr">
@@ -1773,6 +1828,10 @@
         <f>IF(F27&gt;=0,"yes","over by "&amp;TEXT(-F27,"#,##0")&amp;" ₮")</f>
         <v/>
       </c>
+      <c r="M27" s="68">
+        <f>Compare!$B$5-E27/(1+Compare!$B$11)</f>
+        <v/>
+      </c>
     </row>
     <row r="28" s="56">
       <c r="A28" s="67" t="inlineStr">
@@ -1824,229 +1883,284 @@
         <f>IF(F28&gt;=0,"yes","over by "&amp;TEXT(-F28,"#,##0")&amp;" ₮")</f>
         <v/>
       </c>
-    </row>
-    <row r="29" ht="30" customHeight="1" s="56">
+      <c r="M28" s="68">
+        <f>Compare!$B$5-E28/(1+Compare!$B$11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" s="56">
       <c r="A29" s="67" t="inlineStr">
         <is>
-          <t>EC Final Hangzhou – Train</t>
+          <t>Hong Kong – Funded 12M</t>
         </is>
       </c>
       <c r="B29" s="68">
-        <f>'EC Final Hangzhou – Train'!H34</f>
+        <f>'Hong Kong – Funded 12M'!H30</f>
         <v/>
       </c>
       <c r="C29" s="68">
-        <f>'EC Final Hangzhou – Train'!H35</f>
+        <f>'Hong Kong – Funded 12M'!H31</f>
         <v/>
       </c>
       <c r="D29" s="69">
-        <f>'EC Final Hangzhou – Train'!H37</f>
+        <f>'Hong Kong – Funded 12M'!H33</f>
         <v/>
       </c>
       <c r="E29" s="68">
-        <f>'EC Final Hangzhou – Train'!K34</f>
+        <f>'Hong Kong – Funded 12M'!K30</f>
         <v/>
       </c>
       <c r="F29" s="68">
-        <f>'EC Final Hangzhou – Train'!K35</f>
+        <f>'Hong Kong – Funded 12M'!K31</f>
         <v/>
       </c>
       <c r="G29" s="69">
-        <f>'EC Final Hangzhou – Train'!K37</f>
+        <f>'Hong Kong – Funded 12M'!K33</f>
         <v/>
       </c>
       <c r="H29" s="70">
-        <f>'EC Final Hangzhou – Train'!H38</f>
+        <f>'Hong Kong – Funded 12M'!H34</f>
         <v/>
       </c>
       <c r="I29" s="70">
-        <f>'EC Final Hangzhou – Train'!K38</f>
+        <f>'Hong Kong – Funded 12M'!K34</f>
         <v/>
       </c>
       <c r="J29" s="71">
-        <f>'EC Final Hangzhou – Train'!H39</f>
+        <f>'Hong Kong – Funded 12M'!H35</f>
         <v/>
       </c>
       <c r="K29" s="71">
-        <f>'EC Final Hangzhou – Train'!D70</f>
+        <f>'Hong Kong – Funded 12M'!D60</f>
         <v/>
       </c>
       <c r="L29" s="123">
         <f>IF(F29&gt;=0,"yes","over by "&amp;TEXT(-F29,"#,##0")&amp;" ₮")</f>
         <v/>
       </c>
+      <c r="M29" s="68">
+        <f>Compare!$B$5-E29/(1+Compare!$B$11)</f>
+        <v/>
+      </c>
     </row>
     <row r="30" ht="30" customHeight="1" s="56">
       <c r="A30" s="67" t="inlineStr">
         <is>
-          <t>EC Final Hangzhou – Fly</t>
+          <t>EC Final Hangzhou – Train</t>
         </is>
       </c>
       <c r="B30" s="68">
-        <f>'EC Final Hangzhou – Fly'!H33</f>
+        <f>'EC Final Hangzhou – Train'!H34</f>
         <v/>
       </c>
       <c r="C30" s="68">
-        <f>'EC Final Hangzhou – Fly'!H34</f>
+        <f>'EC Final Hangzhou – Train'!H35</f>
         <v/>
       </c>
       <c r="D30" s="69">
-        <f>'EC Final Hangzhou – Fly'!H36</f>
+        <f>'EC Final Hangzhou – Train'!H37</f>
         <v/>
       </c>
       <c r="E30" s="68">
-        <f>'EC Final Hangzhou – Fly'!K33</f>
+        <f>'EC Final Hangzhou – Train'!K34</f>
         <v/>
       </c>
       <c r="F30" s="68">
-        <f>'EC Final Hangzhou – Fly'!K34</f>
+        <f>'EC Final Hangzhou – Train'!K35</f>
         <v/>
       </c>
       <c r="G30" s="69">
-        <f>'EC Final Hangzhou – Fly'!K36</f>
+        <f>'EC Final Hangzhou – Train'!K37</f>
         <v/>
       </c>
       <c r="H30" s="70">
-        <f>'EC Final Hangzhou – Fly'!H37</f>
+        <f>'EC Final Hangzhou – Train'!H38</f>
         <v/>
       </c>
       <c r="I30" s="70">
-        <f>'EC Final Hangzhou – Fly'!K37</f>
+        <f>'EC Final Hangzhou – Train'!K38</f>
         <v/>
       </c>
       <c r="J30" s="71">
-        <f>'EC Final Hangzhou – Fly'!H38</f>
+        <f>'EC Final Hangzhou – Train'!H39</f>
         <v/>
       </c>
       <c r="K30" s="71">
-        <f>'EC Final Hangzhou – Fly'!D70</f>
+        <f>'EC Final Hangzhou – Train'!D70</f>
         <v/>
       </c>
       <c r="L30" s="123">
         <f>IF(F30&gt;=0,"yes","over by "&amp;TEXT(-F30,"#,##0")&amp;" ₮")</f>
         <v/>
       </c>
+      <c r="M30" s="68">
+        <f>Compare!$B$5-E30/(1+Compare!$B$11)</f>
+        <v/>
+      </c>
     </row>
     <row r="31" ht="30" customHeight="1" s="56">
-      <c r="A31" s="75" t="n"/>
-      <c r="B31" s="74" t="n"/>
-    </row>
-    <row r="32" ht="15" customHeight="1" s="56">
-      <c r="A32" s="72" t="inlineStr">
+      <c r="A31" s="67" t="inlineStr">
+        <is>
+          <t>EC Final Hangzhou – Fly</t>
+        </is>
+      </c>
+      <c r="B31" s="68">
+        <f>'EC Final Hangzhou – Fly'!H33</f>
+        <v/>
+      </c>
+      <c r="C31" s="68">
+        <f>'EC Final Hangzhou – Fly'!H34</f>
+        <v/>
+      </c>
+      <c r="D31" s="69">
+        <f>'EC Final Hangzhou – Fly'!H36</f>
+        <v/>
+      </c>
+      <c r="E31" s="68">
+        <f>'EC Final Hangzhou – Fly'!K33</f>
+        <v/>
+      </c>
+      <c r="F31" s="68">
+        <f>'EC Final Hangzhou – Fly'!K34</f>
+        <v/>
+      </c>
+      <c r="G31" s="69">
+        <f>'EC Final Hangzhou – Fly'!K36</f>
+        <v/>
+      </c>
+      <c r="H31" s="70">
+        <f>'EC Final Hangzhou – Fly'!H37</f>
+        <v/>
+      </c>
+      <c r="I31" s="70">
+        <f>'EC Final Hangzhou – Fly'!K37</f>
+        <v/>
+      </c>
+      <c r="J31" s="71">
+        <f>'EC Final Hangzhou – Fly'!H38</f>
+        <v/>
+      </c>
+      <c r="K31" s="71">
+        <f>'EC Final Hangzhou – Fly'!D70</f>
+        <v/>
+      </c>
+      <c r="L31" s="123">
+        <f>IF(F31&gt;=0,"yes","over by "&amp;TEXT(-F31,"#,##0")&amp;" ₮")</f>
+        <v/>
+      </c>
+      <c r="M31" s="68">
+        <f>Compare!$B$5-E31/(1+Compare!$B$11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1" s="56">
+      <c r="A32" s="75" t="n"/>
+      <c r="B32" s="74" t="n"/>
+    </row>
+    <row r="33" ht="15" customHeight="1" s="56">
+      <c r="A33" s="72" t="inlineStr">
         <is>
           <t>Recommended picks (not the expensive ones)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="62" customHeight="1" s="56">
-      <c r="A33" s="73" t="inlineStr">
-        <is>
-          <t>Unfunded regional (3 ppl pay)</t>
-        </is>
-      </c>
-      <c r="B33" s="74" t="inlineStr">
-        <is>
-          <t>Cheapest sleep-safe plans per person incl. fee, taxi, insurance, eSIM and 10% contingency: Shenyang – Budget ₮2.14M per person (soft sleeper before day 1); Shenyang – Comfort ₮2.46M per person; Nanchang – Sleeper ₮2.50M per person; Shanghai – Sleeper ₮2.89M per person; Hong Kong – Budget ₮3.43M per person; EC Final – Train ₮3.14M per person. Shenyang and Nanchang are the cheap ones to pay yourselves.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="62" customHeight="1" s="56">
       <c r="A34" s="73" t="inlineStr">
         <is>
+          <t>Likely pairing (your answer)</t>
+        </is>
+      </c>
+      <c r="B34" s="74" t="inlineStr">
+        <is>
+          <t>Funded = Hong Kong (₮12M, coach): 'Hong Kong – Funded 12M' (MIAT nonstop, 2 rooms ~540 m from HKU, airport bus) costs ₮11.70M before the 10% contingency (₮0.30M spare) and ₮12.87M with it – lock the flights first. Unfunded = Shenyang: Budget ₮2.14M per person (≈ $594; flights are 58% of it), Comfort ₮2.46M per person. The two together are the cheapest sleep-safe pairing; Shanghai or Nanchang as the unfunded one would cost ₮2.50M per person / ₮2.89M per person.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="62" customHeight="1" s="56">
+      <c r="A35" s="73" t="inlineStr">
+        <is>
+          <t>Unfunded regional (3 ppl pay)</t>
+        </is>
+      </c>
+      <c r="B35" s="74" t="inlineStr">
+        <is>
+          <t>Cheapest sleep-safe plans per person incl. fee, taxi, insurance, eSIM and 10% contingency: Shenyang – Budget ₮2.14M per person (soft sleeper before day 1); Shenyang – Comfort ₮2.46M per person; Nanchang – Sleeper ₮2.50M per person; Shanghai – Sleeper ₮2.89M per person; Hong Kong – Budget ₮3.43M per person; EC Final – Train ₮3.14M per person. Shenyang and Nanchang are the cheap ones to pay yourselves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="62" customHeight="1" s="56">
+      <c r="A36" s="73" t="inlineStr">
+        <is>
           <t>Funded regional (₮12M, coach)</t>
         </is>
       </c>
-      <c r="B34" s="74" t="inlineStr">
-        <is>
-          <t>Fits ₮12M: Shenyang – Comfort ₮8.04M (fits, ₮3.96M left); Shanghai – Sleeper ₮9.83M (fits, ₮2.17M left); Nanchang – Sleeper ₮8.19M (fits, ₮3.81M left); EC Final – Train ₮11.12M (fits, ₮0.88M left). Hong Kong – Budget ₮12.12M (over by ₮0.12M) only works without the 10% contingency (subtotal ~₮11.0M); Hong Kong Value / Comfort / Sleep first and EC Final – Fly do not fit. Use the funded trip for the dearest contest you must attend (Shanghai, Hong Kong, EC Final) and pay the cheap one yourselves.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="47" customHeight="1" s="56">
-      <c r="A35" s="73" t="inlineStr">
-        <is>
-          <t>Regional – Shenyang (14–15 Nov)</t>
-        </is>
-      </c>
-      <c r="B35" s="74" t="inlineStr">
-        <is>
-          <t>Comfort: rest day, RiCH family room 1.3 km from NEU, hard sleeper home after the contest. No sleepers at all: G-train Comfort ₮6.72M / ₮8.84M, G-train Budget ₮6.05M / ₮8.27M (3 / 4 ppl). Fly home on Air China 12:55 ($171).</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="47" customHeight="1" s="56">
-      <c r="A36" s="73" t="inlineStr">
-        <is>
-          <t>Regional – Shanghai (5–6 Dec)</t>
-        </is>
-      </c>
       <c r="B36" s="74" t="inlineStr">
         <is>
-          <t>Sleeper: MIAT $151 + G17 out on 3 Dec, Jenny's Apartment 3 nights (1 km), D8 overnight seat back, Air China 12:55 $172 on 7 Dec. Spring nonstop (Tue 1 → Tue 8 Dec, 7 nights) ₮8.21M / ₮10.73M; day train home with a Beijing night ₮8.11M / ₮10.78M. Wildcard: email shu_icpc@163.com now.</t>
+          <t>Fits ₮12M incl. contingency: Shenyang – Comfort ₮8.04M (fits, ₮3.96M left); Shanghai – Sleeper ₮9.83M (fits, ₮2.17M left); Nanchang – Sleeper ₮8.19M (fits, ₮3.81M left); EC Final – Train ₮11.12M (fits, ₮0.88M left). Hong Kong only fits before the 10% contingency (the flights are ₮8.4M of it): Budget ₮11.02M, Value ₮11.26M, Funded 12M ₮11.70M, Comfort ₮11.96M; Sleep first ₮13.14M and EC Final – Fly do not fit at all. Use the funded trip for the dearest contest you must attend and pay the cheap one yourselves.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="47" customHeight="1" s="56">
       <c r="A37" s="73" t="inlineStr">
         <is>
-          <t>Regional – Nanchang (19–20 Dec)</t>
+          <t>Regional – Shenyang (14–15 Nov)</t>
         </is>
       </c>
       <c r="B37" s="74" t="inlineStr">
         <is>
-          <t>Sleeper: Air China $157 + Z111 hard sleeper (arrive 11:52 on 18 Dec), Orange Hotel 2 nights, D136 seat back, Air China 12:55 $172. Comfort (daytime G-train, 3 hotel nights) ₮7.96M / ₮10.32M; Fly in (Air China through ticket $356) ₮8.41M / ₮10.95M.</t>
+          <t>Comfort: rest day, RiCH family room 1.3 km from NEU, hard sleeper home after the contest. No sleepers at all: G-train Comfort ₮6.72M / ₮8.84M, G-train Budget ₮6.05M / ₮8.27M (3 / 4 ppl). Fly home on Air China 12:55 ($171).</t>
         </is>
       </c>
     </row>
     <row r="38" ht="47" customHeight="1" s="56">
       <c r="A38" s="73" t="inlineStr">
         <is>
-          <t>Regional – Hong Kong (9–10 Jan)</t>
+          <t>Regional – Shanghai (5–6 Dec)</t>
         </is>
       </c>
       <c r="B38" s="74" t="inlineStr">
         <is>
-          <t>MIAT nonstop ($586 return on Trip.com, low against the usual $708–900) is the cheapest way in. Budget guesthouse ₮9.08M / ₮12.12M; Value (Kusa Inn 9.6) ₮9.08M / ₮12.38M; Sleep first (2 rooms near HKU) ₮11.63M / ₮14.45M. No route or date is cheaper (checked 10 Oct).</t>
+          <t>Sleeper: MIAT $151 + G17 out on 3 Dec, Jenny's Apartment 3 nights (1 km), D8 overnight seat back, Air China 12:55 $172 on 7 Dec. Spring nonstop (Tue 1 → Tue 8 Dec, 7 nights) ₮8.21M / ₮10.73M; day train home with a Beijing night ₮8.11M / ₮10.78M. Wildcard: email shu_icpc@163.com now.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="47" customHeight="1" s="56">
       <c r="A39" s="73" t="inlineStr">
         <is>
+          <t>Regional – Nanchang (19–20 Dec)</t>
+        </is>
+      </c>
+      <c r="B39" s="74" t="inlineStr">
+        <is>
+          <t>Sleeper: Air China $157 + Z111 hard sleeper (arrive 11:52 on 18 Dec), Orange Hotel 2 nights, D136 seat back, Air China 12:55 $172. Comfort (daytime G-train, 3 hotel nights) ₮7.96M / ₮10.32M; Fly in (Air China through ticket $356) ₮8.41M / ₮10.95M.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="47" customHeight="1" s="56">
+      <c r="A40" s="73" t="inlineStr">
+        <is>
+          <t>Regional – Hong Kong (9–10 Jan)</t>
+        </is>
+      </c>
+      <c r="B40" s="74" t="inlineStr">
+        <is>
+          <t>MIAT nonstop ($586 return on Trip.com, low against the usual $708–900) is the cheapest way in. Budget guesthouse ₮9.08M / ₮12.12M; Value (Kusa Inn 9.6) ₮9.08M / ₮12.38M; Sleep first (2 rooms near HKU) ₮11.63M / ₮14.45M. No route or date is cheaper (checked 10 Oct).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="47" customHeight="1" s="56">
+      <c r="A41" s="73" t="inlineStr">
+        <is>
           <t>EC Final (only if qualified)</t>
         </is>
       </c>
-      <c r="B39" s="74" t="inlineStr">
+      <c r="B41" s="74" t="inlineStr">
         <is>
           <t>Train: MIAT to Beijing, D17 overnight sleeper Beijing 19:10 → Hangzhou 09:15 (¥491), Air China through ticket Hangzhou → UB on 29 Jan: ₮11.12M (fits, ₮0.88M left) for 4 ppl, ₮3.14M per person for 3. Fly (Aero Mongolia + Xiamen via Hohhot) is ₮14.82M (over by ₮2.82M) – does not fit ₮12M. Buy D17 on 12306 at 10:00 on 11 Jan.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="18" customHeight="1" s="56"/>
-    <row r="41" ht="32" customHeight="1" s="56">
-      <c r="A41" s="75" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B41" s="74" t="inlineStr">
-        <is>
-          <t>Dates are provisional (ICPC Beijing HQ summary, 5 Aug 2026). Hong Kong host (HKU) and EC Final venue (HZNU Cangqian) are from secondary sources; Shanghai (Shanghai University Baoshan) follows the 2025 invitation and Nanchang (Jiangxi Normal University Yaohu campus) the 2019 handbook – confirm each invitation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="18" customHeight="1" s="56">
-      <c r="A42" s="75" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B42" s="74" t="inlineStr">
-        <is>
-          <t>EC Final is qualification-only: plan it only once the team has earned a slot at a regional.</t>
-        </is>
-      </c>
-    </row>
+    <row r="42" ht="32" customHeight="1" s="56"/>
     <row r="43" ht="32" customHeight="1" s="56">
       <c r="A43" s="75" t="inlineStr">
         <is>
@@ -2055,11 +2169,11 @@
       </c>
       <c r="B43" s="74" t="inlineStr">
         <is>
-          <t>4-person plans use whatever split is cheapest on Trip.com/Booking.com: one family room for 4 (Shenyang RiCH, Nanchang Orange Hotel), or two rooms. Taxi costs assume one car; with luggage 4 people may need an XL car.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="47" customHeight="1" s="56">
+          <t>Dates are provisional (ICPC Beijing HQ summary, 5 Aug 2026). Hong Kong host (HKU) and EC Final venue (HZNU Cangqian) are from secondary sources; Shanghai (Shanghai University Baoshan) follows the 2025 invitation and Nanchang (Jiangxi Normal University Yaohu campus) the 2019 handbook – confirm each invitation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1" s="56">
       <c r="A44" s="75" t="inlineStr">
         <is>
           <t>Note</t>
@@ -2067,7 +2181,7 @@
       </c>
       <c r="B44" s="74" t="inlineStr">
         <is>
-          <t>Sleep rule (see the 'Sleep check' sheet): the two nights before each contest day are in a quiet bed near the venue; sleepers, early flights and red-eyes are only used before day 1 (soft sleeper) or after the contest (anything goes). Sleeper trains replace hotel nights in the Shenyang, Shanghai (D8 seat), Nanchang (Z111 / D136 seat) and EC Final (D17) plans; the 'G-train' / 'no sleeper' variants cost more per trip. Chinese train tickets go on sale 14 days ahead – dates are in the '12306 &amp; ChinaTicketOnline' and '10 Oct' sheets of the fares workbook.</t>
+          <t>EC Final is qualification-only: plan it only once the team has earned a slot at a regional.</t>
         </is>
       </c>
     </row>
@@ -2079,48 +2193,48 @@
       </c>
       <c r="B45" s="74" t="inlineStr">
         <is>
+          <t>4-person plans use whatever split is cheapest on Trip.com/Booking.com: one family room for 4 (Shenyang RiCH, Nanchang Orange Hotel), or two rooms. Taxi costs assume one car; with luggage 4 people may need an XL car.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="47" customHeight="1" s="56">
+      <c r="A46" s="75" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B46" s="74" t="inlineStr">
+        <is>
+          <t>Sleep rule (see the 'Sleep check' sheet): the two nights before each contest day are in a quiet bed near the venue; sleepers, early flights and red-eyes are only used before day 1 (soft sleeper) or after the contest (anything goes). Sleeper trains replace hotel nights in the Shenyang, Shanghai (D8 seat), Nanchang (Z111 / D136 seat) and EC Final (D17) plans; the 'G-train' / 'no sleeper' variants cost more per trip. Chinese train tickets go on sale 14 days ahead – dates are in the '12306 &amp; ChinaTicketOnline' and '10 Oct' sheets of the fares workbook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="32" customHeight="1" s="56">
+      <c r="A47" s="75" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B47" s="74" t="inlineStr">
+        <is>
           <t>Sources (10 Oct): Trip.com (flights and hotels, built-in browser), 12306 (official train fares), ChinaTicketOnline (timetable and sale-date check; 30–70% dearer than 12306, not used for booking), SlickTrip (MIAT / Spring fares; Air China is unpriced there).</t>
         </is>
       </c>
     </row>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="72"/>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="B45:K45"/>
+    <mergeCell ref="B46:K46"/>
     <mergeCell ref="B41:K41"/>
+    <mergeCell ref="B40:K40"/>
     <mergeCell ref="B35:K35"/>
     <mergeCell ref="B44:K44"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B43:K43"/>
     <mergeCell ref="B39:K39"/>
     <mergeCell ref="B38:K38"/>
+    <mergeCell ref="B47:K47"/>
     <mergeCell ref="B34:K34"/>
-    <mergeCell ref="B33:K33"/>
-    <mergeCell ref="B42:K42"/>
     <mergeCell ref="B36:K36"/>
     <mergeCell ref="B37:K37"/>
   </mergeCells>
@@ -2166,7 +2280,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -2189,7 +2302,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -3041,7 +3153,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31" ht="15" customHeight="1" s="56">
       <c r="G31" s="60" t="n"/>
       <c r="H31" s="96" t="inlineStr">
@@ -3175,7 +3286,6 @@
         <v/>
       </c>
     </row>
-    <row r="40"/>
     <row r="41" ht="15" customHeight="1" s="56">
       <c r="A41" s="72" t="inlineStr">
         <is>
@@ -3231,7 +3341,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47" ht="15" customHeight="1" s="56">
       <c r="A47" s="72" t="inlineStr">
         <is>
@@ -3341,7 +3450,6 @@
         </is>
       </c>
     </row>
-    <row r="54"/>
     <row r="55" ht="15" customHeight="1" s="56">
       <c r="A55" s="72" t="inlineStr">
         <is>
@@ -3746,7 +3854,6 @@
       <c r="K68" s="107" t="n"/>
       <c r="L68" s="107" t="n"/>
     </row>
-    <row r="69"/>
     <row r="70" ht="15" customHeight="1" s="56">
       <c r="C70" s="59" t="inlineStr">
         <is>
@@ -3822,7 +3929,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -3845,7 +3951,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -4787,7 +4892,6 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
     <row r="33" ht="15" customHeight="1" s="56">
       <c r="G33" s="60" t="n"/>
       <c r="H33" s="96" t="inlineStr">
@@ -4921,7 +5025,6 @@
         <v/>
       </c>
     </row>
-    <row r="42"/>
     <row r="43" ht="15" customHeight="1" s="56">
       <c r="A43" s="72" t="inlineStr">
         <is>
@@ -4977,7 +5080,6 @@
         </is>
       </c>
     </row>
-    <row r="48"/>
     <row r="49" ht="15" customHeight="1" s="56">
       <c r="A49" s="72" t="inlineStr">
         <is>
@@ -5087,7 +5189,6 @@
         </is>
       </c>
     </row>
-    <row r="56"/>
     <row r="57" ht="15" customHeight="1" s="56">
       <c r="A57" s="72" t="inlineStr">
         <is>
@@ -5492,7 +5593,6 @@
       <c r="K70" s="107" t="n"/>
       <c r="L70" s="107" t="n"/>
     </row>
-    <row r="71"/>
     <row r="72" ht="15" customHeight="1" s="56">
       <c r="C72" s="59" t="inlineStr">
         <is>
@@ -5568,7 +5668,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -5591,7 +5690,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -6439,7 +6537,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31" ht="15" customHeight="1" s="56">
       <c r="G31" s="60" t="n"/>
       <c r="H31" s="96" t="inlineStr">
@@ -6573,7 +6670,6 @@
         <v/>
       </c>
     </row>
-    <row r="40"/>
     <row r="41" ht="15" customHeight="1" s="56">
       <c r="A41" s="72" t="inlineStr">
         <is>
@@ -6629,7 +6725,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47" ht="15" customHeight="1" s="56">
       <c r="A47" s="72" t="inlineStr">
         <is>
@@ -6739,7 +6834,6 @@
         </is>
       </c>
     </row>
-    <row r="54"/>
     <row r="55" ht="15" customHeight="1" s="56">
       <c r="A55" s="72" t="inlineStr">
         <is>
@@ -7088,7 +7182,6 @@
       <c r="K66" s="107" t="n"/>
       <c r="L66" s="107" t="n"/>
     </row>
-    <row r="67"/>
     <row r="68" ht="15" customHeight="1" s="56">
       <c r="C68" s="59" t="inlineStr">
         <is>
@@ -7162,7 +7255,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -7185,7 +7277,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -7878,7 +7969,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27" ht="15" customHeight="1" s="56">
       <c r="G27" s="60" t="n"/>
       <c r="H27" s="96" t="inlineStr">
@@ -8012,7 +8102,6 @@
         <v/>
       </c>
     </row>
-    <row r="36"/>
     <row r="37" ht="15" customHeight="1" s="56">
       <c r="A37" s="72" t="inlineStr">
         <is>
@@ -8068,7 +8157,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43" ht="15" customHeight="1" s="56">
       <c r="A43" s="72" t="inlineStr">
         <is>
@@ -8161,7 +8249,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
     <row r="50" ht="15" customHeight="1" s="56">
       <c r="A50" s="72" t="inlineStr">
         <is>
@@ -8520,7 +8607,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -8543,7 +8629,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -9236,7 +9321,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27" ht="15" customHeight="1" s="56">
       <c r="G27" s="60" t="n"/>
       <c r="H27" s="96" t="inlineStr">
@@ -9370,7 +9454,6 @@
         <v/>
       </c>
     </row>
-    <row r="36"/>
     <row r="37" ht="15" customHeight="1" s="56">
       <c r="A37" s="72" t="inlineStr">
         <is>
@@ -9426,7 +9509,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43" ht="15" customHeight="1" s="56">
       <c r="A43" s="72" t="inlineStr">
         <is>
@@ -9519,7 +9601,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
     <row r="50" ht="15" customHeight="1" s="56">
       <c r="A50" s="72" t="inlineStr">
         <is>
@@ -9878,7 +9959,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -9901,7 +9981,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -10594,7 +10673,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27" ht="15" customHeight="1" s="56">
       <c r="G27" s="60" t="n"/>
       <c r="H27" s="96" t="inlineStr">
@@ -10728,7 +10806,6 @@
         <v/>
       </c>
     </row>
-    <row r="36"/>
     <row r="37" ht="15" customHeight="1" s="56">
       <c r="A37" s="72" t="inlineStr">
         <is>
@@ -10784,7 +10861,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43" ht="15" customHeight="1" s="56">
       <c r="A43" s="72" t="inlineStr">
         <is>
@@ -10877,7 +10953,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
     <row r="50" ht="15" customHeight="1" s="56">
       <c r="A50" s="72" t="inlineStr">
         <is>
@@ -11236,7 +11311,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -11259,7 +11333,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -11952,7 +12025,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27" ht="15" customHeight="1" s="56">
       <c r="G27" s="60" t="n"/>
       <c r="H27" s="96" t="inlineStr">
@@ -12086,7 +12158,6 @@
         <v/>
       </c>
     </row>
-    <row r="36"/>
     <row r="37" ht="15" customHeight="1" s="56">
       <c r="A37" s="72" t="inlineStr">
         <is>
@@ -12142,7 +12213,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43" ht="15" customHeight="1" s="56">
       <c r="A43" s="72" t="inlineStr">
         <is>
@@ -12235,7 +12305,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
     <row r="50" ht="15" customHeight="1" s="56">
       <c r="A50" s="72" t="inlineStr">
         <is>
@@ -12564,6 +12633,1358 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
+  <dimension ref="A1:L60"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="26" customWidth="1" style="55" min="1" max="1"/>
+    <col width="52" customWidth="1" style="55" min="2" max="2"/>
+    <col width="20" customWidth="1" style="55" min="3" max="3"/>
+    <col width="15" customWidth="1" style="55" min="4" max="4"/>
+    <col width="13" customWidth="1" style="55" min="5" max="5"/>
+    <col width="9" customWidth="1" style="55" min="6" max="7"/>
+    <col width="17" customWidth="1" style="55" min="8" max="8"/>
+    <col width="13" customWidth="1" style="55" min="9" max="9"/>
+    <col width="9" customWidth="1" style="55" min="10" max="10"/>
+    <col width="17" customWidth="1" style="55" min="11" max="11"/>
+    <col width="58" customWidth="1" style="55" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="17.35" customHeight="1" s="56">
+      <c r="A1" s="57" t="inlineStr">
+        <is>
+          <t>Hong Kong – Funded 12M</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1" s="56">
+      <c r="A2" s="62" t="inlineStr">
+        <is>
+          <t>For the funded regional (₮12M, coach travels): MIAT nonstop, two rooms at a hotel ~540 m from HKU (walk, no commute) so each contestant has a bed and the contest-eve sleep is protected; airport bus instead of the Airport Express to stay under the cap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="56">
+      <c r="A4" s="60" t="inlineStr">
+        <is>
+          <t>Days in destination (meals &amp; local transport)</t>
+        </is>
+      </c>
+      <c r="B4" s="76" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="C4" s="62" t="inlineStr">
+        <is>
+          <t>8 Jan midday → 11 Jan morning</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="56">
+      <c r="A5" s="62" t="inlineStr">
+        <is>
+          <t>Shared inputs are on the Compare sheet. Scroll down for the day-by-day plan and door-to-door travel times.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="31.5" customHeight="1" s="56">
+      <c r="A7" s="66" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B7" s="66" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C7" s="66" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D7" s="66" t="inlineStr">
+        <is>
+          <t>Travel time</t>
+        </is>
+      </c>
+      <c r="E7" s="66" t="inlineStr">
+        <is>
+          <t>Unit cost (3 ppl)</t>
+        </is>
+      </c>
+      <c r="F7" s="66" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="G7" s="66" t="inlineStr">
+        <is>
+          <t>Qty (3 ppl)</t>
+        </is>
+      </c>
+      <c r="H7" s="66" t="inlineStr">
+        <is>
+          <t>Total MNT – 3 people</t>
+        </is>
+      </c>
+      <c r="I7" s="66" t="inlineStr">
+        <is>
+          <t>Unit cost (4 ppl)</t>
+        </is>
+      </c>
+      <c r="J7" s="66" t="inlineStr">
+        <is>
+          <t>Qty (4 ppl)</t>
+        </is>
+      </c>
+      <c r="K7" s="66" t="inlineStr">
+        <is>
+          <t>Total MNT – 4 people</t>
+        </is>
+      </c>
+      <c r="L7" s="66" t="inlineStr">
+        <is>
+          <t>Source / notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="56">
+      <c r="A8" s="77" t="inlineStr">
+        <is>
+          <t>PAID BY UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="B8" s="78" t="n"/>
+      <c r="C8" s="78" t="n"/>
+      <c r="D8" s="78" t="n"/>
+      <c r="E8" s="78" t="n"/>
+      <c r="F8" s="78" t="n"/>
+      <c r="G8" s="78" t="n"/>
+      <c r="H8" s="78" t="n"/>
+      <c r="I8" s="78" t="n"/>
+      <c r="J8" s="78" t="n"/>
+      <c r="K8" s="78" t="n"/>
+      <c r="L8" s="78" t="n"/>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="56">
+      <c r="A9" s="79" t="inlineStr">
+        <is>
+          <t>Flights</t>
+        </is>
+      </c>
+      <c r="B9" s="80" t="n"/>
+      <c r="C9" s="80" t="n"/>
+      <c r="D9" s="80" t="n"/>
+      <c r="E9" s="80" t="n"/>
+      <c r="F9" s="80" t="n"/>
+      <c r="G9" s="80" t="n"/>
+      <c r="H9" s="80" t="n"/>
+      <c r="I9" s="80" t="n"/>
+      <c r="J9" s="80" t="n"/>
+      <c r="K9" s="80" t="n"/>
+      <c r="L9" s="80" t="n"/>
+    </row>
+    <row r="10" ht="26.85" customHeight="1" s="56">
+      <c r="A10" s="81" t="n"/>
+      <c r="B10" s="82" t="inlineStr">
+        <is>
+          <t>MIAT OM297 Ulaanbaatar → Hong Kong, nonstop 06:45–11:25</t>
+        </is>
+      </c>
+      <c r="C10" s="83" t="inlineStr">
+        <is>
+          <t>8 Jan</t>
+        </is>
+      </c>
+      <c r="D10" s="84" t="n">
+        <v>0.1944444444444444</v>
+      </c>
+      <c r="E10" s="85" t="n">
+        <v>293</v>
+      </c>
+      <c r="F10" s="86" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G10" s="87">
+        <f>Compare!$B$6</f>
+        <v/>
+      </c>
+      <c r="H10" s="88">
+        <f>E10*G10*IF(F10="USD",Compare!$B$8,IF(F10="CNY",Compare!$B$9,IF(F10="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I10" s="89">
+        <f>E10</f>
+        <v/>
+      </c>
+      <c r="J10" s="87">
+        <f>Compare!$B$7</f>
+        <v/>
+      </c>
+      <c r="K10" s="88">
+        <f>I10*J10*IF(F10="USD",Compare!$B$8,IF(F10="CNY",Compare!$B$9,IF(F10="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L10" s="90" t="inlineStr">
+        <is>
+          <t>Trip.com 10 Oct: MIAT nonstop 07:15–11:50 round trip $586 pp (8–11 Jan), split half each way = $293 (SlickTrip $593; $583 on 30 Sep). Cathay codeshare $626; via Seoul $783+</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="26.85" customHeight="1" s="56">
+      <c r="A11" s="81" t="n"/>
+      <c r="B11" s="82" t="inlineStr">
+        <is>
+          <t>MIAT OM298 Hong Kong → Ulaanbaatar, nonstop 12:25–17:05</t>
+        </is>
+      </c>
+      <c r="C11" s="83" t="inlineStr">
+        <is>
+          <t>11 Jan</t>
+        </is>
+      </c>
+      <c r="D11" s="84" t="n">
+        <v>0.1944444444444444</v>
+      </c>
+      <c r="E11" s="85" t="n">
+        <v>293</v>
+      </c>
+      <c r="F11" s="86" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G11" s="87">
+        <f>Compare!$B$6</f>
+        <v/>
+      </c>
+      <c r="H11" s="88">
+        <f>E11*G11*IF(F11="USD",Compare!$B$8,IF(F11="CNY",Compare!$B$9,IF(F11="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I11" s="89">
+        <f>E11</f>
+        <v/>
+      </c>
+      <c r="J11" s="87">
+        <f>Compare!$B$7</f>
+        <v/>
+      </c>
+      <c r="K11" s="88">
+        <f>I11*J11*IF(F11="USD",Compare!$B$8,IF(F11="CNY",Compare!$B$9,IF(F11="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L11" s="90" t="inlineStr">
+        <is>
+          <t>Return half of the $586 pp Trip.com round trip</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="56">
+      <c r="A12" s="79" t="inlineStr">
+        <is>
+          <t>Accommodation</t>
+        </is>
+      </c>
+      <c r="B12" s="80" t="n"/>
+      <c r="C12" s="80" t="n"/>
+      <c r="D12" s="80" t="n"/>
+      <c r="E12" s="80" t="n"/>
+      <c r="F12" s="80" t="n"/>
+      <c r="G12" s="80" t="n"/>
+      <c r="H12" s="80" t="n"/>
+      <c r="I12" s="80" t="n"/>
+      <c r="J12" s="80" t="n"/>
+      <c r="K12" s="80" t="n"/>
+      <c r="L12" s="80" t="n"/>
+    </row>
+    <row r="13" ht="26.85" customHeight="1" s="56">
+      <c r="A13" s="81" t="n"/>
+      <c r="B13" s="82" t="inlineStr">
+        <is>
+          <t>Best Western Plus Hotel Hong Kong, Sai Ying Pun (~540 m to HKU; 3 ppl 1 room; 4 ppl 2 rooms, 2 beds each)</t>
+        </is>
+      </c>
+      <c r="C13" s="83" t="inlineStr">
+        <is>
+          <t>8–11 Jan (3 nights)</t>
+        </is>
+      </c>
+      <c r="D13" s="81" t="n"/>
+      <c r="E13" s="85" t="n">
+        <v>713</v>
+      </c>
+      <c r="F13" s="86" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="G13" s="91" t="n">
+        <v>3</v>
+      </c>
+      <c r="H13" s="88">
+        <f>E13*G13*IF(F13="USD",Compare!$B$8,IF(F13="CNY",Compare!$B$9,IF(F13="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I13" s="85" t="n">
+        <v>1213.33</v>
+      </c>
+      <c r="J13" s="91" t="n">
+        <v>3</v>
+      </c>
+      <c r="K13" s="88">
+        <f>I13*J13*IF(F13="USD",Compare!$B$8,IF(F13="CNY",Compare!$B$9,IF(F13="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L13" s="90" t="inlineStr">
+        <is>
+          <t>Booking.com 8–11 Jan: HK$2,139 (3 ppl) / HK$3,640 (4 ppl, 2 rooms) for 3 nights; rated 7.4 (4,583 reviews) on Booking.com, 8.2 (3,331) on Trip.com where 4 ppl / 2 rooms is HK$4,243. Read recent noise reviews; the cheaper guesthouses (Good Fortune Inn 8.6, 4 twin beds, HK$2,889) are ~35 min away by MTR</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1" s="56">
+      <c r="A14" s="79" t="inlineStr">
+        <is>
+          <t>Meals &amp; local transport</t>
+        </is>
+      </c>
+      <c r="B14" s="80" t="n"/>
+      <c r="C14" s="80" t="n"/>
+      <c r="D14" s="80" t="n"/>
+      <c r="E14" s="80" t="n"/>
+      <c r="F14" s="80" t="n"/>
+      <c r="G14" s="80" t="n"/>
+      <c r="H14" s="80" t="n"/>
+      <c r="I14" s="80" t="n"/>
+      <c r="J14" s="80" t="n"/>
+      <c r="K14" s="80" t="n"/>
+      <c r="L14" s="80" t="n"/>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="56">
+      <c r="A15" s="81" t="n"/>
+      <c r="B15" s="82" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="C15" s="83" t="inlineStr">
+        <is>
+          <t>in Hong Kong</t>
+        </is>
+      </c>
+      <c r="D15" s="81" t="n"/>
+      <c r="E15" s="92" t="n">
+        <v>180</v>
+      </c>
+      <c r="F15" s="86" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="G15" s="87">
+        <f>Compare!$B$6*$B$4</f>
+        <v/>
+      </c>
+      <c r="H15" s="88">
+        <f>E15*G15*IF(F15="USD",Compare!$B$8,IF(F15="CNY",Compare!$B$9,IF(F15="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I15" s="93">
+        <f>E15</f>
+        <v/>
+      </c>
+      <c r="J15" s="87">
+        <f>Compare!$B$7*$B$4</f>
+        <v/>
+      </c>
+      <c r="K15" s="88">
+        <f>I15*J15*IF(F15="USD",Compare!$B$8,IF(F15="CNY",Compare!$B$9,IF(F15="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L15" s="90" t="inlineStr">
+        <is>
+          <t>ASSUMPTION ~180 HKD/person/day (cha chaan teng, canteens)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="56">
+      <c r="A16" s="81" t="n"/>
+      <c r="B16" s="82" t="inlineStr">
+        <is>
+          <t>MTR / buses (Octopus card)</t>
+        </is>
+      </c>
+      <c r="C16" s="83" t="inlineStr">
+        <is>
+          <t>in Hong Kong</t>
+        </is>
+      </c>
+      <c r="D16" s="81" t="n"/>
+      <c r="E16" s="92" t="n">
+        <v>40</v>
+      </c>
+      <c r="F16" s="86" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="G16" s="87">
+        <f>Compare!$B$6*$B$4</f>
+        <v/>
+      </c>
+      <c r="H16" s="88">
+        <f>E16*G16*IF(F16="USD",Compare!$B$8,IF(F16="CNY",Compare!$B$9,IF(F16="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I16" s="93">
+        <f>E16</f>
+        <v/>
+      </c>
+      <c r="J16" s="87">
+        <f>Compare!$B$7*$B$4</f>
+        <v/>
+      </c>
+      <c r="K16" s="88">
+        <f>I16*J16*IF(F16="USD",Compare!$B$8,IF(F16="CNY",Compare!$B$9,IF(F16="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L16" s="90" t="inlineStr">
+        <is>
+          <t>ASSUMPTION ~40 HKD/person/day</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1" s="56">
+      <c r="A17" s="81" t="n"/>
+      <c r="B17" s="82" t="inlineStr">
+        <is>
+          <t>Airport bus A10 / A12 (HKG ↔ Sheung Wan / Sai Ying Pun), both ways</t>
+        </is>
+      </c>
+      <c r="C17" s="83" t="inlineStr">
+        <is>
+          <t>8 &amp; 11 Jan</t>
+        </is>
+      </c>
+      <c r="D17" s="81" t="n"/>
+      <c r="E17" s="92" t="n">
+        <v>90</v>
+      </c>
+      <c r="F17" s="86" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="G17" s="87">
+        <f>Compare!$B$6</f>
+        <v/>
+      </c>
+      <c r="H17" s="88">
+        <f>E17*G17*IF(F17="USD",Compare!$B$8,IF(F17="CNY",Compare!$B$9,IF(F17="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I17" s="93">
+        <f>E17</f>
+        <v/>
+      </c>
+      <c r="J17" s="87">
+        <f>Compare!$B$7</f>
+        <v/>
+      </c>
+      <c r="K17" s="88">
+        <f>I17*J17*IF(F17="USD",Compare!$B$8,IF(F17="CNY",Compare!$B$9,IF(F17="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L17" s="90" t="inlineStr">
+        <is>
+          <t>ASSUMPTION ~HK$45 per person each way on the A-route airport buses (about 45–60 min) instead of the HK$115 Airport Express (saves HK$140 pp, ~₮0.26M for 4 people)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1" s="56">
+      <c r="A18" s="94" t="inlineStr">
+        <is>
+          <t>PAID PERSONALLY (university won't cover)</t>
+        </is>
+      </c>
+      <c r="B18" s="95" t="n"/>
+      <c r="C18" s="95" t="n"/>
+      <c r="D18" s="95" t="n"/>
+      <c r="E18" s="95" t="n"/>
+      <c r="F18" s="95" t="n"/>
+      <c r="G18" s="95" t="n"/>
+      <c r="H18" s="95" t="n"/>
+      <c r="I18" s="95" t="n"/>
+      <c r="J18" s="95" t="n"/>
+      <c r="K18" s="95" t="n"/>
+      <c r="L18" s="95" t="n"/>
+    </row>
+    <row r="19" ht="15" customHeight="1" s="56">
+      <c r="A19" s="79" t="inlineStr">
+        <is>
+          <t>Contest fee</t>
+        </is>
+      </c>
+      <c r="B19" s="80" t="n"/>
+      <c r="C19" s="80" t="n"/>
+      <c r="D19" s="80" t="n"/>
+      <c r="E19" s="80" t="n"/>
+      <c r="F19" s="80" t="n"/>
+      <c r="G19" s="80" t="n"/>
+      <c r="H19" s="80" t="n"/>
+      <c r="I19" s="80" t="n"/>
+      <c r="J19" s="80" t="n"/>
+      <c r="K19" s="80" t="n"/>
+      <c r="L19" s="80" t="n"/>
+    </row>
+    <row r="20" ht="22.35" customHeight="1" s="56">
+      <c r="A20" s="81" t="n"/>
+      <c r="B20" s="82" t="inlineStr">
+        <is>
+          <t>Hong Kong regional registration fee (per team)</t>
+        </is>
+      </c>
+      <c r="C20" s="83" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D20" s="81" t="n"/>
+      <c r="E20" s="85" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F20" s="86" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="G20" s="91" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="88">
+        <f>E20*G20*IF(F20="USD",Compare!$B$8,IF(F20="CNY",Compare!$B$9,IF(F20="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I20" s="89">
+        <f>E20</f>
+        <v/>
+      </c>
+      <c r="J20" s="91" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="88">
+        <f>I20*J20*IF(F20="USD",Compare!$B$8,IF(F20="CNY",Compare!$B$9,IF(F20="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L20" s="90" t="inlineStr">
+        <is>
+          <t>1,800 HKD/team at the 2025 Hong Kong regional (HKUST); 2026 host listed as HKU – confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1" s="56">
+      <c r="A21" s="79" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B21" s="80" t="n"/>
+      <c r="C21" s="80" t="n"/>
+      <c r="D21" s="80" t="n"/>
+      <c r="E21" s="80" t="n"/>
+      <c r="F21" s="80" t="n"/>
+      <c r="G21" s="80" t="n"/>
+      <c r="H21" s="80" t="n"/>
+      <c r="I21" s="80" t="n"/>
+      <c r="J21" s="80" t="n"/>
+      <c r="K21" s="80" t="n"/>
+      <c r="L21" s="80" t="n"/>
+    </row>
+    <row r="22" ht="15" customHeight="1" s="56">
+      <c r="A22" s="81" t="n"/>
+      <c r="B22" s="82" t="inlineStr">
+        <is>
+          <t>Taxi to/from Chinggis Khaan airport (UB), per trip</t>
+        </is>
+      </c>
+      <c r="C22" s="83" t="inlineStr">
+        <is>
+          <t>out &amp; back</t>
+        </is>
+      </c>
+      <c r="D22" s="84" t="n">
+        <v>0.04166666666666666</v>
+      </c>
+      <c r="E22" s="92" t="n">
+        <v>100000</v>
+      </c>
+      <c r="F22" s="86" t="inlineStr">
+        <is>
+          <t>MNT</t>
+        </is>
+      </c>
+      <c r="G22" s="91" t="n">
+        <v>2</v>
+      </c>
+      <c r="H22" s="88">
+        <f>E22*G22*IF(F22="USD",Compare!$B$8,IF(F22="CNY",Compare!$B$9,IF(F22="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I22" s="93">
+        <f>E22</f>
+        <v/>
+      </c>
+      <c r="J22" s="91" t="n">
+        <v>2</v>
+      </c>
+      <c r="K22" s="88">
+        <f>I22*J22*IF(F22="USD",Compare!$B$8,IF(F22="CNY",Compare!$B$9,IF(F22="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L22" s="90" t="inlineStr">
+        <is>
+          <t>ASSUMPTION 100k MNT per trip for the group</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1" s="56">
+      <c r="A23" s="81" t="n"/>
+      <c r="B23" s="82" t="inlineStr">
+        <is>
+          <t>Travel medical insurance</t>
+        </is>
+      </c>
+      <c r="C23" s="83" t="n"/>
+      <c r="D23" s="81" t="n"/>
+      <c r="E23" s="92" t="n">
+        <v>30000</v>
+      </c>
+      <c r="F23" s="86" t="inlineStr">
+        <is>
+          <t>MNT</t>
+        </is>
+      </c>
+      <c r="G23" s="87">
+        <f>Compare!$B$6</f>
+        <v/>
+      </c>
+      <c r="H23" s="88">
+        <f>E23*G23*IF(F23="USD",Compare!$B$8,IF(F23="CNY",Compare!$B$9,IF(F23="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I23" s="93">
+        <f>E23</f>
+        <v/>
+      </c>
+      <c r="J23" s="87">
+        <f>Compare!$B$7</f>
+        <v/>
+      </c>
+      <c r="K23" s="88">
+        <f>I23*J23*IF(F23="USD",Compare!$B$8,IF(F23="CNY",Compare!$B$9,IF(F23="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L23" s="90" t="inlineStr">
+        <is>
+          <t>ASSUMPTION ~30k MNT per person, Mongolian insurer</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1" s="56">
+      <c r="A24" s="81" t="n"/>
+      <c r="B24" s="82" t="inlineStr">
+        <is>
+          <t>Mobile data eSIM</t>
+        </is>
+      </c>
+      <c r="C24" s="83" t="n"/>
+      <c r="D24" s="81" t="n"/>
+      <c r="E24" s="92" t="n">
+        <v>10</v>
+      </c>
+      <c r="F24" s="86" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G24" s="87">
+        <f>Compare!$B$6</f>
+        <v/>
+      </c>
+      <c r="H24" s="88">
+        <f>E24*G24*IF(F24="USD",Compare!$B$8,IF(F24="CNY",Compare!$B$9,IF(F24="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I24" s="93">
+        <f>E24</f>
+        <v/>
+      </c>
+      <c r="J24" s="87">
+        <f>Compare!$B$7</f>
+        <v/>
+      </c>
+      <c r="K24" s="88">
+        <f>I24*J24*IF(F24="USD",Compare!$B$8,IF(F24="CNY",Compare!$B$9,IF(F24="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L24" s="90" t="inlineStr">
+        <is>
+          <t>ASSUMPTION ~$10 pp</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22.35" customHeight="1" s="56">
+      <c r="A25" s="81" t="n"/>
+      <c r="B25" s="82" t="inlineStr">
+        <is>
+          <t>Visa</t>
+        </is>
+      </c>
+      <c r="C25" s="83" t="n"/>
+      <c r="D25" s="81" t="n"/>
+      <c r="E25" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="86" t="inlineStr">
+        <is>
+          <t>MNT</t>
+        </is>
+      </c>
+      <c r="G25" s="87">
+        <f>Compare!$B$6</f>
+        <v/>
+      </c>
+      <c r="H25" s="88">
+        <f>E25*G25*IF(F25="USD",Compare!$B$8,IF(F25="CNY",Compare!$B$9,IF(F25="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I25" s="89">
+        <f>E25</f>
+        <v/>
+      </c>
+      <c r="J25" s="87">
+        <f>Compare!$B$7</f>
+        <v/>
+      </c>
+      <c r="K25" s="88">
+        <f>I25*J25*IF(F25="USD",Compare!$B$8,IF(F25="CNY",Compare!$B$9,IF(F25="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L25" s="90" t="inlineStr">
+        <is>
+          <t>Mongolian passports: visa-free (mainland China up to 30 days; Hong Kong up to 14 days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1" s="56">
+      <c r="G27" s="60" t="n"/>
+      <c r="H27" s="96" t="inlineStr">
+        <is>
+          <t>3 people – UNFUNDED</t>
+        </is>
+      </c>
+      <c r="K27" s="96" t="inlineStr">
+        <is>
+          <t>4 people – FUNDED ₮12M</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1" s="56">
+      <c r="G28" s="97" t="inlineStr">
+        <is>
+          <t>University-paid subtotal</t>
+        </is>
+      </c>
+      <c r="H28" s="98">
+        <f>SUM(H9:H17)</f>
+        <v/>
+      </c>
+      <c r="K28" s="98">
+        <f>SUM(K9:K17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1" s="56">
+      <c r="G29" s="99" t="inlineStr">
+        <is>
+          <t>Contingency</t>
+        </is>
+      </c>
+      <c r="H29" s="100">
+        <f>H28*Compare!$B$11</f>
+        <v/>
+      </c>
+      <c r="K29" s="100">
+        <f>K28*Compare!$B$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1" s="56">
+      <c r="G30" s="97" t="inlineStr">
+        <is>
+          <t>University-paid total incl. contingency</t>
+        </is>
+      </c>
+      <c r="H30" s="98">
+        <f>H28+H29</f>
+        <v/>
+      </c>
+      <c r="K30" s="98">
+        <f>K28+K29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="56">
+      <c r="G31" s="97" t="inlineStr">
+        <is>
+          <t>Funding left (negative = over)</t>
+        </is>
+      </c>
+      <c r="H31" s="101">
+        <f>Compare!$B$12-H30</f>
+        <v/>
+      </c>
+      <c r="K31" s="101">
+        <f>Compare!$B$5-K30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1" s="56">
+      <c r="G32" s="97" t="inlineStr">
+        <is>
+          <t>Personal costs – team</t>
+        </is>
+      </c>
+      <c r="H32" s="102">
+        <f>SUM(H19:H25)</f>
+        <v/>
+      </c>
+      <c r="K32" s="102">
+        <f>SUM(K19:K25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1" s="56">
+      <c r="G33" s="97" t="inlineStr">
+        <is>
+          <t>Out-of-pocket per person (personal + any overrun)</t>
+        </is>
+      </c>
+      <c r="H33" s="102">
+        <f>(H32+MAX(0,-H31))/Compare!$B$6</f>
+        <v/>
+      </c>
+      <c r="K33" s="102">
+        <f>(K32+MAX(0,-K31))/Compare!$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="15" customHeight="1" s="56">
+      <c r="G34" s="97" t="inlineStr">
+        <is>
+          <t>Whole trip cost (university + personal)</t>
+        </is>
+      </c>
+      <c r="H34" s="103">
+        <f>H30+H32</f>
+        <v/>
+      </c>
+      <c r="K34" s="103">
+        <f>K30+K32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="15" customHeight="1" s="56">
+      <c r="G35" s="99" t="inlineStr">
+        <is>
+          <t>Time in planes &amp; trains</t>
+        </is>
+      </c>
+      <c r="H35" s="104">
+        <f>SUM(D10:D11)</f>
+        <v/>
+      </c>
+      <c r="K35" s="104">
+        <f>SUM(D10:D11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="15" customHeight="1" s="56">
+      <c r="A37" s="72" t="inlineStr">
+        <is>
+          <t>Key facts</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="15" customHeight="1" s="56">
+      <c r="A38" s="75" t="inlineStr">
+        <is>
+          <t>Contest</t>
+        </is>
+      </c>
+      <c r="B38" s="74" t="inlineStr">
+        <is>
+          <t>Asia Hong Kong Regional, 9–10 Jan 2027 (provisional), host listed as HKU – confirm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="15" customHeight="1" s="56">
+      <c r="A39" s="75" t="inlineStr">
+        <is>
+          <t>Why this plan</t>
+        </is>
+      </c>
+      <c r="B39" s="74" t="inlineStr">
+        <is>
+          <t>Flights are fixed (MIAT nonstop is the cheapest way in). The only room for the ₮12M cap is the hotel and the airport transfer, so this plan uses 2 rooms at a hotel next to HKU and the airport bus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="15" customHeight="1" s="56">
+      <c r="A40" s="75" t="inlineStr">
+        <is>
+          <t>Entry</t>
+        </is>
+      </c>
+      <c r="B40" s="74" t="inlineStr">
+        <is>
+          <t>Mongolian passport holders can visit Hong Kong visa-free for up to 14 days.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="15" customHeight="1" s="56">
+      <c r="A41" s="75" t="inlineStr">
+        <is>
+          <t>Trade-off</t>
+        </is>
+      </c>
+      <c r="B41" s="74" t="inlineStr">
+        <is>
+          <t>Fits ₮12M only before the 10% contingency (about ₮11.7M); with contingency it is ~₮0.9M over. Lock the flights first – they are 70% of the cost. Read noise reviews for the hotel before booking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="15" customHeight="1" s="56">
+      <c r="A43" s="72" t="inlineStr">
+        <is>
+          <t>Day-by-day plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="15" customHeight="1" s="56">
+      <c r="A44" s="96" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B44" s="96" t="inlineStr">
+        <is>
+          <t>Sleep in</t>
+        </is>
+      </c>
+      <c r="C44" s="96" t="inlineStr">
+        <is>
+          <t>What happens</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="15" customHeight="1" s="56">
+      <c r="A45" s="74" t="inlineStr">
+        <is>
+          <t>Fri 8 Jan</t>
+        </is>
+      </c>
+      <c r="B45" s="74" t="inlineStr">
+        <is>
+          <t>Hong Kong</t>
+        </is>
+      </c>
+      <c r="C45" s="74" t="inlineStr">
+        <is>
+          <t>MIAT OM297 UB 06:45 → Hong Kong 11:25 (4 h 40 min). Airport bus, check in at the Sai Ying Pun hotel (nap).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="15" customHeight="1" s="56">
+      <c r="A46" s="74" t="inlineStr">
+        <is>
+          <t>Sat 9 Jan</t>
+        </is>
+      </c>
+      <c r="B46" s="74" t="inlineStr">
+        <is>
+          <t>Hong Kong</t>
+        </is>
+      </c>
+      <c r="C46" s="74" t="inlineStr">
+        <is>
+          <t>Registration, opening and warm-up at the University of Hong Kong (2025 HK regional used the same day-1 pattern).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="15" customHeight="1" s="56">
+      <c r="A47" s="74" t="inlineStr">
+        <is>
+          <t>Sun 10 Jan</t>
+        </is>
+      </c>
+      <c r="B47" s="74" t="inlineStr">
+        <is>
+          <t>Hong Kong</t>
+        </is>
+      </c>
+      <c r="C47" s="74" t="inlineStr">
+        <is>
+          <t>HONG KONG REGIONAL contest day, closing &amp; solutions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="15" customHeight="1" s="56">
+      <c r="A48" s="74" t="inlineStr">
+        <is>
+          <t>Mon 11 Jan</t>
+        </is>
+      </c>
+      <c r="B48" s="74" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="C48" s="74" t="inlineStr">
+        <is>
+          <t>MIAT OM298 Hong Kong 12:25 → UB 17:05.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="15" customHeight="1" s="56">
+      <c r="A50" s="72" t="inlineStr">
+        <is>
+          <t>Door-to-door travel times</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="15" customHeight="1" s="56">
+      <c r="A51" s="96" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B51" s="96" t="inlineStr">
+        <is>
+          <t>Leg</t>
+        </is>
+      </c>
+      <c r="C51" s="96" t="inlineStr">
+        <is>
+          <t>Mode</t>
+        </is>
+      </c>
+      <c r="D51" s="96" t="inlineStr">
+        <is>
+          <t>Expected time</t>
+        </is>
+      </c>
+      <c r="E51" s="96" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="15" customHeight="1" s="56">
+      <c r="A52" s="105" t="inlineStr">
+        <is>
+          <t>8 Jan</t>
+        </is>
+      </c>
+      <c r="B52" s="105" t="inlineStr">
+        <is>
+          <t>Home → Chinggis Khaan airport</t>
+        </is>
+      </c>
+      <c r="C52" s="82" t="inlineStr">
+        <is>
+          <t>Taxi (~50 km)</t>
+        </is>
+      </c>
+      <c r="D52" s="104" t="n">
+        <v>0.04166666666666666</v>
+      </c>
+      <c r="E52" s="106" t="inlineStr">
+        <is>
+          <t>Leave ~03:45 for 06:45 flight</t>
+        </is>
+      </c>
+      <c r="F52" s="107" t="n"/>
+      <c r="G52" s="107" t="n"/>
+      <c r="H52" s="107" t="n"/>
+      <c r="I52" s="107" t="n"/>
+      <c r="J52" s="107" t="n"/>
+      <c r="K52" s="107" t="n"/>
+      <c r="L52" s="107" t="n"/>
+    </row>
+    <row r="53" ht="26.85" customHeight="1" s="56">
+      <c r="A53" s="105" t="inlineStr">
+        <is>
+          <t>8 Jan</t>
+        </is>
+      </c>
+      <c r="B53" s="105" t="inlineStr">
+        <is>
+          <t>Ulaanbaatar → Hong Kong (HKG)</t>
+        </is>
+      </c>
+      <c r="C53" s="82" t="inlineStr">
+        <is>
+          <t>MIAT OM297 06:45–11:25</t>
+        </is>
+      </c>
+      <c r="D53" s="84" t="n">
+        <v>0.1944444444444444</v>
+      </c>
+      <c r="E53" s="106" t="n"/>
+      <c r="F53" s="107" t="n"/>
+      <c r="G53" s="107" t="n"/>
+      <c r="H53" s="107" t="n"/>
+      <c r="I53" s="107" t="n"/>
+      <c r="J53" s="107" t="n"/>
+      <c r="K53" s="107" t="n"/>
+      <c r="L53" s="107" t="n"/>
+    </row>
+    <row r="54" ht="15" customHeight="1" s="56">
+      <c r="A54" s="105" t="inlineStr">
+        <is>
+          <t>8 Jan</t>
+        </is>
+      </c>
+      <c r="B54" s="105" t="inlineStr">
+        <is>
+          <t>HKG arrival: immigration, bags</t>
+        </is>
+      </c>
+      <c r="C54" s="82" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D54" s="104" t="n">
+        <v>0.02777777777777778</v>
+      </c>
+      <c r="E54" s="106" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="F54" s="107" t="n"/>
+      <c r="G54" s="107" t="n"/>
+      <c r="H54" s="107" t="n"/>
+      <c r="I54" s="107" t="n"/>
+      <c r="J54" s="107" t="n"/>
+      <c r="K54" s="107" t="n"/>
+      <c r="L54" s="107" t="n"/>
+    </row>
+    <row r="55" ht="39.55" customHeight="1" s="56">
+      <c r="A55" s="105" t="inlineStr">
+        <is>
+          <t>8 Jan</t>
+        </is>
+      </c>
+      <c r="B55" s="105" t="inlineStr">
+        <is>
+          <t>HKG → Sai Ying Pun hotel</t>
+        </is>
+      </c>
+      <c r="C55" s="82" t="inlineStr">
+        <is>
+          <t>Airport bus to Sheung Wan / Sai Ying Pun + walk</t>
+        </is>
+      </c>
+      <c r="D55" s="104" t="n">
+        <v>0.03472222222222222</v>
+      </c>
+      <c r="E55" s="106" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="F55" s="107" t="n"/>
+      <c r="G55" s="107" t="n"/>
+      <c r="H55" s="107" t="n"/>
+      <c r="I55" s="107" t="n"/>
+      <c r="J55" s="107" t="n"/>
+      <c r="K55" s="107" t="n"/>
+      <c r="L55" s="107" t="n"/>
+    </row>
+    <row r="56" ht="15" customHeight="1" s="56">
+      <c r="A56" s="105" t="inlineStr">
+        <is>
+          <t>9–10 Jan</t>
+        </is>
+      </c>
+      <c r="B56" s="105" t="inlineStr">
+        <is>
+          <t>Hotel ↔ HKU (each way)</t>
+        </is>
+      </c>
+      <c r="C56" s="82" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D56" s="108" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="E56" s="106" t="inlineStr">
+        <is>
+          <t>~10–15 min (walk or 1 MTR stop to HKU station)</t>
+        </is>
+      </c>
+      <c r="F56" s="107" t="n"/>
+      <c r="G56" s="107" t="n"/>
+      <c r="H56" s="107" t="n"/>
+      <c r="I56" s="107" t="n"/>
+      <c r="J56" s="107" t="n"/>
+      <c r="K56" s="107" t="n"/>
+      <c r="L56" s="107" t="n"/>
+    </row>
+    <row r="57" ht="26.85" customHeight="1" s="56">
+      <c r="A57" s="105" t="inlineStr">
+        <is>
+          <t>11 Jan</t>
+        </is>
+      </c>
+      <c r="B57" s="105" t="inlineStr">
+        <is>
+          <t>Hotel → HKG</t>
+        </is>
+      </c>
+      <c r="C57" s="82" t="inlineStr">
+        <is>
+          <t>Walk + airport bus</t>
+        </is>
+      </c>
+      <c r="D57" s="104" t="n">
+        <v>0.03472222222222222</v>
+      </c>
+      <c r="E57" s="106" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="F57" s="107" t="n"/>
+      <c r="G57" s="107" t="n"/>
+      <c r="H57" s="107" t="n"/>
+      <c r="I57" s="107" t="n"/>
+      <c r="J57" s="107" t="n"/>
+      <c r="K57" s="107" t="n"/>
+      <c r="L57" s="107" t="n"/>
+    </row>
+    <row r="58" ht="26.85" customHeight="1" s="56">
+      <c r="A58" s="105" t="inlineStr">
+        <is>
+          <t>11 Jan</t>
+        </is>
+      </c>
+      <c r="B58" s="105" t="inlineStr">
+        <is>
+          <t>Hong Kong (HKG) → Ulaanbaatar</t>
+        </is>
+      </c>
+      <c r="C58" s="82" t="inlineStr">
+        <is>
+          <t>MIAT OM298 12:25–17:05</t>
+        </is>
+      </c>
+      <c r="D58" s="84" t="n">
+        <v>0.1944444444444444</v>
+      </c>
+      <c r="E58" s="106" t="inlineStr">
+        <is>
+          <t>Be at HKG by ~10:25</t>
+        </is>
+      </c>
+      <c r="F58" s="107" t="n"/>
+      <c r="G58" s="107" t="n"/>
+      <c r="H58" s="107" t="n"/>
+      <c r="I58" s="107" t="n"/>
+      <c r="J58" s="107" t="n"/>
+      <c r="K58" s="107" t="n"/>
+      <c r="L58" s="107" t="n"/>
+    </row>
+    <row r="59" ht="14.15" customHeight="1" s="56">
+      <c r="A59" s="105" t="inlineStr">
+        <is>
+          <t>11 Jan</t>
+        </is>
+      </c>
+      <c r="B59" s="105" t="inlineStr">
+        <is>
+          <t>Chinggis Khaan airport → home</t>
+        </is>
+      </c>
+      <c r="C59" s="82" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="D59" s="104" t="n">
+        <v>0.04166666666666666</v>
+      </c>
+      <c r="E59" s="106" t="n"/>
+      <c r="F59" s="107" t="n"/>
+      <c r="G59" s="107" t="n"/>
+      <c r="H59" s="107" t="n"/>
+      <c r="I59" s="107" t="n"/>
+      <c r="J59" s="107" t="n"/>
+      <c r="K59" s="107" t="n"/>
+      <c r="L59" s="107" t="n"/>
+    </row>
+    <row r="60" ht="15" customHeight="1" s="56">
+      <c r="C60" s="59" t="inlineStr">
+        <is>
+          <t>Total door-to-door</t>
+        </is>
+      </c>
+      <c r="D60" s="109">
+        <f>SUM(D52:D59)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="18">
+    <mergeCell ref="E57:L57"/>
+    <mergeCell ref="E56:L56"/>
+    <mergeCell ref="E58:L58"/>
+    <mergeCell ref="C45:L45"/>
+    <mergeCell ref="B38:L38"/>
+    <mergeCell ref="E59:L59"/>
+    <mergeCell ref="E51:L51"/>
+    <mergeCell ref="C48:L48"/>
+    <mergeCell ref="B39:L39"/>
+    <mergeCell ref="E54:L54"/>
+    <mergeCell ref="C44:L44"/>
+    <mergeCell ref="E55:L55"/>
+    <mergeCell ref="E52:L52"/>
+    <mergeCell ref="C46:L46"/>
+    <mergeCell ref="C47:L47"/>
+    <mergeCell ref="E53:L53"/>
+    <mergeCell ref="B41:L41"/>
+    <mergeCell ref="B40:L40"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
   <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
@@ -12594,7 +14015,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -12617,7 +14037,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -13434,7 +14853,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31" ht="15" customHeight="1" s="56">
       <c r="G31" s="60" t="n"/>
       <c r="H31" s="96" t="inlineStr">
@@ -13568,7 +14986,6 @@
         <v/>
       </c>
     </row>
-    <row r="40"/>
     <row r="41" ht="15" customHeight="1" s="56">
       <c r="A41" s="72" t="inlineStr">
         <is>
@@ -13612,7 +15029,6 @@
         </is>
       </c>
     </row>
-    <row r="45"/>
     <row r="46" ht="15" customHeight="1" s="56">
       <c r="A46" s="72" t="inlineStr">
         <is>
@@ -13727,7 +15143,6 @@
       <c r="B53" s="74" t="n"/>
       <c r="C53" s="74" t="n"/>
     </row>
-    <row r="54"/>
     <row r="55" ht="15" customHeight="1" s="56">
       <c r="A55" s="72" t="inlineStr">
         <is>
@@ -14200,7 +15615,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14236,7 +15651,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -14259,7 +15673,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -15027,7 +16440,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30" ht="15" customHeight="1" s="56">
       <c r="G30" s="60" t="n"/>
       <c r="H30" s="96" t="inlineStr">
@@ -15161,7 +16573,6 @@
         <v/>
       </c>
     </row>
-    <row r="39"/>
     <row r="40" ht="15" customHeight="1" s="56">
       <c r="A40" s="72" t="inlineStr">
         <is>
@@ -15205,7 +16616,6 @@
         </is>
       </c>
     </row>
-    <row r="44"/>
     <row r="45" ht="15" customHeight="1" s="56">
       <c r="A45" s="72" t="inlineStr">
         <is>
@@ -15320,7 +16730,6 @@
       <c r="B52" s="74" t="n"/>
       <c r="C52" s="74" t="n"/>
     </row>
-    <row r="53"/>
     <row r="54" ht="15" customHeight="1" s="56">
       <c r="A54" s="72" t="inlineStr">
         <is>
@@ -15792,7 +17201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="56" min="1" max="1"/>
@@ -16452,49 +17861,49 @@
     <row r="19" ht="66" customHeight="1" s="56">
       <c r="A19" s="118" t="inlineStr">
         <is>
-          <t>EC Final – Train</t>
+          <t>Hong Kong – Funded 12M (funded regional)</t>
         </is>
       </c>
       <c r="B19" s="116" t="inlineStr">
         <is>
-          <t>Wed 27 Jan / Tue 26 Jan</t>
+          <t>Sun 10 Jan / Sat 9 Jan</t>
         </is>
       </c>
       <c r="C19" s="116" t="inlineStr">
         <is>
-          <t>24 Jan at home</t>
+          <t>7 Jan at home (04:00 start; arrive 11:50, nap)</t>
         </is>
       </c>
       <c r="D19" s="116" t="inlineStr">
         <is>
-          <t>25 Jan D17 2nd-class sleeper 19:10–09:15 (4-berth cabin, ~6 h) → arrive on day 1</t>
+          <t>8 Jan Best Western Plus, Sai Ying Pun, 2 rooms (2 beds each)</t>
         </is>
       </c>
       <c r="E19" s="116" t="inlineStr">
         <is>
-          <t>26 Jan HanTing, 1.6 km</t>
+          <t>9 Jan same, ~540 m to HKU</t>
         </is>
       </c>
       <c r="F19" s="116" t="inlineStr">
         <is>
-          <t>Walk ~20 min, wake ~07:00</t>
-        </is>
-      </c>
-      <c r="G19" s="120" t="inlineStr">
-        <is>
-          <t>WATCH</t>
+          <t>Walk ~10 min, wake ~07:00</t>
+        </is>
+      </c>
+      <c r="G19" s="121" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="H19" s="116" t="inlineStr">
         <is>
-          <t>The sleeper is the night before the check-in / warm-up day (not the contest day), with a hotel night in between. Safer: leave Beijing 24 Jan (one more hotel night, ~₮0.35M) or take the afternoon G-train + hotel (old plan, ~+₮0.44M).</t>
+          <t>Fits ₮12M only before the 10% contingency (~₮11.7M). Separate beds and no commute; the hotel is rated 7.4–8.2, so read noise reviews. Cheaper alternative with separate beds: Good Fortune Inn (8.6, 4 twin beds) but ~35 min MTR.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="66" customHeight="1" s="56">
       <c r="A20" s="118" t="inlineStr">
         <is>
-          <t>EC Final – Fly</t>
+          <t>EC Final – Train</t>
         </is>
       </c>
       <c r="B20" s="116" t="inlineStr">
@@ -16504,107 +17913,150 @@
       </c>
       <c r="C20" s="116" t="inlineStr">
         <is>
-          <t>24 Jan at home (wake ~03:30 on 25 Jan for Aero Mongolia 06:30)</t>
+          <t>24 Jan at home</t>
         </is>
       </c>
       <c r="D20" s="116" t="inlineStr">
         <is>
-          <t>25 Jan Mehood Theater Hotel (arrive ~13:40; nap)</t>
+          <t>25 Jan D17 2nd-class sleeper 19:10–09:15 (4-berth cabin, ~6 h) → arrive on day 1</t>
         </is>
       </c>
       <c r="E20" s="116" t="inlineStr">
         <is>
-          <t>26 Jan same, 1.7 km</t>
+          <t>26 Jan HanTing, 1.6 km</t>
         </is>
       </c>
       <c r="F20" s="116" t="inlineStr">
         <is>
-          <t>Walk ~20 min</t>
-        </is>
-      </c>
-      <c r="G20" s="121" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>Walk ~20 min, wake ~07:00</t>
+        </is>
+      </c>
+      <c r="G20" s="120" t="inlineStr">
+        <is>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="H20" s="116" t="inlineStr">
         <is>
-          <t>Early start two nights before; arrives early afternoon, then two hotel nights.</t>
+          <t>The sleeper is the night before the check-in / warm-up day (not the contest day), with a hotel night in between. Safer: leave Beijing 24 Jan (one more hotel night, ~₮0.35M) or take the afternoon G-train + hotel (old plan, ~+₮0.44M).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="66" customHeight="1" s="56">
       <c r="A21" s="118" t="inlineStr">
         <is>
+          <t>EC Final – Fly</t>
+        </is>
+      </c>
+      <c r="B21" s="116" t="inlineStr">
+        <is>
+          <t>Wed 27 Jan / Tue 26 Jan</t>
+        </is>
+      </c>
+      <c r="C21" s="116" t="inlineStr">
+        <is>
+          <t>24 Jan at home (wake ~03:30 on 25 Jan for Aero Mongolia 06:30)</t>
+        </is>
+      </c>
+      <c r="D21" s="116" t="inlineStr">
+        <is>
+          <t>25 Jan Mehood Theater Hotel (arrive ~13:40; nap)</t>
+        </is>
+      </c>
+      <c r="E21" s="116" t="inlineStr">
+        <is>
+          <t>26 Jan same, 1.7 km</t>
+        </is>
+      </c>
+      <c r="F21" s="116" t="inlineStr">
+        <is>
+          <t>Walk ~20 min</t>
+        </is>
+      </c>
+      <c r="G21" s="121" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H21" s="116" t="inlineStr">
+        <is>
+          <t>Early start two nights before; arrives early afternoon, then two hotel nights.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="66" customHeight="1" s="56">
+      <c r="A22" s="118" t="inlineStr">
+        <is>
           <t>Nanjing + Shenyang (older workbook A / B)</t>
         </is>
       </c>
-      <c r="B21" s="116" t="inlineStr">
+      <c r="B22" s="116" t="inlineStr">
         <is>
           <t>Nanjing Sun 8 Nov; Shenyang Sun 15 Nov</t>
         </is>
       </c>
-      <c r="C21" s="116" t="inlineStr">
+      <c r="C22" s="116" t="inlineStr">
         <is>
           <t>6 Nov Beijing hotel after MIAT lands 19:30, wake ~06:00 for the G-train</t>
         </is>
       </c>
-      <c r="D21" s="116" t="inlineStr">
+      <c r="D22" s="116" t="inlineStr">
         <is>
           <t>7 Nov Nanjing hotel (A 1 km, B 15 min metro)</t>
         </is>
       </c>
-      <c r="E21" s="116" t="inlineStr">
+      <c r="E22" s="116" t="inlineStr">
         <is>
           <t>Shenyang: Z366 sleeper 12 Nov → hotels 13 and 14 Nov</t>
         </is>
       </c>
-      <c r="F21" s="116" t="inlineStr">
+      <c r="F22" s="116" t="inlineStr">
         <is>
           <t>Nanjing walk / Shenyang walk</t>
         </is>
       </c>
-      <c r="G21" s="121" t="inlineStr">
+      <c r="G22" s="121" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="H21" s="116" t="inlineStr">
+      <c r="H22" s="116" t="inlineStr">
         <is>
           <t>K54 home after the Shenyang contest is now a hard sleeper (soft was ¥263). Plan C (home between) uses K53 soft sleeper on 13 Nov = night before day 1 (WATCH).</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="122" t="inlineStr">
+    <row r="23" s="56"/>
+    <row r="24" s="56">
+      <c r="A24" s="122" t="inlineStr">
         <is>
           <t>Where the money goes (use the headroom on sleep)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="36" customHeight="1" s="56">
-      <c r="A24" s="116" t="inlineStr">
-        <is>
-          <t>One regional is funded with ₮12M (coach travels, 4 people); the other is unfunded (3 contestants pay). The funded trip has little headroom (Hong Kong does not fit), and the unfunded trip pays for every hotel night, so protect sleep with timing and location first: arrive a day early only where it is cheap (Shenyang, Nanchang), pick the hotel closest to the venue, and take the cheap-but-bad options only after the contest.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="36" customHeight="1" s="56">
       <c r="A25" s="116" t="inlineStr">
         <is>
-          <t>Pre-contest upgrades applied: Shenyang Budget K53 hard → soft; Hong Kong Sleep first (2 rooms near HKU). Post-contest downgrades applied: Shenyang K54 soft → hard, Shanghai D8 sleeper → seat, Nanchang D136 sleeper → seat.</t>
+          <t>One regional is funded with ₮12M (coach travels, 4 people); the other is unfunded (3 contestants pay). The funded trip has little headroom (Hong Kong does not fit), and the unfunded trip pays for every hotel night, so protect sleep with timing and location first: arrive a day early only where it is cheap (Shenyang, Nanchang), pick the hotel closest to the venue, and take the cheap-but-bad options only after the contest.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="36" customHeight="1" s="56">
       <c r="A26" s="116" t="inlineStr">
         <is>
-          <t>Cheapest post-contest options if you want to go further: Nanchang Z182 20:01 → 08:46 hard seat (¥173.5 vs ¥271); Shanghai G808 17:25 is too early after the awards, so the D8 seat stays.</t>
+          <t>Pre-contest upgrades applied: Shenyang Budget K53 hard → soft; Hong Kong Sleep first (2 rooms near HKU). Post-contest downgrades applied: Shenyang K54 soft → hard, Shanghai D8 sleeper → seat, Nanchang D136 sleeper → seat.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="36" customHeight="1" s="56">
       <c r="A27" s="116" t="inlineStr">
+        <is>
+          <t>Cheapest post-contest options if you want to go further: Nanchang Z182 20:01 → 08:46 hard seat (¥173.5 vs ¥271); Shanghai G808 17:25 is too early after the awards, so the D8 seat stays.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="36" customHeight="1" s="56">
+      <c r="A28" s="116" t="inlineStr">
         <is>
           <t>Contest-day wake-up rule of thumb: bed by 22:30–23:00, up by 06:00–06:30 for a 09:00 start; avoid alcohol and late team dinners; no phone-based all-nighters on day 1.</t>
         </is>
@@ -16614,8 +18066,8 @@
   <mergeCells count="5">
     <mergeCell ref="A26:H26"/>
     <mergeCell ref="A25:H25"/>
-    <mergeCell ref="A24:H24"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A28:H28"/>
     <mergeCell ref="A27:H27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16658,7 +18110,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -16681,7 +18132,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -17471,7 +18921,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31" ht="15" customHeight="1" s="56">
       <c r="G31" s="60" t="n"/>
       <c r="H31" s="96" t="inlineStr">
@@ -17605,7 +19054,6 @@
         <v/>
       </c>
     </row>
-    <row r="40"/>
     <row r="41" ht="15" customHeight="1" s="56">
       <c r="A41" s="72" t="inlineStr">
         <is>
@@ -17649,7 +19097,6 @@
         </is>
       </c>
     </row>
-    <row r="45"/>
     <row r="46" ht="15" customHeight="1" s="56">
       <c r="A46" s="72" t="inlineStr">
         <is>
@@ -17742,7 +19189,6 @@
         </is>
       </c>
     </row>
-    <row r="52"/>
     <row r="53" ht="15" customHeight="1" s="56">
       <c r="A53" s="72" t="inlineStr">
         <is>
@@ -18258,7 +19704,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -18281,7 +19726,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -19057,7 +20501,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30" ht="15" customHeight="1" s="56">
       <c r="G30" s="60" t="n"/>
       <c r="H30" s="96" t="inlineStr">
@@ -19191,7 +20634,6 @@
         <v/>
       </c>
     </row>
-    <row r="39"/>
     <row r="40" ht="15" customHeight="1" s="56">
       <c r="A40" s="72" t="inlineStr">
         <is>
@@ -19235,7 +20677,6 @@
         </is>
       </c>
     </row>
-    <row r="44"/>
     <row r="45" ht="15" customHeight="1" s="56">
       <c r="A45" s="72" t="inlineStr">
         <is>
@@ -19345,7 +20786,6 @@
         </is>
       </c>
     </row>
-    <row r="52"/>
     <row r="53" ht="15" customHeight="1" s="56">
       <c r="A53" s="72" t="inlineStr">
         <is>
@@ -19839,7 +21279,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -19862,7 +21301,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -20758,7 +22196,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32" ht="15" customHeight="1" s="56">
       <c r="G32" s="60" t="n"/>
       <c r="H32" s="96" t="inlineStr">
@@ -20892,7 +22329,6 @@
         <v/>
       </c>
     </row>
-    <row r="41"/>
     <row r="42" ht="15" customHeight="1" s="56">
       <c r="A42" s="72" t="inlineStr">
         <is>
@@ -20936,7 +22372,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47" ht="15" customHeight="1" s="56">
       <c r="A47" s="72" t="inlineStr">
         <is>
@@ -21029,7 +22464,6 @@
         </is>
       </c>
     </row>
-    <row r="53"/>
     <row r="54" ht="15" customHeight="1" s="56">
       <c r="A54" s="72" t="inlineStr">
         <is>
@@ -21458,7 +22892,6 @@
       <c r="K68" s="107" t="n"/>
       <c r="L68" s="107" t="n"/>
     </row>
-    <row r="69"/>
     <row r="70" ht="15" customHeight="1" s="56">
       <c r="C70" s="59" t="inlineStr">
         <is>
@@ -21533,7 +22966,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -21556,7 +22988,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -22452,7 +23883,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32" ht="15" customHeight="1" s="56">
       <c r="G32" s="60" t="n"/>
       <c r="H32" s="96" t="inlineStr">
@@ -22586,7 +24016,6 @@
         <v/>
       </c>
     </row>
-    <row r="41"/>
     <row r="42" ht="15" customHeight="1" s="56">
       <c r="A42" s="72" t="inlineStr">
         <is>
@@ -22630,7 +24059,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47" ht="15" customHeight="1" s="56">
       <c r="A47" s="72" t="inlineStr">
         <is>
@@ -22740,7 +24168,6 @@
         </is>
       </c>
     </row>
-    <row r="54"/>
     <row r="55" ht="15" customHeight="1" s="56">
       <c r="A55" s="72" t="inlineStr">
         <is>
@@ -23169,7 +24596,6 @@
       <c r="K69" s="107" t="n"/>
       <c r="L69" s="107" t="n"/>
     </row>
-    <row r="70"/>
     <row r="71" ht="15" customHeight="1" s="56">
       <c r="C71" s="59" t="inlineStr">
         <is>
@@ -23245,7 +24671,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -23268,7 +24693,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -24165,7 +25589,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32" ht="15" customHeight="1" s="56">
       <c r="G32" s="60" t="n"/>
       <c r="H32" s="96" t="inlineStr">
@@ -24299,7 +25722,6 @@
         <v/>
       </c>
     </row>
-    <row r="41"/>
     <row r="42" ht="15" customHeight="1" s="56">
       <c r="A42" s="72" t="inlineStr">
         <is>
@@ -24355,7 +25777,6 @@
         </is>
       </c>
     </row>
-    <row r="47"/>
     <row r="48" ht="15" customHeight="1" s="56">
       <c r="A48" s="72" t="inlineStr">
         <is>
@@ -24465,7 +25886,6 @@
         </is>
       </c>
     </row>
-    <row r="55"/>
     <row r="56" ht="15" customHeight="1" s="56">
       <c r="A56" s="72" t="inlineStr">
         <is>
@@ -24870,7 +26290,6 @@
       <c r="K69" s="107" t="n"/>
       <c r="L69" s="107" t="n"/>
     </row>
-    <row r="70"/>
     <row r="71" ht="15" customHeight="1" s="56">
       <c r="C71" s="59" t="inlineStr">
         <is>
@@ -24946,7 +26365,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -24969,7 +26387,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -25707,7 +27124,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
     <row r="28" ht="15" customHeight="1" s="56">
       <c r="G28" s="60" t="n"/>
       <c r="H28" s="96" t="inlineStr">
@@ -25841,7 +27257,6 @@
         <v/>
       </c>
     </row>
-    <row r="37"/>
     <row r="38" ht="15" customHeight="1" s="56">
       <c r="A38" s="72" t="inlineStr">
         <is>
@@ -25897,7 +27312,6 @@
         </is>
       </c>
     </row>
-    <row r="43"/>
     <row r="44" ht="15" customHeight="1" s="56">
       <c r="A44" s="72" t="inlineStr">
         <is>
@@ -26024,7 +27438,6 @@
         </is>
       </c>
     </row>
-    <row r="52"/>
     <row r="53" ht="15" customHeight="1" s="56">
       <c r="A53" s="72" t="inlineStr">
         <is>
@@ -26337,7 +27750,6 @@
       <c r="K63" s="107" t="n"/>
       <c r="L63" s="107" t="n"/>
     </row>
-    <row r="64"/>
     <row r="65" ht="15" customHeight="1" s="56">
       <c r="C65" s="59" t="inlineStr">
         <is>
@@ -26411,7 +27823,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="56">
       <c r="A4" s="60" t="inlineStr">
         <is>
@@ -26434,7 +27845,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="31.5" customHeight="1" s="56">
       <c r="A7" s="66" t="inlineStr">
         <is>
@@ -27420,7 +28830,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
     <row r="34" ht="15" customHeight="1" s="56">
       <c r="G34" s="60" t="n"/>
       <c r="H34" s="96" t="inlineStr">
@@ -27554,7 +28963,6 @@
         <v/>
       </c>
     </row>
-    <row r="43"/>
     <row r="44" ht="15" customHeight="1" s="56">
       <c r="A44" s="72" t="inlineStr">
         <is>
@@ -27610,7 +29018,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
     <row r="50" ht="15" customHeight="1" s="56">
       <c r="A50" s="72" t="inlineStr">
         <is>
@@ -27720,7 +29127,6 @@
         </is>
       </c>
     </row>
-    <row r="57"/>
     <row r="58" ht="15" customHeight="1" s="56">
       <c r="A58" s="72" t="inlineStr">
         <is>
@@ -28153,7 +29559,6 @@
       <c r="K72" s="107" t="n"/>
       <c r="L72" s="107" t="n"/>
     </row>
-    <row r="73"/>
     <row r="74" ht="15" customHeight="1" s="56">
       <c r="C74" s="59" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Hong Kong: sleep-priority hotel (4 twin beds) under the 12M cap
- New Hong Kong - Sleep priority sheet: Good Fortune Inn, 2 rooms, A21 airport bus
- Compare row and picks, Sleep check row; details.md hotel findings

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ICPC_Single_Contest_Plans.xlsx
+++ b/ICPC_Single_Contest_Plans.xlsx
@@ -24,8 +24,9 @@
     <sheet name="Hong Kong – Value" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="Hong Kong – Sleep first" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="Hong Kong – Funded 12M" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="EC Final Hangzhou – Train" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="EC Final Hangzhou – Fly" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Hong Kong – Sleep priority" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="EC Final Hangzhou – Train" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="EC Final Hangzhou – Fly" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -894,7 +895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:M47"/>
+  <dimension ref="A1:M49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="55" min="1" max="1"/>
@@ -1943,50 +1944,50 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="30" customHeight="1" s="56">
+    <row r="30" s="56">
       <c r="A30" s="67" t="inlineStr">
         <is>
-          <t>EC Final Hangzhou – Train</t>
+          <t>Hong Kong – Sleep priority</t>
         </is>
       </c>
       <c r="B30" s="68">
-        <f>'EC Final Hangzhou – Train'!H34</f>
+        <f>'Hong Kong – Sleep priority'!H30</f>
         <v/>
       </c>
       <c r="C30" s="68">
-        <f>'EC Final Hangzhou – Train'!H35</f>
+        <f>'Hong Kong – Sleep priority'!H31</f>
         <v/>
       </c>
       <c r="D30" s="69">
-        <f>'EC Final Hangzhou – Train'!H37</f>
+        <f>'Hong Kong – Sleep priority'!H33</f>
         <v/>
       </c>
       <c r="E30" s="68">
-        <f>'EC Final Hangzhou – Train'!K34</f>
+        <f>'Hong Kong – Sleep priority'!K30</f>
         <v/>
       </c>
       <c r="F30" s="68">
-        <f>'EC Final Hangzhou – Train'!K35</f>
+        <f>'Hong Kong – Sleep priority'!K31</f>
         <v/>
       </c>
       <c r="G30" s="69">
-        <f>'EC Final Hangzhou – Train'!K37</f>
+        <f>'Hong Kong – Sleep priority'!K33</f>
         <v/>
       </c>
       <c r="H30" s="70">
-        <f>'EC Final Hangzhou – Train'!H38</f>
+        <f>'Hong Kong – Sleep priority'!H34</f>
         <v/>
       </c>
       <c r="I30" s="70">
-        <f>'EC Final Hangzhou – Train'!K38</f>
+        <f>'Hong Kong – Sleep priority'!K34</f>
         <v/>
       </c>
       <c r="J30" s="71">
-        <f>'EC Final Hangzhou – Train'!H39</f>
+        <f>'Hong Kong – Sleep priority'!H35</f>
         <v/>
       </c>
       <c r="K30" s="71">
-        <f>'EC Final Hangzhou – Train'!D70</f>
+        <f>'Hong Kong – Sleep priority'!D60</f>
         <v/>
       </c>
       <c r="L30" s="123">
@@ -2001,226 +2002,282 @@
     <row r="31" ht="30" customHeight="1" s="56">
       <c r="A31" s="67" t="inlineStr">
         <is>
+          <t>EC Final Hangzhou – Train</t>
+        </is>
+      </c>
+      <c r="B31" s="68">
+        <f>'EC Final Hangzhou – Train'!H34</f>
+        <v/>
+      </c>
+      <c r="C31" s="68">
+        <f>'EC Final Hangzhou – Train'!H35</f>
+        <v/>
+      </c>
+      <c r="D31" s="69">
+        <f>'EC Final Hangzhou – Train'!H37</f>
+        <v/>
+      </c>
+      <c r="E31" s="68">
+        <f>'EC Final Hangzhou – Train'!K34</f>
+        <v/>
+      </c>
+      <c r="F31" s="68">
+        <f>'EC Final Hangzhou – Train'!K35</f>
+        <v/>
+      </c>
+      <c r="G31" s="69">
+        <f>'EC Final Hangzhou – Train'!K37</f>
+        <v/>
+      </c>
+      <c r="H31" s="70">
+        <f>'EC Final Hangzhou – Train'!H38</f>
+        <v/>
+      </c>
+      <c r="I31" s="70">
+        <f>'EC Final Hangzhou – Train'!K38</f>
+        <v/>
+      </c>
+      <c r="J31" s="71">
+        <f>'EC Final Hangzhou – Train'!H39</f>
+        <v/>
+      </c>
+      <c r="K31" s="71">
+        <f>'EC Final Hangzhou – Train'!D70</f>
+        <v/>
+      </c>
+      <c r="L31" s="123">
+        <f>IF(F30&gt;=0,"yes","over by "&amp;TEXT(-F30,"#,##0")&amp;" ₮")</f>
+        <v/>
+      </c>
+      <c r="M31" s="68">
+        <f>Compare!$B$5-E30/(1+Compare!$B$11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1" s="56">
+      <c r="A32" s="67" t="inlineStr">
+        <is>
           <t>EC Final Hangzhou – Fly</t>
         </is>
       </c>
-      <c r="B31" s="68">
+      <c r="B32" s="68">
         <f>'EC Final Hangzhou – Fly'!H33</f>
         <v/>
       </c>
-      <c r="C31" s="68">
+      <c r="C32" s="68">
         <f>'EC Final Hangzhou – Fly'!H34</f>
         <v/>
       </c>
-      <c r="D31" s="69">
+      <c r="D32" s="69">
         <f>'EC Final Hangzhou – Fly'!H36</f>
         <v/>
       </c>
-      <c r="E31" s="68">
+      <c r="E32" s="68">
         <f>'EC Final Hangzhou – Fly'!K33</f>
         <v/>
       </c>
-      <c r="F31" s="68">
+      <c r="F32" s="68">
         <f>'EC Final Hangzhou – Fly'!K34</f>
         <v/>
       </c>
-      <c r="G31" s="69">
+      <c r="G32" s="69">
         <f>'EC Final Hangzhou – Fly'!K36</f>
         <v/>
       </c>
-      <c r="H31" s="70">
+      <c r="H32" s="70">
         <f>'EC Final Hangzhou – Fly'!H37</f>
         <v/>
       </c>
-      <c r="I31" s="70">
+      <c r="I32" s="70">
         <f>'EC Final Hangzhou – Fly'!K37</f>
         <v/>
       </c>
-      <c r="J31" s="71">
+      <c r="J32" s="71">
         <f>'EC Final Hangzhou – Fly'!H38</f>
         <v/>
       </c>
-      <c r="K31" s="71">
+      <c r="K32" s="71">
         <f>'EC Final Hangzhou – Fly'!D70</f>
         <v/>
       </c>
-      <c r="L31" s="123">
+      <c r="L32" s="123">
         <f>IF(F31&gt;=0,"yes","over by "&amp;TEXT(-F31,"#,##0")&amp;" ₮")</f>
         <v/>
       </c>
-      <c r="M31" s="68">
+      <c r="M32" s="68">
         <f>Compare!$B$5-E31/(1+Compare!$B$11)</f>
         <v/>
       </c>
     </row>
-    <row r="32" ht="30" customHeight="1" s="56">
-      <c r="A32" s="75" t="n"/>
-      <c r="B32" s="74" t="n"/>
-    </row>
-    <row r="33" ht="15" customHeight="1" s="56">
-      <c r="A33" s="72" t="inlineStr">
+    <row r="33" ht="30" customHeight="1" s="56">
+      <c r="A33" s="75" t="n"/>
+      <c r="B33" s="74" t="n"/>
+    </row>
+    <row r="34" ht="15" customHeight="1" s="56">
+      <c r="A34" s="72" t="inlineStr">
         <is>
           <t>Recommended picks (not the expensive ones)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="62" customHeight="1" s="56">
-      <c r="A34" s="73" t="inlineStr">
-        <is>
-          <t>Likely pairing (your answer)</t>
-        </is>
-      </c>
-      <c r="B34" s="74" t="inlineStr">
-        <is>
-          <t>Funded = Hong Kong (₮12M, coach): 'Hong Kong – Funded 12M' (MIAT nonstop, 2 rooms ~540 m from HKU, airport bus) costs ₮11.70M before the 10% contingency (₮0.30M spare) and ₮12.87M with it – lock the flights first. Unfunded = Shenyang: Budget ₮2.14M per person (≈ $594; flights are 58% of it), Comfort ₮2.46M per person. The two together are the cheapest sleep-safe pairing; Shanghai or Nanchang as the unfunded one would cost ₮2.50M per person / ₮2.89M per person.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="62" customHeight="1" s="56">
       <c r="A35" s="73" t="inlineStr">
         <is>
-          <t>Unfunded regional (3 ppl pay)</t>
+          <t>Likely pairing (your answer)</t>
         </is>
       </c>
       <c r="B35" s="74" t="inlineStr">
         <is>
-          <t>Cheapest sleep-safe plans per person incl. fee, taxi, insurance, eSIM and 10% contingency: Shenyang – Budget ₮2.14M per person (soft sleeper before day 1); Shenyang – Comfort ₮2.46M per person; Nanchang – Sleeper ₮2.50M per person; Shanghai – Sleeper ₮2.89M per person; Hong Kong – Budget ₮3.43M per person; EC Final – Train ₮3.14M per person. Shenyang and Nanchang are the cheap ones to pay yourselves.</t>
+          <t>Funded = Hong Kong (₮12M, coach): lead with 'Hong Kong – Sleep priority' – MIAT nonstop, 2 rooms with 4 separate twin beds and private bathrooms at Good Fortune Inn (8.6, 715 reviews, ~35–40 min MTR to HKU), airport bus: ₮11.33M before the 10% contingency (₮0.67M spare), ₮12.47M with it. Walking alternative: 'Funded 12M' (Best Western Plus, ~540 m to HKU) ₮11.70M before contingency (₮0.30M spare). Unfunded = Shenyang: Budget ₮2.14M per person (≈ $594; flights are 58% of it), Comfort ₮2.46M per person. The HK 2026 host may not be HKU (2025 was HKUST), which favours sleeping well and staying on the MTR over a hotel next to one campus.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="62" customHeight="1" s="56">
       <c r="A36" s="73" t="inlineStr">
         <is>
+          <t>Unfunded regional (3 ppl pay)</t>
+        </is>
+      </c>
+      <c r="B36" s="74" t="inlineStr">
+        <is>
+          <t>Cheapest sleep-safe plans per person incl. fee, taxi, insurance, eSIM and 10% contingency: Shenyang – Budget ₮2.14M per person (soft sleeper before day 1); Shenyang – Comfort ₮2.46M per person; Nanchang – Sleeper ₮2.50M per person; Shanghai – Sleeper ₮2.89M per person; Hong Kong – Budget ₮3.43M per person; EC Final – Train ₮3.14M per person. Shenyang and Nanchang are the cheap ones to pay yourselves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="62" customHeight="1" s="56">
+      <c r="A37" s="73" t="inlineStr">
+        <is>
           <t>Funded regional (₮12M, coach)</t>
         </is>
       </c>
-      <c r="B36" s="74" t="inlineStr">
-        <is>
-          <t>Fits ₮12M incl. contingency: Shenyang – Comfort ₮8.04M (fits, ₮3.96M left); Shanghai – Sleeper ₮9.83M (fits, ₮2.17M left); Nanchang – Sleeper ₮8.19M (fits, ₮3.81M left); EC Final – Train ₮11.12M (fits, ₮0.88M left). Hong Kong only fits before the 10% contingency (the flights are ₮8.4M of it): Budget ₮11.02M, Value ₮11.26M, Funded 12M ₮11.70M, Comfort ₮11.96M; Sleep first ₮13.14M and EC Final – Fly do not fit at all. Use the funded trip for the dearest contest you must attend and pay the cheap one yourselves.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="47" customHeight="1" s="56">
-      <c r="A37" s="73" t="inlineStr">
-        <is>
-          <t>Regional – Shenyang (14–15 Nov)</t>
-        </is>
-      </c>
       <c r="B37" s="74" t="inlineStr">
         <is>
-          <t>Comfort: rest day, RiCH family room 1.3 km from NEU, hard sleeper home after the contest. No sleepers at all: G-train Comfort ₮6.72M / ₮8.84M, G-train Budget ₮6.05M / ₮8.27M (3 / 4 ppl). Fly home on Air China 12:55 ($171).</t>
+          <t>Fits ₮12M incl. contingency: Shenyang – Comfort ₮8.04M (fits, ₮3.96M left); Shanghai – Sleeper ₮9.83M (fits, ₮2.17M left); Nanchang – Sleeper ₮8.19M (fits, ₮3.81M left); EC Final – Train ₮11.12M (fits, ₮0.88M left). Hong Kong only fits before the 10% contingency (the flights are ₮8.4M of it): Budget ₮11.02M, Value ₮11.26M, Sleep priority ₮11.33M, Funded 12M ₮11.70M, Comfort ₮11.96M; Sleep first ₮13.14M and EC Final – Fly do not fit at all. Use the funded trip for the dearest contest you must attend and pay the cheap one yourselves.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="47" customHeight="1" s="56">
       <c r="A38" s="73" t="inlineStr">
         <is>
-          <t>Regional – Shanghai (5–6 Dec)</t>
+          <t>Regional – Shenyang (14–15 Nov)</t>
         </is>
       </c>
       <c r="B38" s="74" t="inlineStr">
         <is>
-          <t>Sleeper: MIAT $151 + G17 out on 3 Dec, Jenny's Apartment 3 nights (1 km), D8 overnight seat back, Air China 12:55 $172 on 7 Dec. Spring nonstop (Tue 1 → Tue 8 Dec, 7 nights) ₮8.21M / ₮10.73M; day train home with a Beijing night ₮8.11M / ₮10.78M. Wildcard: email shu_icpc@163.com now.</t>
+          <t>Comfort: rest day, RiCH family room 1.3 km from NEU, hard sleeper home after the contest. No sleepers at all: G-train Comfort ₮6.72M / ₮8.84M, G-train Budget ₮6.05M / ₮8.27M (3 / 4 ppl). Fly home on Air China 12:55 ($171).</t>
         </is>
       </c>
     </row>
     <row r="39" ht="47" customHeight="1" s="56">
       <c r="A39" s="73" t="inlineStr">
         <is>
-          <t>Regional – Nanchang (19–20 Dec)</t>
+          <t>Regional – Shanghai (5–6 Dec)</t>
         </is>
       </c>
       <c r="B39" s="74" t="inlineStr">
         <is>
-          <t>Sleeper: Air China $157 + Z111 hard sleeper (arrive 11:52 on 18 Dec), Orange Hotel 2 nights, D136 seat back, Air China 12:55 $172. Comfort (daytime G-train, 3 hotel nights) ₮7.96M / ₮10.32M; Fly in (Air China through ticket $356) ₮8.41M / ₮10.95M.</t>
+          <t>Sleeper: MIAT $151 + G17 out on 3 Dec, Jenny's Apartment 3 nights (1 km), D8 overnight seat back, Air China 12:55 $172 on 7 Dec. Spring nonstop (Tue 1 → Tue 8 Dec, 7 nights) ₮8.21M / ₮10.73M; day train home with a Beijing night ₮8.11M / ₮10.78M. Wildcard: email shu_icpc@163.com now.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="47" customHeight="1" s="56">
       <c r="A40" s="73" t="inlineStr">
         <is>
+          <t>Regional – Nanchang (19–20 Dec)</t>
+        </is>
+      </c>
+      <c r="B40" s="74" t="inlineStr">
+        <is>
+          <t>Sleeper: Air China $157 + Z111 hard sleeper (arrive 11:52 on 18 Dec), Orange Hotel 2 nights, D136 seat back, Air China 12:55 $172. Comfort (daytime G-train, 3 hotel nights) ₮7.96M / ₮10.32M; Fly in (Air China through ticket $356) ₮8.41M / ₮10.95M.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="62" customHeight="1" s="56">
+      <c r="A41" s="73" t="inlineStr">
+        <is>
           <t>Regional – Hong Kong (9–10 Jan)</t>
         </is>
       </c>
-      <c r="B40" s="74" t="inlineStr">
-        <is>
-          <t>MIAT nonstop ($586 return on Trip.com, low against the usual $708–900) is the cheapest way in. Budget guesthouse ₮9.08M / ₮12.12M; Value (Kusa Inn 9.6) ₮9.08M / ₮12.38M; Sleep first (2 rooms near HKU) ₮11.63M / ₮14.45M. No route or date is cheaper (checked 10 Oct).</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="47" customHeight="1" s="56">
-      <c r="A41" s="73" t="inlineStr">
+      <c r="B41" s="74" t="inlineStr">
+        <is>
+          <t>MIAT nonstop ($586 return on Trip.com, low against the usual $708–900) is the cheapest way in; flights are ₮8.4M of the 4-person cost. With sleep prioritised over distance: Sleep priority (Good Fortune Inn, 4 twin beds, ~35–40 min MTR) ₮9.14M / ₮12.47M, Funded 12M (BW Plus, 2 rooms, walk to HKU) ₮9.35M / ₮12.87M, Budget guesthouse ₮9.08M / ₮12.12M, Value (Kusa Inn 9.6) ₮9.08M / ₮12.38M, Sleep first (2 rooms in Sheung Wan) ₮11.63M / ₮14.45M (3 / 4 ppl). No route or date is cheaper (checked 10 Oct).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="47" customHeight="1" s="56">
+      <c r="A42" s="73" t="inlineStr">
         <is>
           <t>EC Final (only if qualified)</t>
         </is>
       </c>
-      <c r="B41" s="74" t="inlineStr">
+      <c r="B42" s="74" t="inlineStr">
         <is>
           <t>Train: MIAT to Beijing, D17 overnight sleeper Beijing 19:10 → Hangzhou 09:15 (¥491), Air China through ticket Hangzhou → UB on 29 Jan: ₮11.12M (fits, ₮0.88M left) for 4 ppl, ₮3.14M per person for 3. Fly (Aero Mongolia + Xiamen via Hohhot) is ₮14.82M (over by ₮2.82M) – does not fit ₮12M. Buy D17 on 12306 at 10:00 on 11 Jan.</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="32" customHeight="1" s="56"/>
-    <row r="43" ht="32" customHeight="1" s="56">
-      <c r="A43" s="75" t="inlineStr">
+    <row r="43" ht="32" customHeight="1" s="56"/>
+    <row r="44" ht="32" customHeight="1" s="56">
+      <c r="A44" s="75" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B43" s="74" t="inlineStr">
+      <c r="B44" s="74" t="inlineStr">
         <is>
           <t>Dates are provisional (ICPC Beijing HQ summary, 5 Aug 2026). Hong Kong host (HKU) and EC Final venue (HZNU Cangqian) are from secondary sources; Shanghai (Shanghai University Baoshan) follows the 2025 invitation and Nanchang (Jiangxi Normal University Yaohu campus) the 2019 handbook – confirm each invitation.</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="18" customHeight="1" s="56">
-      <c r="A44" s="75" t="inlineStr">
+    <row r="45" ht="18" customHeight="1" s="56">
+      <c r="A45" s="75" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B44" s="74" t="inlineStr">
+      <c r="B45" s="74" t="inlineStr">
         <is>
           <t>EC Final is qualification-only: plan it only once the team has earned a slot at a regional.</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="32" customHeight="1" s="56">
-      <c r="A45" s="75" t="inlineStr">
+    <row r="46" ht="32" customHeight="1" s="56">
+      <c r="A46" s="75" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B45" s="74" t="inlineStr">
+      <c r="B46" s="74" t="inlineStr">
         <is>
           <t>4-person plans use whatever split is cheapest on Trip.com/Booking.com: one family room for 4 (Shenyang RiCH, Nanchang Orange Hotel), or two rooms. Taxi costs assume one car; with luggage 4 people may need an XL car.</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="47" customHeight="1" s="56">
-      <c r="A46" s="75" t="inlineStr">
+    <row r="47" ht="47" customHeight="1" s="56">
+      <c r="A47" s="75" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B46" s="74" t="inlineStr">
+      <c r="B47" s="74" t="inlineStr">
         <is>
           <t>Sleep rule (see the 'Sleep check' sheet): the two nights before each contest day are in a quiet bed near the venue; sleepers, early flights and red-eyes are only used before day 1 (soft sleeper) or after the contest (anything goes). Sleeper trains replace hotel nights in the Shenyang, Shanghai (D8 seat), Nanchang (Z111 / D136 seat) and EC Final (D17) plans; the 'G-train' / 'no sleeper' variants cost more per trip. Chinese train tickets go on sale 14 days ahead – dates are in the '12306 &amp; ChinaTicketOnline' and '10 Oct' sheets of the fares workbook.</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="32" customHeight="1" s="56">
-      <c r="A47" s="75" t="inlineStr">
+    <row r="48" ht="32" customHeight="1" s="56">
+      <c r="A48" s="75" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B47" s="74" t="inlineStr">
+      <c r="B48" s="74" t="inlineStr">
         <is>
           <t>Sources (10 Oct): Trip.com (flights and hotels, built-in browser), 12306 (official train fares), ChinaTicketOnline (timetable and sale-date check; 30–70% dearer than 12306, not used for booking), SlickTrip (MIAT / Spring fares; Air China is unpriced there).</t>
         </is>
       </c>
     </row>
+    <row r="49"/>
   </sheetData>
   <mergeCells count="14">
     <mergeCell ref="B45:K45"/>
@@ -2230,11 +2287,11 @@
     <mergeCell ref="B35:K35"/>
     <mergeCell ref="B44:K44"/>
     <mergeCell ref="A2:K2"/>
-    <mergeCell ref="B43:K43"/>
     <mergeCell ref="B39:K39"/>
+    <mergeCell ref="B47:K47"/>
+    <mergeCell ref="B48:K48"/>
     <mergeCell ref="B38:K38"/>
-    <mergeCell ref="B47:K47"/>
-    <mergeCell ref="B34:K34"/>
+    <mergeCell ref="B42:K42"/>
     <mergeCell ref="B36:K36"/>
     <mergeCell ref="B37:K37"/>
   </mergeCells>
@@ -8551,19 +8608,19 @@
     <mergeCell ref="E58:L58"/>
     <mergeCell ref="C45:L45"/>
     <mergeCell ref="B38:L38"/>
+    <mergeCell ref="E53:L53"/>
     <mergeCell ref="E59:L59"/>
     <mergeCell ref="E51:L51"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="E54:L54"/>
-    <mergeCell ref="C44:L44"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
-    <mergeCell ref="E53:L53"/>
+    <mergeCell ref="B40:L40"/>
     <mergeCell ref="B41:L41"/>
-    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="C44:L44"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -9903,19 +9960,19 @@
     <mergeCell ref="E58:L58"/>
     <mergeCell ref="C45:L45"/>
     <mergeCell ref="B38:L38"/>
+    <mergeCell ref="E53:L53"/>
     <mergeCell ref="E59:L59"/>
     <mergeCell ref="E51:L51"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="E54:L54"/>
-    <mergeCell ref="C44:L44"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
-    <mergeCell ref="E53:L53"/>
+    <mergeCell ref="B40:L40"/>
     <mergeCell ref="B41:L41"/>
-    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="C44:L44"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -11255,17 +11312,17 @@
     <mergeCell ref="E58:L58"/>
     <mergeCell ref="C45:L45"/>
     <mergeCell ref="B38:L38"/>
-    <mergeCell ref="E53:L53"/>
     <mergeCell ref="E59:L59"/>
     <mergeCell ref="E51:L51"/>
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="E54:L54"/>
+    <mergeCell ref="B40:L40"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
-    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="E53:L53"/>
     <mergeCell ref="B41:L41"/>
     <mergeCell ref="C44:L44"/>
   </mergeCells>
@@ -12612,14 +12669,14 @@
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="E54:L54"/>
-    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="C44:L44"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
     <mergeCell ref="E53:L53"/>
     <mergeCell ref="B41:L41"/>
-    <mergeCell ref="C44:L44"/>
+    <mergeCell ref="B40:L40"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -13959,19 +14016,19 @@
     <mergeCell ref="E58:L58"/>
     <mergeCell ref="C45:L45"/>
     <mergeCell ref="B38:L38"/>
+    <mergeCell ref="E53:L53"/>
     <mergeCell ref="E59:L59"/>
     <mergeCell ref="E51:L51"/>
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="E54:L54"/>
-    <mergeCell ref="C44:L44"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
-    <mergeCell ref="E53:L53"/>
+    <mergeCell ref="B40:L40"/>
     <mergeCell ref="B41:L41"/>
-    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="C44:L44"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -13980,6 +14037,1358 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:L60"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="26" customWidth="1" style="55" min="1" max="1"/>
+    <col width="52" customWidth="1" style="55" min="2" max="2"/>
+    <col width="20" customWidth="1" style="55" min="3" max="3"/>
+    <col width="15" customWidth="1" style="55" min="4" max="4"/>
+    <col width="13" customWidth="1" style="55" min="5" max="5"/>
+    <col width="9" customWidth="1" style="55" min="6" max="7"/>
+    <col width="17" customWidth="1" style="55" min="8" max="8"/>
+    <col width="13" customWidth="1" style="55" min="9" max="9"/>
+    <col width="9" customWidth="1" style="55" min="10" max="10"/>
+    <col width="17" customWidth="1" style="55" min="11" max="11"/>
+    <col width="58" customWidth="1" style="55" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="17.35" customHeight="1" s="56">
+      <c r="A1" s="57" t="inlineStr">
+        <is>
+          <t>Hong Kong – Sleep priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1" s="56">
+      <c r="A2" s="62" t="inlineStr">
+        <is>
+          <t>Sleep over distance: MIAT nonstop, two rooms with four separate twin beds and private bathrooms in a well-reviewed guesthouse in Kowloon (~35–40 min MTR to HKU), airport bus; stays under the ₮12M cap before contingency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="56">
+      <c r="A4" s="60" t="inlineStr">
+        <is>
+          <t>Days in destination (meals &amp; local transport)</t>
+        </is>
+      </c>
+      <c r="B4" s="76" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="C4" s="62" t="inlineStr">
+        <is>
+          <t>8 Jan midday → 11 Jan morning</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="56">
+      <c r="A5" s="62" t="inlineStr">
+        <is>
+          <t>Shared inputs are on the Compare sheet. Scroll down for the day-by-day plan and door-to-door travel times.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="31.5" customHeight="1" s="56">
+      <c r="A7" s="66" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B7" s="66" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C7" s="66" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D7" s="66" t="inlineStr">
+        <is>
+          <t>Travel time</t>
+        </is>
+      </c>
+      <c r="E7" s="66" t="inlineStr">
+        <is>
+          <t>Unit cost (3 ppl)</t>
+        </is>
+      </c>
+      <c r="F7" s="66" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="G7" s="66" t="inlineStr">
+        <is>
+          <t>Qty (3 ppl)</t>
+        </is>
+      </c>
+      <c r="H7" s="66" t="inlineStr">
+        <is>
+          <t>Total MNT – 3 people</t>
+        </is>
+      </c>
+      <c r="I7" s="66" t="inlineStr">
+        <is>
+          <t>Unit cost (4 ppl)</t>
+        </is>
+      </c>
+      <c r="J7" s="66" t="inlineStr">
+        <is>
+          <t>Qty (4 ppl)</t>
+        </is>
+      </c>
+      <c r="K7" s="66" t="inlineStr">
+        <is>
+          <t>Total MNT – 4 people</t>
+        </is>
+      </c>
+      <c r="L7" s="66" t="inlineStr">
+        <is>
+          <t>Source / notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="56">
+      <c r="A8" s="77" t="inlineStr">
+        <is>
+          <t>PAID BY UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="B8" s="78" t="n"/>
+      <c r="C8" s="78" t="n"/>
+      <c r="D8" s="78" t="n"/>
+      <c r="E8" s="78" t="n"/>
+      <c r="F8" s="78" t="n"/>
+      <c r="G8" s="78" t="n"/>
+      <c r="H8" s="78" t="n"/>
+      <c r="I8" s="78" t="n"/>
+      <c r="J8" s="78" t="n"/>
+      <c r="K8" s="78" t="n"/>
+      <c r="L8" s="78" t="n"/>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="56">
+      <c r="A9" s="79" t="inlineStr">
+        <is>
+          <t>Flights</t>
+        </is>
+      </c>
+      <c r="B9" s="80" t="n"/>
+      <c r="C9" s="80" t="n"/>
+      <c r="D9" s="80" t="n"/>
+      <c r="E9" s="80" t="n"/>
+      <c r="F9" s="80" t="n"/>
+      <c r="G9" s="80" t="n"/>
+      <c r="H9" s="80" t="n"/>
+      <c r="I9" s="80" t="n"/>
+      <c r="J9" s="80" t="n"/>
+      <c r="K9" s="80" t="n"/>
+      <c r="L9" s="80" t="n"/>
+    </row>
+    <row r="10" ht="26.85" customHeight="1" s="56">
+      <c r="A10" s="81" t="n"/>
+      <c r="B10" s="82" t="inlineStr">
+        <is>
+          <t>MIAT OM297 Ulaanbaatar → Hong Kong, nonstop 06:45–11:25</t>
+        </is>
+      </c>
+      <c r="C10" s="83" t="inlineStr">
+        <is>
+          <t>8 Jan</t>
+        </is>
+      </c>
+      <c r="D10" s="84" t="n">
+        <v>0.1944444444444444</v>
+      </c>
+      <c r="E10" s="85" t="n">
+        <v>293</v>
+      </c>
+      <c r="F10" s="86" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G10" s="87">
+        <f>Compare!$B$6</f>
+        <v/>
+      </c>
+      <c r="H10" s="88">
+        <f>E10*G10*IF(F10="USD",Compare!$B$8,IF(F10="CNY",Compare!$B$9,IF(F10="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I10" s="89">
+        <f>E10</f>
+        <v/>
+      </c>
+      <c r="J10" s="87">
+        <f>Compare!$B$7</f>
+        <v/>
+      </c>
+      <c r="K10" s="88">
+        <f>I10*J10*IF(F10="USD",Compare!$B$8,IF(F10="CNY",Compare!$B$9,IF(F10="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L10" s="90" t="inlineStr">
+        <is>
+          <t>Trip.com 10 Oct: MIAT nonstop 07:15–11:50 round trip $586 pp (8–11 Jan), split half each way = $293 (SlickTrip $593; $583 on 30 Sep). Cathay codeshare $626; via Seoul $783+</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="26.85" customHeight="1" s="56">
+      <c r="A11" s="81" t="n"/>
+      <c r="B11" s="82" t="inlineStr">
+        <is>
+          <t>MIAT OM298 Hong Kong → Ulaanbaatar, nonstop 12:25–17:05</t>
+        </is>
+      </c>
+      <c r="C11" s="83" t="inlineStr">
+        <is>
+          <t>11 Jan</t>
+        </is>
+      </c>
+      <c r="D11" s="84" t="n">
+        <v>0.1944444444444444</v>
+      </c>
+      <c r="E11" s="85" t="n">
+        <v>293</v>
+      </c>
+      <c r="F11" s="86" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G11" s="87">
+        <f>Compare!$B$6</f>
+        <v/>
+      </c>
+      <c r="H11" s="88">
+        <f>E11*G11*IF(F11="USD",Compare!$B$8,IF(F11="CNY",Compare!$B$9,IF(F11="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I11" s="89">
+        <f>E11</f>
+        <v/>
+      </c>
+      <c r="J11" s="87">
+        <f>Compare!$B$7</f>
+        <v/>
+      </c>
+      <c r="K11" s="88">
+        <f>I11*J11*IF(F11="USD",Compare!$B$8,IF(F11="CNY",Compare!$B$9,IF(F11="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L11" s="90" t="inlineStr">
+        <is>
+          <t>Return half of the $586 pp Trip.com round trip</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="56">
+      <c r="A12" s="79" t="inlineStr">
+        <is>
+          <t>Accommodation</t>
+        </is>
+      </c>
+      <c r="B12" s="80" t="n"/>
+      <c r="C12" s="80" t="n"/>
+      <c r="D12" s="80" t="n"/>
+      <c r="E12" s="80" t="n"/>
+      <c r="F12" s="80" t="n"/>
+      <c r="G12" s="80" t="n"/>
+      <c r="H12" s="80" t="n"/>
+      <c r="I12" s="80" t="n"/>
+      <c r="J12" s="80" t="n"/>
+      <c r="K12" s="80" t="n"/>
+      <c r="L12" s="80" t="n"/>
+    </row>
+    <row r="13" ht="26.85" customHeight="1" s="56">
+      <c r="A13" s="81" t="n"/>
+      <c r="B13" s="82" t="inlineStr">
+        <is>
+          <t>Good Fortune Inn, Kowloon (3 ppl: triple room; 4 ppl: 2 rooms, 2 twin beds each, private bathroom; ~35–40 min MTR to HKU)</t>
+        </is>
+      </c>
+      <c r="C13" s="83" t="inlineStr">
+        <is>
+          <t>8–11 Jan (3 nights)</t>
+        </is>
+      </c>
+      <c r="D13" s="81" t="n"/>
+      <c r="E13" s="85" t="n">
+        <v>586.33</v>
+      </c>
+      <c r="F13" s="86" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="G13" s="91" t="n">
+        <v>3</v>
+      </c>
+      <c r="H13" s="88">
+        <f>E13*G13*IF(F13="USD",Compare!$B$8,IF(F13="CNY",Compare!$B$9,IF(F13="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I13" s="85" t="n">
+        <v>963</v>
+      </c>
+      <c r="J13" s="91" t="n">
+        <v>3</v>
+      </c>
+      <c r="K13" s="88">
+        <f>I13*J13*IF(F13="USD",Compare!$B$8,IF(F13="CNY",Compare!$B$9,IF(F13="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L13" s="90" t="inlineStr">
+        <is>
+          <t>Booking.com 10 Oct, 8–11 Jan: HK$1,759 (3 ppl, triple room) / HK$2,889 (4 ppl, 2 rooms with 4 twin beds) for 3 nights; rated 8.6 (715 reviews). Alternatives with real hotel rooms: ALVA Hotel by Royal, Tsuen Wan (8.5, 1,038 reviews) HK$3,890, two queen beds, ~50 min to HKU; Sleep Inn (8.4) HK$3,401 but one full bed per room (two people share a bed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1" s="56">
+      <c r="A14" s="79" t="inlineStr">
+        <is>
+          <t>Meals &amp; local transport</t>
+        </is>
+      </c>
+      <c r="B14" s="80" t="n"/>
+      <c r="C14" s="80" t="n"/>
+      <c r="D14" s="80" t="n"/>
+      <c r="E14" s="80" t="n"/>
+      <c r="F14" s="80" t="n"/>
+      <c r="G14" s="80" t="n"/>
+      <c r="H14" s="80" t="n"/>
+      <c r="I14" s="80" t="n"/>
+      <c r="J14" s="80" t="n"/>
+      <c r="K14" s="80" t="n"/>
+      <c r="L14" s="80" t="n"/>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="56">
+      <c r="A15" s="81" t="n"/>
+      <c r="B15" s="82" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="C15" s="83" t="inlineStr">
+        <is>
+          <t>in Hong Kong</t>
+        </is>
+      </c>
+      <c r="D15" s="81" t="n"/>
+      <c r="E15" s="92" t="n">
+        <v>180</v>
+      </c>
+      <c r="F15" s="86" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="G15" s="87">
+        <f>Compare!$B$6*$B$4</f>
+        <v/>
+      </c>
+      <c r="H15" s="88">
+        <f>E15*G15*IF(F15="USD",Compare!$B$8,IF(F15="CNY",Compare!$B$9,IF(F15="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I15" s="93">
+        <f>E15</f>
+        <v/>
+      </c>
+      <c r="J15" s="87">
+        <f>Compare!$B$7*$B$4</f>
+        <v/>
+      </c>
+      <c r="K15" s="88">
+        <f>I15*J15*IF(F15="USD",Compare!$B$8,IF(F15="CNY",Compare!$B$9,IF(F15="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L15" s="90" t="inlineStr">
+        <is>
+          <t>ASSUMPTION ~180 HKD/person/day (cha chaan teng, canteens)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="56">
+      <c r="A16" s="81" t="n"/>
+      <c r="B16" s="82" t="inlineStr">
+        <is>
+          <t>MTR / buses (Octopus card)</t>
+        </is>
+      </c>
+      <c r="C16" s="83" t="inlineStr">
+        <is>
+          <t>in Hong Kong</t>
+        </is>
+      </c>
+      <c r="D16" s="81" t="n"/>
+      <c r="E16" s="92" t="n">
+        <v>40</v>
+      </c>
+      <c r="F16" s="86" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="G16" s="87">
+        <f>Compare!$B$6*$B$4</f>
+        <v/>
+      </c>
+      <c r="H16" s="88">
+        <f>E16*G16*IF(F16="USD",Compare!$B$8,IF(F16="CNY",Compare!$B$9,IF(F16="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I16" s="93">
+        <f>E16</f>
+        <v/>
+      </c>
+      <c r="J16" s="87">
+        <f>Compare!$B$7*$B$4</f>
+        <v/>
+      </c>
+      <c r="K16" s="88">
+        <f>I16*J16*IF(F16="USD",Compare!$B$8,IF(F16="CNY",Compare!$B$9,IF(F16="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L16" s="90" t="inlineStr">
+        <is>
+          <t>ASSUMPTION ~40 HKD/person/day</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1" s="56">
+      <c r="A17" s="81" t="n"/>
+      <c r="B17" s="82" t="inlineStr">
+        <is>
+          <t>Airport bus A21 (HKG ↔ Kowloon / Yau Ma Tei), both ways</t>
+        </is>
+      </c>
+      <c r="C17" s="83" t="inlineStr">
+        <is>
+          <t>8 &amp; 11 Jan</t>
+        </is>
+      </c>
+      <c r="D17" s="81" t="n"/>
+      <c r="E17" s="92" t="n">
+        <v>80</v>
+      </c>
+      <c r="F17" s="86" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="G17" s="87">
+        <f>Compare!$B$6</f>
+        <v/>
+      </c>
+      <c r="H17" s="88">
+        <f>E17*G17*IF(F17="USD",Compare!$B$8,IF(F17="CNY",Compare!$B$9,IF(F17="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I17" s="93">
+        <f>E17</f>
+        <v/>
+      </c>
+      <c r="J17" s="87">
+        <f>Compare!$B$7</f>
+        <v/>
+      </c>
+      <c r="K17" s="88">
+        <f>I17*J17*IF(F17="USD",Compare!$B$8,IF(F17="CNY",Compare!$B$9,IF(F17="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L17" s="90" t="inlineStr">
+        <is>
+          <t>ASSUMPTION ~HK$40 per person each way on the A21 airport bus (~60 min) instead of the HK$115 Airport Express + walk</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1" s="56">
+      <c r="A18" s="94" t="inlineStr">
+        <is>
+          <t>PAID PERSONALLY (university won't cover)</t>
+        </is>
+      </c>
+      <c r="B18" s="95" t="n"/>
+      <c r="C18" s="95" t="n"/>
+      <c r="D18" s="95" t="n"/>
+      <c r="E18" s="95" t="n"/>
+      <c r="F18" s="95" t="n"/>
+      <c r="G18" s="95" t="n"/>
+      <c r="H18" s="95" t="n"/>
+      <c r="I18" s="95" t="n"/>
+      <c r="J18" s="95" t="n"/>
+      <c r="K18" s="95" t="n"/>
+      <c r="L18" s="95" t="n"/>
+    </row>
+    <row r="19" ht="15" customHeight="1" s="56">
+      <c r="A19" s="79" t="inlineStr">
+        <is>
+          <t>Contest fee</t>
+        </is>
+      </c>
+      <c r="B19" s="80" t="n"/>
+      <c r="C19" s="80" t="n"/>
+      <c r="D19" s="80" t="n"/>
+      <c r="E19" s="80" t="n"/>
+      <c r="F19" s="80" t="n"/>
+      <c r="G19" s="80" t="n"/>
+      <c r="H19" s="80" t="n"/>
+      <c r="I19" s="80" t="n"/>
+      <c r="J19" s="80" t="n"/>
+      <c r="K19" s="80" t="n"/>
+      <c r="L19" s="80" t="n"/>
+    </row>
+    <row r="20" ht="22.35" customHeight="1" s="56">
+      <c r="A20" s="81" t="n"/>
+      <c r="B20" s="82" t="inlineStr">
+        <is>
+          <t>Hong Kong regional registration fee (per team)</t>
+        </is>
+      </c>
+      <c r="C20" s="83" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D20" s="81" t="n"/>
+      <c r="E20" s="85" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F20" s="86" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="G20" s="91" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="88">
+        <f>E20*G20*IF(F20="USD",Compare!$B$8,IF(F20="CNY",Compare!$B$9,IF(F20="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I20" s="89">
+        <f>E20</f>
+        <v/>
+      </c>
+      <c r="J20" s="91" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="88">
+        <f>I20*J20*IF(F20="USD",Compare!$B$8,IF(F20="CNY",Compare!$B$9,IF(F20="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L20" s="90" t="inlineStr">
+        <is>
+          <t>1,800 HKD/team at the 2025 Hong Kong regional (HKUST); 2026 host listed as HKU – confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1" s="56">
+      <c r="A21" s="79" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B21" s="80" t="n"/>
+      <c r="C21" s="80" t="n"/>
+      <c r="D21" s="80" t="n"/>
+      <c r="E21" s="80" t="n"/>
+      <c r="F21" s="80" t="n"/>
+      <c r="G21" s="80" t="n"/>
+      <c r="H21" s="80" t="n"/>
+      <c r="I21" s="80" t="n"/>
+      <c r="J21" s="80" t="n"/>
+      <c r="K21" s="80" t="n"/>
+      <c r="L21" s="80" t="n"/>
+    </row>
+    <row r="22" ht="15" customHeight="1" s="56">
+      <c r="A22" s="81" t="n"/>
+      <c r="B22" s="82" t="inlineStr">
+        <is>
+          <t>Taxi to/from Chinggis Khaan airport (UB), per trip</t>
+        </is>
+      </c>
+      <c r="C22" s="83" t="inlineStr">
+        <is>
+          <t>out &amp; back</t>
+        </is>
+      </c>
+      <c r="D22" s="84" t="n">
+        <v>0.04166666666666666</v>
+      </c>
+      <c r="E22" s="92" t="n">
+        <v>100000</v>
+      </c>
+      <c r="F22" s="86" t="inlineStr">
+        <is>
+          <t>MNT</t>
+        </is>
+      </c>
+      <c r="G22" s="91" t="n">
+        <v>2</v>
+      </c>
+      <c r="H22" s="88">
+        <f>E22*G22*IF(F22="USD",Compare!$B$8,IF(F22="CNY",Compare!$B$9,IF(F22="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I22" s="93">
+        <f>E22</f>
+        <v/>
+      </c>
+      <c r="J22" s="91" t="n">
+        <v>2</v>
+      </c>
+      <c r="K22" s="88">
+        <f>I22*J22*IF(F22="USD",Compare!$B$8,IF(F22="CNY",Compare!$B$9,IF(F22="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L22" s="90" t="inlineStr">
+        <is>
+          <t>ASSUMPTION 100k MNT per trip for the group</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1" s="56">
+      <c r="A23" s="81" t="n"/>
+      <c r="B23" s="82" t="inlineStr">
+        <is>
+          <t>Travel medical insurance</t>
+        </is>
+      </c>
+      <c r="C23" s="83" t="n"/>
+      <c r="D23" s="81" t="n"/>
+      <c r="E23" s="92" t="n">
+        <v>30000</v>
+      </c>
+      <c r="F23" s="86" t="inlineStr">
+        <is>
+          <t>MNT</t>
+        </is>
+      </c>
+      <c r="G23" s="87">
+        <f>Compare!$B$6</f>
+        <v/>
+      </c>
+      <c r="H23" s="88">
+        <f>E23*G23*IF(F23="USD",Compare!$B$8,IF(F23="CNY",Compare!$B$9,IF(F23="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I23" s="93">
+        <f>E23</f>
+        <v/>
+      </c>
+      <c r="J23" s="87">
+        <f>Compare!$B$7</f>
+        <v/>
+      </c>
+      <c r="K23" s="88">
+        <f>I23*J23*IF(F23="USD",Compare!$B$8,IF(F23="CNY",Compare!$B$9,IF(F23="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L23" s="90" t="inlineStr">
+        <is>
+          <t>ASSUMPTION ~30k MNT per person, Mongolian insurer</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1" s="56">
+      <c r="A24" s="81" t="n"/>
+      <c r="B24" s="82" t="inlineStr">
+        <is>
+          <t>Mobile data eSIM</t>
+        </is>
+      </c>
+      <c r="C24" s="83" t="n"/>
+      <c r="D24" s="81" t="n"/>
+      <c r="E24" s="92" t="n">
+        <v>10</v>
+      </c>
+      <c r="F24" s="86" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G24" s="87">
+        <f>Compare!$B$6</f>
+        <v/>
+      </c>
+      <c r="H24" s="88">
+        <f>E24*G24*IF(F24="USD",Compare!$B$8,IF(F24="CNY",Compare!$B$9,IF(F24="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I24" s="93">
+        <f>E24</f>
+        <v/>
+      </c>
+      <c r="J24" s="87">
+        <f>Compare!$B$7</f>
+        <v/>
+      </c>
+      <c r="K24" s="88">
+        <f>I24*J24*IF(F24="USD",Compare!$B$8,IF(F24="CNY",Compare!$B$9,IF(F24="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L24" s="90" t="inlineStr">
+        <is>
+          <t>ASSUMPTION ~$10 pp</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22.35" customHeight="1" s="56">
+      <c r="A25" s="81" t="n"/>
+      <c r="B25" s="82" t="inlineStr">
+        <is>
+          <t>Visa</t>
+        </is>
+      </c>
+      <c r="C25" s="83" t="n"/>
+      <c r="D25" s="81" t="n"/>
+      <c r="E25" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="86" t="inlineStr">
+        <is>
+          <t>MNT</t>
+        </is>
+      </c>
+      <c r="G25" s="87">
+        <f>Compare!$B$6</f>
+        <v/>
+      </c>
+      <c r="H25" s="88">
+        <f>E25*G25*IF(F25="USD",Compare!$B$8,IF(F25="CNY",Compare!$B$9,IF(F25="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="I25" s="89">
+        <f>E25</f>
+        <v/>
+      </c>
+      <c r="J25" s="87">
+        <f>Compare!$B$7</f>
+        <v/>
+      </c>
+      <c r="K25" s="88">
+        <f>I25*J25*IF(F25="USD",Compare!$B$8,IF(F25="CNY",Compare!$B$9,IF(F25="HKD",Compare!$B$10,1)))</f>
+        <v/>
+      </c>
+      <c r="L25" s="90" t="inlineStr">
+        <is>
+          <t>Mongolian passports: visa-free (mainland China up to 30 days; Hong Kong up to 14 days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1" s="56">
+      <c r="G27" s="60" t="n"/>
+      <c r="H27" s="96" t="inlineStr">
+        <is>
+          <t>3 people – UNFUNDED</t>
+        </is>
+      </c>
+      <c r="K27" s="96" t="inlineStr">
+        <is>
+          <t>4 people – FUNDED ₮12M</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1" s="56">
+      <c r="G28" s="97" t="inlineStr">
+        <is>
+          <t>University-paid subtotal</t>
+        </is>
+      </c>
+      <c r="H28" s="98">
+        <f>SUM(H9:H17)</f>
+        <v/>
+      </c>
+      <c r="K28" s="98">
+        <f>SUM(K9:K17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1" s="56">
+      <c r="G29" s="99" t="inlineStr">
+        <is>
+          <t>Contingency</t>
+        </is>
+      </c>
+      <c r="H29" s="100">
+        <f>H28*Compare!$B$11</f>
+        <v/>
+      </c>
+      <c r="K29" s="100">
+        <f>K28*Compare!$B$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1" s="56">
+      <c r="G30" s="97" t="inlineStr">
+        <is>
+          <t>University-paid total incl. contingency</t>
+        </is>
+      </c>
+      <c r="H30" s="98">
+        <f>H28+H29</f>
+        <v/>
+      </c>
+      <c r="K30" s="98">
+        <f>K28+K29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="56">
+      <c r="G31" s="97" t="inlineStr">
+        <is>
+          <t>Funding left (negative = over)</t>
+        </is>
+      </c>
+      <c r="H31" s="101">
+        <f>Compare!$B$12-H30</f>
+        <v/>
+      </c>
+      <c r="K31" s="101">
+        <f>Compare!$B$5-K30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1" s="56">
+      <c r="G32" s="97" t="inlineStr">
+        <is>
+          <t>Personal costs – team</t>
+        </is>
+      </c>
+      <c r="H32" s="102">
+        <f>SUM(H19:H25)</f>
+        <v/>
+      </c>
+      <c r="K32" s="102">
+        <f>SUM(K19:K25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1" s="56">
+      <c r="G33" s="97" t="inlineStr">
+        <is>
+          <t>Out-of-pocket per person (personal + any overrun)</t>
+        </is>
+      </c>
+      <c r="H33" s="102">
+        <f>(H32+MAX(0,-H31))/Compare!$B$6</f>
+        <v/>
+      </c>
+      <c r="K33" s="102">
+        <f>(K32+MAX(0,-K31))/Compare!$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="15" customHeight="1" s="56">
+      <c r="G34" s="97" t="inlineStr">
+        <is>
+          <t>Whole trip cost (university + personal)</t>
+        </is>
+      </c>
+      <c r="H34" s="103">
+        <f>H30+H32</f>
+        <v/>
+      </c>
+      <c r="K34" s="103">
+        <f>K30+K32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="15" customHeight="1" s="56">
+      <c r="G35" s="99" t="inlineStr">
+        <is>
+          <t>Time in planes &amp; trains</t>
+        </is>
+      </c>
+      <c r="H35" s="104">
+        <f>SUM(D10:D11)</f>
+        <v/>
+      </c>
+      <c r="K35" s="104">
+        <f>SUM(D10:D11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="15" customHeight="1" s="56">
+      <c r="A37" s="72" t="inlineStr">
+        <is>
+          <t>Key facts</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="15" customHeight="1" s="56">
+      <c r="A38" s="75" t="inlineStr">
+        <is>
+          <t>Contest</t>
+        </is>
+      </c>
+      <c r="B38" s="74" t="inlineStr">
+        <is>
+          <t>Asia Hong Kong Regional, 9–10 Jan 2027 (provisional). Host listed as HKU on a coach's tracking page, but the 2025 regional was at HKUST (Clear Water Bay) – the site rotates, so confirm before paying for a hotel near any one campus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="15" customHeight="1" s="56">
+      <c r="A39" s="75" t="inlineStr">
+        <is>
+          <t>Why this plan</t>
+        </is>
+      </c>
+      <c r="B39" s="74" t="inlineStr">
+        <is>
+          <t>The hotel is chosen for the sleep, not the distance: every contestant has their own bed, a private bathroom and a quiet room; the flights are fixed. A guesthouse in Kowloon also keeps the team on the MTR whichever campus hosts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="15" customHeight="1" s="56">
+      <c r="A40" s="75" t="inlineStr">
+        <is>
+          <t>Entry</t>
+        </is>
+      </c>
+      <c r="B40" s="74" t="inlineStr">
+        <is>
+          <t>Mongolian passport holders can visit Hong Kong visa-free for up to 14 days.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="15" customHeight="1" s="56">
+      <c r="A41" s="75" t="inlineStr">
+        <is>
+          <t>Trade-off</t>
+        </is>
+      </c>
+      <c r="B41" s="74" t="inlineStr">
+        <is>
+          <t>~35–40 min each way on the MTR (wake ~06:15 for a 09:00 start; still ≥7.5 h in bed with lights out at 22:30). Request a high floor away from the street, bring earplugs. Guesthouse rooms are small. Fits ₮12M before the 10% contingency (about ₮11.3M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="15" customHeight="1" s="56">
+      <c r="A43" s="72" t="inlineStr">
+        <is>
+          <t>Day-by-day plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="15" customHeight="1" s="56">
+      <c r="A44" s="96" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B44" s="96" t="inlineStr">
+        <is>
+          <t>Sleep in</t>
+        </is>
+      </c>
+      <c r="C44" s="96" t="inlineStr">
+        <is>
+          <t>What happens</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="15" customHeight="1" s="56">
+      <c r="A45" s="74" t="inlineStr">
+        <is>
+          <t>Fri 8 Jan</t>
+        </is>
+      </c>
+      <c r="B45" s="74" t="inlineStr">
+        <is>
+          <t>Hong Kong</t>
+        </is>
+      </c>
+      <c r="C45" s="74" t="inlineStr">
+        <is>
+          <t>MIAT OM297 UB 06:45 → Hong Kong 11:25 (4 h 40 min). Airport bus A21 to Yau Ma Tei, leave bags, check in at the guesthouse and nap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="15" customHeight="1" s="56">
+      <c r="A46" s="74" t="inlineStr">
+        <is>
+          <t>Sat 9 Jan</t>
+        </is>
+      </c>
+      <c r="B46" s="74" t="inlineStr">
+        <is>
+          <t>Hong Kong</t>
+        </is>
+      </c>
+      <c r="C46" s="74" t="inlineStr">
+        <is>
+          <t>Registration, opening and warm-up at the University of Hong Kong (2025 HK regional used the same day-1 pattern).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="15" customHeight="1" s="56">
+      <c r="A47" s="74" t="inlineStr">
+        <is>
+          <t>Sun 10 Jan</t>
+        </is>
+      </c>
+      <c r="B47" s="74" t="inlineStr">
+        <is>
+          <t>Hong Kong</t>
+        </is>
+      </c>
+      <c r="C47" s="74" t="inlineStr">
+        <is>
+          <t>HONG KONG REGIONAL contest day, closing &amp; solutions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="15" customHeight="1" s="56">
+      <c r="A48" s="74" t="inlineStr">
+        <is>
+          <t>Mon 11 Jan</t>
+        </is>
+      </c>
+      <c r="B48" s="74" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="C48" s="74" t="inlineStr">
+        <is>
+          <t>MIAT OM298 Hong Kong 12:25 → UB 17:05.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="15" customHeight="1" s="56">
+      <c r="A50" s="72" t="inlineStr">
+        <is>
+          <t>Door-to-door travel times</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="15" customHeight="1" s="56">
+      <c r="A51" s="96" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B51" s="96" t="inlineStr">
+        <is>
+          <t>Leg</t>
+        </is>
+      </c>
+      <c r="C51" s="96" t="inlineStr">
+        <is>
+          <t>Mode</t>
+        </is>
+      </c>
+      <c r="D51" s="96" t="inlineStr">
+        <is>
+          <t>Expected time</t>
+        </is>
+      </c>
+      <c r="E51" s="96" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="15" customHeight="1" s="56">
+      <c r="A52" s="105" t="inlineStr">
+        <is>
+          <t>8 Jan</t>
+        </is>
+      </c>
+      <c r="B52" s="105" t="inlineStr">
+        <is>
+          <t>Home → Chinggis Khaan airport</t>
+        </is>
+      </c>
+      <c r="C52" s="82" t="inlineStr">
+        <is>
+          <t>Taxi (~50 km)</t>
+        </is>
+      </c>
+      <c r="D52" s="104" t="n">
+        <v>0.04166666666666666</v>
+      </c>
+      <c r="E52" s="106" t="inlineStr">
+        <is>
+          <t>Leave ~03:45 for 06:45 flight</t>
+        </is>
+      </c>
+      <c r="F52" s="107" t="n"/>
+      <c r="G52" s="107" t="n"/>
+      <c r="H52" s="107" t="n"/>
+      <c r="I52" s="107" t="n"/>
+      <c r="J52" s="107" t="n"/>
+      <c r="K52" s="107" t="n"/>
+      <c r="L52" s="107" t="n"/>
+    </row>
+    <row r="53" ht="26.85" customHeight="1" s="56">
+      <c r="A53" s="105" t="inlineStr">
+        <is>
+          <t>8 Jan</t>
+        </is>
+      </c>
+      <c r="B53" s="105" t="inlineStr">
+        <is>
+          <t>Ulaanbaatar → Hong Kong (HKG)</t>
+        </is>
+      </c>
+      <c r="C53" s="82" t="inlineStr">
+        <is>
+          <t>MIAT OM297 06:45–11:25</t>
+        </is>
+      </c>
+      <c r="D53" s="84" t="n">
+        <v>0.1944444444444444</v>
+      </c>
+      <c r="E53" s="106" t="n"/>
+      <c r="F53" s="107" t="n"/>
+      <c r="G53" s="107" t="n"/>
+      <c r="H53" s="107" t="n"/>
+      <c r="I53" s="107" t="n"/>
+      <c r="J53" s="107" t="n"/>
+      <c r="K53" s="107" t="n"/>
+      <c r="L53" s="107" t="n"/>
+    </row>
+    <row r="54" ht="15" customHeight="1" s="56">
+      <c r="A54" s="105" t="inlineStr">
+        <is>
+          <t>8 Jan</t>
+        </is>
+      </c>
+      <c r="B54" s="105" t="inlineStr">
+        <is>
+          <t>HKG arrival: immigration, bags</t>
+        </is>
+      </c>
+      <c r="C54" s="82" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D54" s="104" t="n">
+        <v>0.02777777777777778</v>
+      </c>
+      <c r="E54" s="106" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="F54" s="107" t="n"/>
+      <c r="G54" s="107" t="n"/>
+      <c r="H54" s="107" t="n"/>
+      <c r="I54" s="107" t="n"/>
+      <c r="J54" s="107" t="n"/>
+      <c r="K54" s="107" t="n"/>
+      <c r="L54" s="107" t="n"/>
+    </row>
+    <row r="55" ht="39.55" customHeight="1" s="56">
+      <c r="A55" s="105" t="inlineStr">
+        <is>
+          <t>8 Jan</t>
+        </is>
+      </c>
+      <c r="B55" s="105" t="inlineStr">
+        <is>
+          <t>HKG → Good Fortune Inn</t>
+        </is>
+      </c>
+      <c r="C55" s="82" t="inlineStr">
+        <is>
+          <t>Airport bus A21 + walk</t>
+        </is>
+      </c>
+      <c r="D55" s="104" t="n">
+        <v>0.04166666666666666</v>
+      </c>
+      <c r="E55" s="106" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="F55" s="107" t="n"/>
+      <c r="G55" s="107" t="n"/>
+      <c r="H55" s="107" t="n"/>
+      <c r="I55" s="107" t="n"/>
+      <c r="J55" s="107" t="n"/>
+      <c r="K55" s="107" t="n"/>
+      <c r="L55" s="107" t="n"/>
+    </row>
+    <row r="56" ht="15" customHeight="1" s="56">
+      <c r="A56" s="105" t="inlineStr">
+        <is>
+          <t>9–10 Jan</t>
+        </is>
+      </c>
+      <c r="B56" s="105" t="inlineStr">
+        <is>
+          <t>Hotel ↔ HKU (each way)</t>
+        </is>
+      </c>
+      <c r="C56" s="82" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D56" s="108" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="E56" s="106" t="inlineStr">
+        <is>
+          <t>~35–40 min MTR (Yau Ma Tei → Admiralty → HKU); leave ~07:15 for a 09:00 start</t>
+        </is>
+      </c>
+      <c r="F56" s="107" t="n"/>
+      <c r="G56" s="107" t="n"/>
+      <c r="H56" s="107" t="n"/>
+      <c r="I56" s="107" t="n"/>
+      <c r="J56" s="107" t="n"/>
+      <c r="K56" s="107" t="n"/>
+      <c r="L56" s="107" t="n"/>
+    </row>
+    <row r="57" ht="26.85" customHeight="1" s="56">
+      <c r="A57" s="105" t="inlineStr">
+        <is>
+          <t>11 Jan</t>
+        </is>
+      </c>
+      <c r="B57" s="105" t="inlineStr">
+        <is>
+          <t>Guesthouse → HKG</t>
+        </is>
+      </c>
+      <c r="C57" s="82" t="inlineStr">
+        <is>
+          <t>Airport bus A21 + walk</t>
+        </is>
+      </c>
+      <c r="D57" s="104" t="n">
+        <v>0.04166666666666666</v>
+      </c>
+      <c r="E57" s="106" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="F57" s="107" t="n"/>
+      <c r="G57" s="107" t="n"/>
+      <c r="H57" s="107" t="n"/>
+      <c r="I57" s="107" t="n"/>
+      <c r="J57" s="107" t="n"/>
+      <c r="K57" s="107" t="n"/>
+      <c r="L57" s="107" t="n"/>
+    </row>
+    <row r="58" ht="26.85" customHeight="1" s="56">
+      <c r="A58" s="105" t="inlineStr">
+        <is>
+          <t>11 Jan</t>
+        </is>
+      </c>
+      <c r="B58" s="105" t="inlineStr">
+        <is>
+          <t>Hong Kong (HKG) → Ulaanbaatar</t>
+        </is>
+      </c>
+      <c r="C58" s="82" t="inlineStr">
+        <is>
+          <t>MIAT OM298 12:25–17:05</t>
+        </is>
+      </c>
+      <c r="D58" s="84" t="n">
+        <v>0.1944444444444444</v>
+      </c>
+      <c r="E58" s="106" t="inlineStr">
+        <is>
+          <t>Be at HKG by ~10:25</t>
+        </is>
+      </c>
+      <c r="F58" s="107" t="n"/>
+      <c r="G58" s="107" t="n"/>
+      <c r="H58" s="107" t="n"/>
+      <c r="I58" s="107" t="n"/>
+      <c r="J58" s="107" t="n"/>
+      <c r="K58" s="107" t="n"/>
+      <c r="L58" s="107" t="n"/>
+    </row>
+    <row r="59" ht="14.15" customHeight="1" s="56">
+      <c r="A59" s="105" t="inlineStr">
+        <is>
+          <t>11 Jan</t>
+        </is>
+      </c>
+      <c r="B59" s="105" t="inlineStr">
+        <is>
+          <t>Chinggis Khaan airport → home</t>
+        </is>
+      </c>
+      <c r="C59" s="82" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="D59" s="104" t="n">
+        <v>0.04166666666666666</v>
+      </c>
+      <c r="E59" s="106" t="n"/>
+      <c r="F59" s="107" t="n"/>
+      <c r="G59" s="107" t="n"/>
+      <c r="H59" s="107" t="n"/>
+      <c r="I59" s="107" t="n"/>
+      <c r="J59" s="107" t="n"/>
+      <c r="K59" s="107" t="n"/>
+      <c r="L59" s="107" t="n"/>
+    </row>
+    <row r="60" ht="15" customHeight="1" s="56">
+      <c r="C60" s="59" t="inlineStr">
+        <is>
+          <t>Total door-to-door</t>
+        </is>
+      </c>
+      <c r="D60" s="109">
+        <f>SUM(D52:D59)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="18">
+    <mergeCell ref="E57:L57"/>
+    <mergeCell ref="E56:L56"/>
+    <mergeCell ref="E58:L58"/>
+    <mergeCell ref="C45:L45"/>
+    <mergeCell ref="B38:L38"/>
+    <mergeCell ref="E53:L53"/>
+    <mergeCell ref="E59:L59"/>
+    <mergeCell ref="E51:L51"/>
+    <mergeCell ref="C48:L48"/>
+    <mergeCell ref="B39:L39"/>
+    <mergeCell ref="E54:L54"/>
+    <mergeCell ref="E55:L55"/>
+    <mergeCell ref="E52:L52"/>
+    <mergeCell ref="C46:L46"/>
+    <mergeCell ref="C47:L47"/>
+    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="B41:L41"/>
+    <mergeCell ref="C44:L44"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15615,7 +17024,934 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" style="56" min="1" max="1"/>
+    <col width="22" customWidth="1" style="56" min="2" max="2"/>
+    <col width="32" customWidth="1" style="56" min="3" max="3"/>
+    <col width="34" customWidth="1" style="56" min="4" max="4"/>
+    <col width="30" customWidth="1" style="56" min="5" max="5"/>
+    <col width="22" customWidth="1" style="56" min="6" max="6"/>
+    <col width="10" customWidth="1" style="56" min="7" max="7"/>
+    <col width="70" customWidth="1" style="56" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="115" t="inlineStr">
+        <is>
+          <t>Sleep check – protect the nights before the contest, spend nothing on comfort after it</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="78" customHeight="1" s="56">
+      <c r="A2" s="116" t="inlineStr">
+        <is>
+          <t>Rules used: (1) the two nights before the contest day are in a real bed, quiet, ≤30 min from the venue, ≥7.5 h in bed and no wake-up before ~06:00 on contest morning; (2) no overnight train or flight on the contest eve; a sleeper before day 1 only if it is a soft sleeper that arrives by midday and there is a bed night in between; (3) flights before 08:00 only ≥2 nights before the contest; (4) after the contest anything goes – hard sleepers, seats, red-eye trains, 04:30 airport runs – so the cheapest option is used. No time-zone effect: Mongolia, China and Hong Kong are all UTC+8.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="117" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="B4" s="117" t="inlineStr">
+        <is>
+          <t>Contest day / day 1</t>
+        </is>
+      </c>
+      <c r="C4" s="117" t="inlineStr">
+        <is>
+          <t>Night −3</t>
+        </is>
+      </c>
+      <c r="D4" s="117" t="inlineStr">
+        <is>
+          <t>Night −2 (before day 1)</t>
+        </is>
+      </c>
+      <c r="E4" s="117" t="inlineStr">
+        <is>
+          <t>Night −1 (contest eve)</t>
+        </is>
+      </c>
+      <c r="F4" s="117" t="inlineStr">
+        <is>
+          <t>Contest morning</t>
+        </is>
+      </c>
+      <c r="G4" s="117" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="H4" s="117" t="inlineStr">
+        <is>
+          <t>Sleep fix / what changed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="66" customHeight="1" s="56">
+      <c r="A5" s="118" t="inlineStr">
+        <is>
+          <t>Shenyang – Comfort</t>
+        </is>
+      </c>
+      <c r="B5" s="116" t="inlineStr">
+        <is>
+          <t>Sun 15 Nov / Sat 14 Nov</t>
+        </is>
+      </c>
+      <c r="C5" s="116" t="inlineStr">
+        <is>
+          <t>12 Nov RiCH hotel (after a 04:30 start for MIAT 07:30; nap in the afternoon)</t>
+        </is>
+      </c>
+      <c r="D5" s="116" t="inlineStr">
+        <is>
+          <t>13 Nov RiCH, free rest day</t>
+        </is>
+      </c>
+      <c r="E5" s="116" t="inlineStr">
+        <is>
+          <t>14 Nov RiCH, family room, quiet</t>
+        </is>
+      </c>
+      <c r="F5" s="116" t="inlineStr">
+        <is>
+          <t>Walk 18 min, wake ~07:00</t>
+        </is>
+      </c>
+      <c r="G5" s="119" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="H5" s="116" t="inlineStr">
+        <is>
+          <t>Sleeper K54 is after the contest, so it is now a hard sleeper (soft was ¥263): saves ~₮0.16M (₮6.2M total).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="66" customHeight="1" s="56">
+      <c r="A6" s="118" t="inlineStr">
+        <is>
+          <t>Shenyang – Budget</t>
+        </is>
+      </c>
+      <c r="B6" s="116" t="inlineStr">
+        <is>
+          <t>Sun 15 Nov / Sat 14 Nov</t>
+        </is>
+      </c>
+      <c r="C6" s="116" t="inlineStr">
+        <is>
+          <t>12 Nov at home</t>
+        </is>
+      </c>
+      <c r="D6" s="116" t="inlineStr">
+        <is>
+          <t>13 Nov K53 soft sleeper 22:35–07:00 (was hard): ~5–6 h, then day-1 registration</t>
+        </is>
+      </c>
+      <c r="E6" s="116" t="inlineStr">
+        <is>
+          <t>14 Nov Bestay hotel (8.2, budget chain)</t>
+        </is>
+      </c>
+      <c r="F6" s="116" t="inlineStr">
+        <is>
+          <t>Metro 25 min, wake ~06:30</t>
+        </is>
+      </c>
+      <c r="G6" s="120" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="H6" s="116" t="inlineStr">
+        <is>
+          <t>K53 is the night before day 1, so it is now a soft sleeper (+¥92 pp, +₮0.16M; ₮5.2M total). Nap on arrival; the contest eve is in a bed. Safer: Comfort or either G-train variant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="66" customHeight="1" s="56">
+      <c r="A7" s="118" t="inlineStr">
+        <is>
+          <t>Shenyang – Comfort (G-train)</t>
+        </is>
+      </c>
+      <c r="B7" s="116" t="inlineStr">
+        <is>
+          <t>Sun 15 Nov / Sat 14 Nov</t>
+        </is>
+      </c>
+      <c r="C7" s="116" t="inlineStr">
+        <is>
+          <t>12 Nov RiCH hotel</t>
+        </is>
+      </c>
+      <c r="D7" s="116" t="inlineStr">
+        <is>
+          <t>13 Nov RiCH</t>
+        </is>
+      </c>
+      <c r="E7" s="116" t="inlineStr">
+        <is>
+          <t>14 Nov RiCH</t>
+        </is>
+      </c>
+      <c r="F7" s="116" t="inlineStr">
+        <is>
+          <t>Walk 18 min, wake ~07:00</t>
+        </is>
+      </c>
+      <c r="G7" s="119" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="H7" s="116" t="inlineStr">
+        <is>
+          <t>All beds before the contest; the Beijing hotel night (Dequan) is after it. +0.5M vs the sleeper plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="66" customHeight="1" s="56">
+      <c r="A8" s="118" t="inlineStr">
+        <is>
+          <t>Shenyang – Budget (G-train)</t>
+        </is>
+      </c>
+      <c r="B8" s="116" t="inlineStr">
+        <is>
+          <t>Sun 15 Nov / Sat 14 Nov</t>
+        </is>
+      </c>
+      <c r="C8" s="116" t="inlineStr">
+        <is>
+          <t>12 Nov at home</t>
+        </is>
+      </c>
+      <c r="D8" s="116" t="inlineStr">
+        <is>
+          <t>13 Nov Dequan hotel Beijing, wake 05:45 for G101 08:00 (~6.5 h)</t>
+        </is>
+      </c>
+      <c r="E8" s="116" t="inlineStr">
+        <is>
+          <t>14 Nov Bestay hotel</t>
+        </is>
+      </c>
+      <c r="F8" s="116" t="inlineStr">
+        <is>
+          <t>Metro 25 min, wake ~06:30</t>
+        </is>
+      </c>
+      <c r="G8" s="121" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H8" s="116" t="inlineStr">
+        <is>
+          <t>Two nights in beds; one early wake two nights before the contest. Cheapest plan with no sleeper before the contest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="66" customHeight="1" s="56">
+      <c r="A9" s="118" t="inlineStr">
+        <is>
+          <t>Shanghai – Sleeper</t>
+        </is>
+      </c>
+      <c r="B9" s="116" t="inlineStr">
+        <is>
+          <t>Sun 6 Dec / Sat 5 Dec</t>
+        </is>
+      </c>
+      <c r="C9" s="116" t="inlineStr">
+        <is>
+          <t>3 Dec Jenny's Apartment (after a 04:30 start for MIAT 07:30; arrive 17:35)</t>
+        </is>
+      </c>
+      <c r="D9" s="116" t="inlineStr">
+        <is>
+          <t>4 Dec Jenny's, free day</t>
+        </is>
+      </c>
+      <c r="E9" s="116" t="inlineStr">
+        <is>
+          <t>5 Dec Jenny's, 1 km</t>
+        </is>
+      </c>
+      <c r="F9" s="116" t="inlineStr">
+        <is>
+          <t>Walk ~15 min, wake ~07:00</t>
+        </is>
+      </c>
+      <c r="G9" s="119" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="H9" s="116" t="inlineStr">
+        <is>
+          <t>D8 is after the contest: now a 2nd-class seat (¥361, sleeper was ¥440). Total ₮7.5M.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="66" customHeight="1" s="56">
+      <c r="A10" s="118" t="inlineStr">
+        <is>
+          <t>Shanghai – Spring nonstop</t>
+        </is>
+      </c>
+      <c r="B10" s="116" t="inlineStr">
+        <is>
+          <t>Sun 6 Dec / Sat 5 Dec</t>
+        </is>
+      </c>
+      <c r="C10" s="116" t="inlineStr">
+        <is>
+          <t>2–3 Dec Jenny's</t>
+        </is>
+      </c>
+      <c r="D10" s="116" t="inlineStr">
+        <is>
+          <t>4 Dec Jenny's</t>
+        </is>
+      </c>
+      <c r="E10" s="116" t="inlineStr">
+        <is>
+          <t>5 Dec Jenny's</t>
+        </is>
+      </c>
+      <c r="F10" s="116" t="inlineStr">
+        <is>
+          <t>Walk ~15 min</t>
+        </is>
+      </c>
+      <c r="G10" s="119" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="H10" s="116" t="inlineStr">
+        <is>
+          <t>Five bed nights before the contest (more than needed). The 08:00 flight on 8 Dec is after the contest, so the 05:00 start does not matter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="66" customHeight="1" s="56">
+      <c r="A11" s="118" t="inlineStr">
+        <is>
+          <t>Shanghai – Train (no sleeper)</t>
+        </is>
+      </c>
+      <c r="B11" s="116" t="inlineStr">
+        <is>
+          <t>Sun 6 Dec / Sat 5 Dec</t>
+        </is>
+      </c>
+      <c r="C11" s="116" t="inlineStr">
+        <is>
+          <t>3 Dec Jenny's</t>
+        </is>
+      </c>
+      <c r="D11" s="116" t="inlineStr">
+        <is>
+          <t>4 Dec Jenny's</t>
+        </is>
+      </c>
+      <c r="E11" s="116" t="inlineStr">
+        <is>
+          <t>5 Dec Jenny's</t>
+        </is>
+      </c>
+      <c r="F11" s="116" t="inlineStr">
+        <is>
+          <t>Walk ~15 min</t>
+        </is>
+      </c>
+      <c r="G11" s="119" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="H11" s="116" t="inlineStr">
+        <is>
+          <t>Identical before the contest; the Beijing hotel night after it costs +0.6M more for nothing – use the sleeper plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="66" customHeight="1" s="56">
+      <c r="A12" s="118" t="inlineStr">
+        <is>
+          <t>Nanchang – Sleeper</t>
+        </is>
+      </c>
+      <c r="B12" s="116" t="inlineStr">
+        <is>
+          <t>Sun 20 Dec / Sat 19 Dec</t>
+        </is>
+      </c>
+      <c r="C12" s="116" t="inlineStr">
+        <is>
+          <t>17 Dec Z111 hard sleeper 23:06–11:52 (~5–6 h, broken)</t>
+        </is>
+      </c>
+      <c r="D12" s="116" t="inlineStr">
+        <is>
+          <t>18 Dec Orange Hotel, arrive 11:52 → nap</t>
+        </is>
+      </c>
+      <c r="E12" s="116" t="inlineStr">
+        <is>
+          <t>19 Dec Orange Hotel, 0.7 km</t>
+        </is>
+      </c>
+      <c r="F12" s="116" t="inlineStr">
+        <is>
+          <t>Walk ~10–15 min, wake ~07:00</t>
+        </is>
+      </c>
+      <c r="G12" s="121" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H12" s="116" t="inlineStr">
+        <is>
+          <t>Two hotel nights sit between the sleeper and the contest. D136 home is after the contest: now a 2nd-class seat (¥271, sleeper was ¥382). Soft sleeper on Z111 (+¥168 pp, ~₮0.3M) is the upgrade. Total ₮6.3M.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="66" customHeight="1" s="56">
+      <c r="A13" s="118" t="inlineStr">
+        <is>
+          <t>Nanchang – Comfort</t>
+        </is>
+      </c>
+      <c r="B13" s="116" t="inlineStr">
+        <is>
+          <t>Sun 20 Dec / Sat 19 Dec</t>
+        </is>
+      </c>
+      <c r="C13" s="116" t="inlineStr">
+        <is>
+          <t>17 Dec Orange Hotel (after a 04:30 start; arrive 17:52)</t>
+        </is>
+      </c>
+      <c r="D13" s="116" t="inlineStr">
+        <is>
+          <t>18 Dec Orange Hotel</t>
+        </is>
+      </c>
+      <c r="E13" s="116" t="inlineStr">
+        <is>
+          <t>19 Dec Orange Hotel</t>
+        </is>
+      </c>
+      <c r="F13" s="116" t="inlineStr">
+        <is>
+          <t>Walk ~10–15 min</t>
+        </is>
+      </c>
+      <c r="G13" s="119" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="H13" s="116" t="inlineStr">
+        <is>
+          <t>Three bed nights; +1.6M vs the sleeper plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="66" customHeight="1" s="56">
+      <c r="A14" s="118" t="inlineStr">
+        <is>
+          <t>Nanchang – Fly in (Air China)</t>
+        </is>
+      </c>
+      <c r="B14" s="116" t="inlineStr">
+        <is>
+          <t>Sun 20 Dec / Sat 19 Dec</t>
+        </is>
+      </c>
+      <c r="C14" s="116" t="inlineStr">
+        <is>
+          <t>17 Dec Orange Hotel (lands 21:40, bed ~23:00)</t>
+        </is>
+      </c>
+      <c r="D14" s="116" t="inlineStr">
+        <is>
+          <t>18 Dec Orange Hotel</t>
+        </is>
+      </c>
+      <c r="E14" s="116" t="inlineStr">
+        <is>
+          <t>19 Dec Orange Hotel</t>
+        </is>
+      </c>
+      <c r="F14" s="116" t="inlineStr">
+        <is>
+          <t>Walk ~10–15 min</t>
+        </is>
+      </c>
+      <c r="G14" s="119" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="H14" s="116" t="inlineStr">
+        <is>
+          <t>No early start at all; +2.1M vs the sleeper plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="66" customHeight="1" s="56">
+      <c r="A15" s="118" t="inlineStr">
+        <is>
+          <t>Hong Kong – Budget</t>
+        </is>
+      </c>
+      <c r="B15" s="116" t="inlineStr">
+        <is>
+          <t>Sun 10 Jan / Sat 9 Jan</t>
+        </is>
+      </c>
+      <c r="C15" s="116" t="inlineStr">
+        <is>
+          <t>7 Jan at home (wake ~04:00 on 8 Jan for MIAT 07:15)</t>
+        </is>
+      </c>
+      <c r="D15" s="116" t="inlineStr">
+        <is>
+          <t>8 Jan Chungking Mansion guesthouse, 3 in one small room</t>
+        </is>
+      </c>
+      <c r="E15" s="116" t="inlineStr">
+        <is>
+          <t>9 Jan same room</t>
+        </is>
+      </c>
+      <c r="F15" s="116" t="inlineStr">
+        <is>
+          <t>MTR ~35 min, wake ~06:15</t>
+        </is>
+      </c>
+      <c r="G15" s="120" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="H15" s="116" t="inlineStr">
+        <is>
+          <t>Cheapest, but small noisy rooms, three people in one room and a long commute are the worst pre-contest sleep of any plan. Use Value or Sleep first for the nights of 8 and 9 Jan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="66" customHeight="1" s="56">
+      <c r="A16" s="118" t="inlineStr">
+        <is>
+          <t>Hong Kong – Comfort</t>
+        </is>
+      </c>
+      <c r="B16" s="116" t="inlineStr">
+        <is>
+          <t>Sun 10 Jan / Sat 9 Jan</t>
+        </is>
+      </c>
+      <c r="C16" s="116" t="inlineStr">
+        <is>
+          <t>7 Jan at home (04:00 start on 8 Jan)</t>
+        </is>
+      </c>
+      <c r="D16" s="116" t="inlineStr">
+        <is>
+          <t>8 Jan Best Western Plus, Sai Ying Pun</t>
+        </is>
+      </c>
+      <c r="E16" s="116" t="inlineStr">
+        <is>
+          <t>9 Jan same</t>
+        </is>
+      </c>
+      <c r="F16" s="116" t="inlineStr">
+        <is>
+          <t>Walk / 1 MTR stop ~10–15 min</t>
+        </is>
+      </c>
+      <c r="G16" s="121" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H16" s="116" t="inlineStr">
+        <is>
+          <t>Close to HKU but rated only 7.4 (4,583 reviews) – read the noise reviews before booking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="66" customHeight="1" s="56">
+      <c r="A17" s="118" t="inlineStr">
+        <is>
+          <t>Hong Kong – Value</t>
+        </is>
+      </c>
+      <c r="B17" s="116" t="inlineStr">
+        <is>
+          <t>Sun 10 Jan / Sat 9 Jan</t>
+        </is>
+      </c>
+      <c r="C17" s="116" t="inlineStr">
+        <is>
+          <t>7 Jan at home (04:00 start)</t>
+        </is>
+      </c>
+      <c r="D17" s="116" t="inlineStr">
+        <is>
+          <t>8 Jan Kusa Inn (9.6, 15 reviews), Kowloon</t>
+        </is>
+      </c>
+      <c r="E17" s="116" t="inlineStr">
+        <is>
+          <t>9 Jan same</t>
+        </is>
+      </c>
+      <c r="F17" s="116" t="inlineStr">
+        <is>
+          <t>MTR ~35 min, wake ~06:15</t>
+        </is>
+      </c>
+      <c r="G17" s="121" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H17" s="116" t="inlineStr">
+        <is>
+          <t>Better-rated room for the same money, but few reviews and the same 35-min commute.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="66" customHeight="1" s="56">
+      <c r="A18" s="118" t="inlineStr">
+        <is>
+          <t>Hong Kong – Sleep first</t>
+        </is>
+      </c>
+      <c r="B18" s="116" t="inlineStr">
+        <is>
+          <t>Sun 10 Jan / Sat 9 Jan</t>
+        </is>
+      </c>
+      <c r="C18" s="116" t="inlineStr">
+        <is>
+          <t>7 Jan at home (04:00 start; arrive 11:50 and nap)</t>
+        </is>
+      </c>
+      <c r="D18" s="116" t="inlineStr">
+        <is>
+          <t>8 Jan iclub AMTD Sheung Wan, 2 rooms</t>
+        </is>
+      </c>
+      <c r="E18" s="116" t="inlineStr">
+        <is>
+          <t>9 Jan same, 2 MTR stops to HKU</t>
+        </is>
+      </c>
+      <c r="F18" s="116" t="inlineStr">
+        <is>
+          <t>MTR ~10–15 min, wake ~07:00</t>
+        </is>
+      </c>
+      <c r="G18" s="119" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+      <c r="H18" s="116" t="inlineStr">
+        <is>
+          <t>Two rooms in an 8.6-rated hotel: ₮2.55M (3 ppl) / ₮2.33M (4 ppl) vs Budget (₮11.63M / ₮14.45M total). Over the ₮12M with the coach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="66" customHeight="1" s="56">
+      <c r="A19" s="118" t="inlineStr">
+        <is>
+          <t>Hong Kong – Funded 12M (funded regional)</t>
+        </is>
+      </c>
+      <c r="B19" s="116" t="inlineStr">
+        <is>
+          <t>Sun 10 Jan / Sat 9 Jan</t>
+        </is>
+      </c>
+      <c r="C19" s="116" t="inlineStr">
+        <is>
+          <t>7 Jan at home (04:00 start; arrive 11:50, nap)</t>
+        </is>
+      </c>
+      <c r="D19" s="116" t="inlineStr">
+        <is>
+          <t>8 Jan Best Western Plus, Sai Ying Pun, 2 rooms (2 beds each)</t>
+        </is>
+      </c>
+      <c r="E19" s="116" t="inlineStr">
+        <is>
+          <t>9 Jan same, ~540 m to HKU</t>
+        </is>
+      </c>
+      <c r="F19" s="116" t="inlineStr">
+        <is>
+          <t>Walk ~10 min, wake ~07:00</t>
+        </is>
+      </c>
+      <c r="G19" s="121" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H19" s="116" t="inlineStr">
+        <is>
+          <t>Fits ₮12M only before the 10% contingency (~₮11.7M). Separate beds and no commute; the hotel is rated 7.4–8.2, so read noise reviews. Cheaper alternative with separate beds: Good Fortune Inn (8.6, 4 twin beds) but ~35 min MTR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="78" customHeight="1" s="56">
+      <c r="A20" s="118" t="inlineStr">
+        <is>
+          <t>Hong Kong – Sleep priority (funded regional)</t>
+        </is>
+      </c>
+      <c r="B20" s="116" t="inlineStr">
+        <is>
+          <t>Sun 10 Jan / Sat 9 Jan</t>
+        </is>
+      </c>
+      <c r="C20" s="116" t="inlineStr">
+        <is>
+          <t>7 Jan at home (04:00 start; arrive 11:50, nap)</t>
+        </is>
+      </c>
+      <c r="D20" s="116" t="inlineStr">
+        <is>
+          <t>8 Jan Good Fortune Inn: 2 rooms, 4 twin beds, private bathrooms</t>
+        </is>
+      </c>
+      <c r="E20" s="116" t="inlineStr">
+        <is>
+          <t>9 Jan same</t>
+        </is>
+      </c>
+      <c r="F20" s="116" t="inlineStr">
+        <is>
+          <t>MTR ~35–40 min, wake ~06:15 (lights out 22:30 = 7.75 h)</t>
+        </is>
+      </c>
+      <c r="G20" s="121" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H20" s="116" t="inlineStr">
+        <is>
+          <t>Best bed arrangement under the ₮12M cap (everyone has their own bed and bathroom, 8.6 from 715 reviews) at ~₮11.3M before contingency; costs ~35 min of sleep a day in commute versus the BW Plus walk. Better still if the host campus turns out to be near Kowloon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="66" customHeight="1" s="56">
+      <c r="A21" s="118" t="inlineStr">
+        <is>
+          <t>EC Final – Train</t>
+        </is>
+      </c>
+      <c r="B21" s="116" t="inlineStr">
+        <is>
+          <t>Wed 27 Jan / Tue 26 Jan</t>
+        </is>
+      </c>
+      <c r="C21" s="116" t="inlineStr">
+        <is>
+          <t>24 Jan at home</t>
+        </is>
+      </c>
+      <c r="D21" s="116" t="inlineStr">
+        <is>
+          <t>25 Jan D17 2nd-class sleeper 19:10–09:15 (4-berth cabin, ~6 h) → arrive on day 1</t>
+        </is>
+      </c>
+      <c r="E21" s="116" t="inlineStr">
+        <is>
+          <t>26 Jan HanTing, 1.6 km</t>
+        </is>
+      </c>
+      <c r="F21" s="116" t="inlineStr">
+        <is>
+          <t>Walk ~20 min, wake ~07:00</t>
+        </is>
+      </c>
+      <c r="G21" s="120" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="H21" s="116" t="inlineStr">
+        <is>
+          <t>The sleeper is the night before the check-in / warm-up day (not the contest day), with a hotel night in between. Safer: leave Beijing 24 Jan (one more hotel night, ~₮0.35M) or take the afternoon G-train + hotel (old plan, ~+₮0.44M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="66" customHeight="1" s="56">
+      <c r="A22" s="118" t="inlineStr">
+        <is>
+          <t>EC Final – Fly</t>
+        </is>
+      </c>
+      <c r="B22" s="116" t="inlineStr">
+        <is>
+          <t>Wed 27 Jan / Tue 26 Jan</t>
+        </is>
+      </c>
+      <c r="C22" s="116" t="inlineStr">
+        <is>
+          <t>24 Jan at home (wake ~03:30 on 25 Jan for Aero Mongolia 06:30)</t>
+        </is>
+      </c>
+      <c r="D22" s="116" t="inlineStr">
+        <is>
+          <t>25 Jan Mehood Theater Hotel (arrive ~13:40; nap)</t>
+        </is>
+      </c>
+      <c r="E22" s="116" t="inlineStr">
+        <is>
+          <t>26 Jan same, 1.7 km</t>
+        </is>
+      </c>
+      <c r="F22" s="116" t="inlineStr">
+        <is>
+          <t>Walk ~20 min</t>
+        </is>
+      </c>
+      <c r="G22" s="121" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H22" s="116" t="inlineStr">
+        <is>
+          <t>Early start two nights before; arrives early afternoon, then two hotel nights.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="66" customHeight="1" s="56">
+      <c r="A23" s="118" t="inlineStr">
+        <is>
+          <t>Nanjing + Shenyang (older workbook A / B)</t>
+        </is>
+      </c>
+      <c r="B23" s="116" t="inlineStr">
+        <is>
+          <t>Nanjing Sun 8 Nov; Shenyang Sun 15 Nov</t>
+        </is>
+      </c>
+      <c r="C23" s="116" t="inlineStr">
+        <is>
+          <t>6 Nov Beijing hotel after MIAT lands 19:30, wake ~06:00 for the G-train</t>
+        </is>
+      </c>
+      <c r="D23" s="116" t="inlineStr">
+        <is>
+          <t>7 Nov Nanjing hotel (A 1 km, B 15 min metro)</t>
+        </is>
+      </c>
+      <c r="E23" s="116" t="inlineStr">
+        <is>
+          <t>Shenyang: Z366 sleeper 12 Nov → hotels 13 and 14 Nov</t>
+        </is>
+      </c>
+      <c r="F23" s="116" t="inlineStr">
+        <is>
+          <t>Nanjing walk / Shenyang walk</t>
+        </is>
+      </c>
+      <c r="G23" s="121" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H23" s="116" t="inlineStr">
+        <is>
+          <t>K54 home after the Shenyang contest is now a hard sleeper (soft was ¥263). Plan C (home between) uses K53 soft sleeper on 13 Nov = night before day 1 (WATCH).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" s="56">
+      <c r="A24" s="55" t="inlineStr">
+        <is>
+          <t>One regional is funded with ₮12M (coach travels, 4 people); the other is unfunded (3 contestants pay). The funded trip has little headroom (Hong Kong does not fit), and the unfunded trip pays for every hotel night, so protect sleep with timing and location first: arrive a day early only where it is cheap (Shenyang, Nanchang), pick the hotel closest to the venue, and take the cheap-but-bad options only after the contest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" s="56">
+      <c r="A25" s="122" t="inlineStr">
+        <is>
+          <t>Where the money goes (use the headroom on sleep)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="36" customHeight="1" s="56">
+      <c r="A26" s="116" t="inlineStr">
+        <is>
+          <t>One regional is funded with ₮12M (coach travels, 4 people); the other is unfunded (3 contestants pay). The funded trip has little headroom (Hong Kong does not fit), and the unfunded trip pays for every hotel night, so protect sleep with timing and location first: arrive a day early only where it is cheap (Shenyang, Nanchang), pick the hotel closest to the venue, and take the cheap-but-bad options only after the contest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="36" customHeight="1" s="56">
+      <c r="A27" s="116" t="inlineStr">
+        <is>
+          <t>Pre-contest upgrades applied: Shenyang Budget K53 hard → soft; Hong Kong Sleep first (2 rooms near HKU). Post-contest downgrades applied: Shenyang K54 soft → hard, Shanghai D8 sleeper → seat, Nanchang D136 sleeper → seat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="36" customHeight="1" s="56">
+      <c r="A28" s="116" t="inlineStr">
+        <is>
+          <t>Cheapest post-contest options if you want to go further: Nanchang Z182 20:01 → 08:46 hard seat (¥173.5 vs ¥271); Shanghai G808 17:25 is too early after the awards, so the D8 seat stays.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="36" customHeight="1" s="56">
+      <c r="A29" s="116" t="inlineStr">
+        <is>
+          <t>Contest-day wake-up rule of thumb: bed by 22:30–23:00, up by 06:00–06:30 for a 09:00 start; avoid alcohol and late team dinners; no phone-based all-nighters on day 1.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A27:H27"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17192,885 +19528,6 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" style="56" min="1" max="1"/>
-    <col width="22" customWidth="1" style="56" min="2" max="2"/>
-    <col width="32" customWidth="1" style="56" min="3" max="3"/>
-    <col width="34" customWidth="1" style="56" min="4" max="4"/>
-    <col width="30" customWidth="1" style="56" min="5" max="5"/>
-    <col width="22" customWidth="1" style="56" min="6" max="6"/>
-    <col width="10" customWidth="1" style="56" min="7" max="7"/>
-    <col width="70" customWidth="1" style="56" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="115" t="inlineStr">
-        <is>
-          <t>Sleep check – protect the nights before the contest, spend nothing on comfort after it</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="78" customHeight="1" s="56">
-      <c r="A2" s="116" t="inlineStr">
-        <is>
-          <t>Rules used: (1) the two nights before the contest day are in a real bed, quiet, ≤30 min from the venue, ≥7.5 h in bed and no wake-up before ~06:00 on contest morning; (2) no overnight train or flight on the contest eve; a sleeper before day 1 only if it is a soft sleeper that arrives by midday and there is a bed night in between; (3) flights before 08:00 only ≥2 nights before the contest; (4) after the contest anything goes – hard sleepers, seats, red-eye trains, 04:30 airport runs – so the cheapest option is used. No time-zone effect: Mongolia, China and Hong Kong are all UTC+8.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="117" t="inlineStr">
-        <is>
-          <t>Plan</t>
-        </is>
-      </c>
-      <c r="B4" s="117" t="inlineStr">
-        <is>
-          <t>Contest day / day 1</t>
-        </is>
-      </c>
-      <c r="C4" s="117" t="inlineStr">
-        <is>
-          <t>Night −3</t>
-        </is>
-      </c>
-      <c r="D4" s="117" t="inlineStr">
-        <is>
-          <t>Night −2 (before day 1)</t>
-        </is>
-      </c>
-      <c r="E4" s="117" t="inlineStr">
-        <is>
-          <t>Night −1 (contest eve)</t>
-        </is>
-      </c>
-      <c r="F4" s="117" t="inlineStr">
-        <is>
-          <t>Contest morning</t>
-        </is>
-      </c>
-      <c r="G4" s="117" t="inlineStr">
-        <is>
-          <t>Verdict</t>
-        </is>
-      </c>
-      <c r="H4" s="117" t="inlineStr">
-        <is>
-          <t>Sleep fix / what changed</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="66" customHeight="1" s="56">
-      <c r="A5" s="118" t="inlineStr">
-        <is>
-          <t>Shenyang – Comfort</t>
-        </is>
-      </c>
-      <c r="B5" s="116" t="inlineStr">
-        <is>
-          <t>Sun 15 Nov / Sat 14 Nov</t>
-        </is>
-      </c>
-      <c r="C5" s="116" t="inlineStr">
-        <is>
-          <t>12 Nov RiCH hotel (after a 04:30 start for MIAT 07:30; nap in the afternoon)</t>
-        </is>
-      </c>
-      <c r="D5" s="116" t="inlineStr">
-        <is>
-          <t>13 Nov RiCH, free rest day</t>
-        </is>
-      </c>
-      <c r="E5" s="116" t="inlineStr">
-        <is>
-          <t>14 Nov RiCH, family room, quiet</t>
-        </is>
-      </c>
-      <c r="F5" s="116" t="inlineStr">
-        <is>
-          <t>Walk 18 min, wake ~07:00</t>
-        </is>
-      </c>
-      <c r="G5" s="119" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="H5" s="116" t="inlineStr">
-        <is>
-          <t>Sleeper K54 is after the contest, so it is now a hard sleeper (soft was ¥263): saves ~₮0.16M (₮6.2M total).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="66" customHeight="1" s="56">
-      <c r="A6" s="118" t="inlineStr">
-        <is>
-          <t>Shenyang – Budget</t>
-        </is>
-      </c>
-      <c r="B6" s="116" t="inlineStr">
-        <is>
-          <t>Sun 15 Nov / Sat 14 Nov</t>
-        </is>
-      </c>
-      <c r="C6" s="116" t="inlineStr">
-        <is>
-          <t>12 Nov at home</t>
-        </is>
-      </c>
-      <c r="D6" s="116" t="inlineStr">
-        <is>
-          <t>13 Nov K53 soft sleeper 22:35–07:00 (was hard): ~5–6 h, then day-1 registration</t>
-        </is>
-      </c>
-      <c r="E6" s="116" t="inlineStr">
-        <is>
-          <t>14 Nov Bestay hotel (8.2, budget chain)</t>
-        </is>
-      </c>
-      <c r="F6" s="116" t="inlineStr">
-        <is>
-          <t>Metro 25 min, wake ~06:30</t>
-        </is>
-      </c>
-      <c r="G6" s="120" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
-      <c r="H6" s="116" t="inlineStr">
-        <is>
-          <t>K53 is the night before day 1, so it is now a soft sleeper (+¥92 pp, +₮0.16M; ₮5.2M total). Nap on arrival; the contest eve is in a bed. Safer: Comfort or either G-train variant.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="66" customHeight="1" s="56">
-      <c r="A7" s="118" t="inlineStr">
-        <is>
-          <t>Shenyang – Comfort (G-train)</t>
-        </is>
-      </c>
-      <c r="B7" s="116" t="inlineStr">
-        <is>
-          <t>Sun 15 Nov / Sat 14 Nov</t>
-        </is>
-      </c>
-      <c r="C7" s="116" t="inlineStr">
-        <is>
-          <t>12 Nov RiCH hotel</t>
-        </is>
-      </c>
-      <c r="D7" s="116" t="inlineStr">
-        <is>
-          <t>13 Nov RiCH</t>
-        </is>
-      </c>
-      <c r="E7" s="116" t="inlineStr">
-        <is>
-          <t>14 Nov RiCH</t>
-        </is>
-      </c>
-      <c r="F7" s="116" t="inlineStr">
-        <is>
-          <t>Walk 18 min, wake ~07:00</t>
-        </is>
-      </c>
-      <c r="G7" s="119" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="H7" s="116" t="inlineStr">
-        <is>
-          <t>All beds before the contest; the Beijing hotel night (Dequan) is after it. +0.5M vs the sleeper plan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="66" customHeight="1" s="56">
-      <c r="A8" s="118" t="inlineStr">
-        <is>
-          <t>Shenyang – Budget (G-train)</t>
-        </is>
-      </c>
-      <c r="B8" s="116" t="inlineStr">
-        <is>
-          <t>Sun 15 Nov / Sat 14 Nov</t>
-        </is>
-      </c>
-      <c r="C8" s="116" t="inlineStr">
-        <is>
-          <t>12 Nov at home</t>
-        </is>
-      </c>
-      <c r="D8" s="116" t="inlineStr">
-        <is>
-          <t>13 Nov Dequan hotel Beijing, wake 05:45 for G101 08:00 (~6.5 h)</t>
-        </is>
-      </c>
-      <c r="E8" s="116" t="inlineStr">
-        <is>
-          <t>14 Nov Bestay hotel</t>
-        </is>
-      </c>
-      <c r="F8" s="116" t="inlineStr">
-        <is>
-          <t>Metro 25 min, wake ~06:30</t>
-        </is>
-      </c>
-      <c r="G8" s="121" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H8" s="116" t="inlineStr">
-        <is>
-          <t>Two nights in beds; one early wake two nights before the contest. Cheapest plan with no sleeper before the contest.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="66" customHeight="1" s="56">
-      <c r="A9" s="118" t="inlineStr">
-        <is>
-          <t>Shanghai – Sleeper</t>
-        </is>
-      </c>
-      <c r="B9" s="116" t="inlineStr">
-        <is>
-          <t>Sun 6 Dec / Sat 5 Dec</t>
-        </is>
-      </c>
-      <c r="C9" s="116" t="inlineStr">
-        <is>
-          <t>3 Dec Jenny's Apartment (after a 04:30 start for MIAT 07:30; arrive 17:35)</t>
-        </is>
-      </c>
-      <c r="D9" s="116" t="inlineStr">
-        <is>
-          <t>4 Dec Jenny's, free day</t>
-        </is>
-      </c>
-      <c r="E9" s="116" t="inlineStr">
-        <is>
-          <t>5 Dec Jenny's, 1 km</t>
-        </is>
-      </c>
-      <c r="F9" s="116" t="inlineStr">
-        <is>
-          <t>Walk ~15 min, wake ~07:00</t>
-        </is>
-      </c>
-      <c r="G9" s="119" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="H9" s="116" t="inlineStr">
-        <is>
-          <t>D8 is after the contest: now a 2nd-class seat (¥361, sleeper was ¥440). Total ₮7.5M.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="66" customHeight="1" s="56">
-      <c r="A10" s="118" t="inlineStr">
-        <is>
-          <t>Shanghai – Spring nonstop</t>
-        </is>
-      </c>
-      <c r="B10" s="116" t="inlineStr">
-        <is>
-          <t>Sun 6 Dec / Sat 5 Dec</t>
-        </is>
-      </c>
-      <c r="C10" s="116" t="inlineStr">
-        <is>
-          <t>2–3 Dec Jenny's</t>
-        </is>
-      </c>
-      <c r="D10" s="116" t="inlineStr">
-        <is>
-          <t>4 Dec Jenny's</t>
-        </is>
-      </c>
-      <c r="E10" s="116" t="inlineStr">
-        <is>
-          <t>5 Dec Jenny's</t>
-        </is>
-      </c>
-      <c r="F10" s="116" t="inlineStr">
-        <is>
-          <t>Walk ~15 min</t>
-        </is>
-      </c>
-      <c r="G10" s="119" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="H10" s="116" t="inlineStr">
-        <is>
-          <t>Five bed nights before the contest (more than needed). The 08:00 flight on 8 Dec is after the contest, so the 05:00 start does not matter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="66" customHeight="1" s="56">
-      <c r="A11" s="118" t="inlineStr">
-        <is>
-          <t>Shanghai – Train (no sleeper)</t>
-        </is>
-      </c>
-      <c r="B11" s="116" t="inlineStr">
-        <is>
-          <t>Sun 6 Dec / Sat 5 Dec</t>
-        </is>
-      </c>
-      <c r="C11" s="116" t="inlineStr">
-        <is>
-          <t>3 Dec Jenny's</t>
-        </is>
-      </c>
-      <c r="D11" s="116" t="inlineStr">
-        <is>
-          <t>4 Dec Jenny's</t>
-        </is>
-      </c>
-      <c r="E11" s="116" t="inlineStr">
-        <is>
-          <t>5 Dec Jenny's</t>
-        </is>
-      </c>
-      <c r="F11" s="116" t="inlineStr">
-        <is>
-          <t>Walk ~15 min</t>
-        </is>
-      </c>
-      <c r="G11" s="119" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="H11" s="116" t="inlineStr">
-        <is>
-          <t>Identical before the contest; the Beijing hotel night after it costs +0.6M more for nothing – use the sleeper plan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="66" customHeight="1" s="56">
-      <c r="A12" s="118" t="inlineStr">
-        <is>
-          <t>Nanchang – Sleeper</t>
-        </is>
-      </c>
-      <c r="B12" s="116" t="inlineStr">
-        <is>
-          <t>Sun 20 Dec / Sat 19 Dec</t>
-        </is>
-      </c>
-      <c r="C12" s="116" t="inlineStr">
-        <is>
-          <t>17 Dec Z111 hard sleeper 23:06–11:52 (~5–6 h, broken)</t>
-        </is>
-      </c>
-      <c r="D12" s="116" t="inlineStr">
-        <is>
-          <t>18 Dec Orange Hotel, arrive 11:52 → nap</t>
-        </is>
-      </c>
-      <c r="E12" s="116" t="inlineStr">
-        <is>
-          <t>19 Dec Orange Hotel, 0.7 km</t>
-        </is>
-      </c>
-      <c r="F12" s="116" t="inlineStr">
-        <is>
-          <t>Walk ~10–15 min, wake ~07:00</t>
-        </is>
-      </c>
-      <c r="G12" s="121" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H12" s="116" t="inlineStr">
-        <is>
-          <t>Two hotel nights sit between the sleeper and the contest. D136 home is after the contest: now a 2nd-class seat (¥271, sleeper was ¥382). Soft sleeper on Z111 (+¥168 pp, ~₮0.3M) is the upgrade. Total ₮6.3M.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="66" customHeight="1" s="56">
-      <c r="A13" s="118" t="inlineStr">
-        <is>
-          <t>Nanchang – Comfort</t>
-        </is>
-      </c>
-      <c r="B13" s="116" t="inlineStr">
-        <is>
-          <t>Sun 20 Dec / Sat 19 Dec</t>
-        </is>
-      </c>
-      <c r="C13" s="116" t="inlineStr">
-        <is>
-          <t>17 Dec Orange Hotel (after a 04:30 start; arrive 17:52)</t>
-        </is>
-      </c>
-      <c r="D13" s="116" t="inlineStr">
-        <is>
-          <t>18 Dec Orange Hotel</t>
-        </is>
-      </c>
-      <c r="E13" s="116" t="inlineStr">
-        <is>
-          <t>19 Dec Orange Hotel</t>
-        </is>
-      </c>
-      <c r="F13" s="116" t="inlineStr">
-        <is>
-          <t>Walk ~10–15 min</t>
-        </is>
-      </c>
-      <c r="G13" s="119" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="H13" s="116" t="inlineStr">
-        <is>
-          <t>Three bed nights; +1.6M vs the sleeper plan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="66" customHeight="1" s="56">
-      <c r="A14" s="118" t="inlineStr">
-        <is>
-          <t>Nanchang – Fly in (Air China)</t>
-        </is>
-      </c>
-      <c r="B14" s="116" t="inlineStr">
-        <is>
-          <t>Sun 20 Dec / Sat 19 Dec</t>
-        </is>
-      </c>
-      <c r="C14" s="116" t="inlineStr">
-        <is>
-          <t>17 Dec Orange Hotel (lands 21:40, bed ~23:00)</t>
-        </is>
-      </c>
-      <c r="D14" s="116" t="inlineStr">
-        <is>
-          <t>18 Dec Orange Hotel</t>
-        </is>
-      </c>
-      <c r="E14" s="116" t="inlineStr">
-        <is>
-          <t>19 Dec Orange Hotel</t>
-        </is>
-      </c>
-      <c r="F14" s="116" t="inlineStr">
-        <is>
-          <t>Walk ~10–15 min</t>
-        </is>
-      </c>
-      <c r="G14" s="119" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="H14" s="116" t="inlineStr">
-        <is>
-          <t>No early start at all; +2.1M vs the sleeper plan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="66" customHeight="1" s="56">
-      <c r="A15" s="118" t="inlineStr">
-        <is>
-          <t>Hong Kong – Budget</t>
-        </is>
-      </c>
-      <c r="B15" s="116" t="inlineStr">
-        <is>
-          <t>Sun 10 Jan / Sat 9 Jan</t>
-        </is>
-      </c>
-      <c r="C15" s="116" t="inlineStr">
-        <is>
-          <t>7 Jan at home (wake ~04:00 on 8 Jan for MIAT 07:15)</t>
-        </is>
-      </c>
-      <c r="D15" s="116" t="inlineStr">
-        <is>
-          <t>8 Jan Chungking Mansion guesthouse, 3 in one small room</t>
-        </is>
-      </c>
-      <c r="E15" s="116" t="inlineStr">
-        <is>
-          <t>9 Jan same room</t>
-        </is>
-      </c>
-      <c r="F15" s="116" t="inlineStr">
-        <is>
-          <t>MTR ~35 min, wake ~06:15</t>
-        </is>
-      </c>
-      <c r="G15" s="120" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
-      <c r="H15" s="116" t="inlineStr">
-        <is>
-          <t>Cheapest, but small noisy rooms, three people in one room and a long commute are the worst pre-contest sleep of any plan. Use Value or Sleep first for the nights of 8 and 9 Jan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="66" customHeight="1" s="56">
-      <c r="A16" s="118" t="inlineStr">
-        <is>
-          <t>Hong Kong – Comfort</t>
-        </is>
-      </c>
-      <c r="B16" s="116" t="inlineStr">
-        <is>
-          <t>Sun 10 Jan / Sat 9 Jan</t>
-        </is>
-      </c>
-      <c r="C16" s="116" t="inlineStr">
-        <is>
-          <t>7 Jan at home (04:00 start on 8 Jan)</t>
-        </is>
-      </c>
-      <c r="D16" s="116" t="inlineStr">
-        <is>
-          <t>8 Jan Best Western Plus, Sai Ying Pun</t>
-        </is>
-      </c>
-      <c r="E16" s="116" t="inlineStr">
-        <is>
-          <t>9 Jan same</t>
-        </is>
-      </c>
-      <c r="F16" s="116" t="inlineStr">
-        <is>
-          <t>Walk / 1 MTR stop ~10–15 min</t>
-        </is>
-      </c>
-      <c r="G16" s="121" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H16" s="116" t="inlineStr">
-        <is>
-          <t>Close to HKU but rated only 7.4 (4,583 reviews) – read the noise reviews before booking.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="66" customHeight="1" s="56">
-      <c r="A17" s="118" t="inlineStr">
-        <is>
-          <t>Hong Kong – Value</t>
-        </is>
-      </c>
-      <c r="B17" s="116" t="inlineStr">
-        <is>
-          <t>Sun 10 Jan / Sat 9 Jan</t>
-        </is>
-      </c>
-      <c r="C17" s="116" t="inlineStr">
-        <is>
-          <t>7 Jan at home (04:00 start)</t>
-        </is>
-      </c>
-      <c r="D17" s="116" t="inlineStr">
-        <is>
-          <t>8 Jan Kusa Inn (9.6, 15 reviews), Kowloon</t>
-        </is>
-      </c>
-      <c r="E17" s="116" t="inlineStr">
-        <is>
-          <t>9 Jan same</t>
-        </is>
-      </c>
-      <c r="F17" s="116" t="inlineStr">
-        <is>
-          <t>MTR ~35 min, wake ~06:15</t>
-        </is>
-      </c>
-      <c r="G17" s="121" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H17" s="116" t="inlineStr">
-        <is>
-          <t>Better-rated room for the same money, but few reviews and the same 35-min commute.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="66" customHeight="1" s="56">
-      <c r="A18" s="118" t="inlineStr">
-        <is>
-          <t>Hong Kong – Sleep first</t>
-        </is>
-      </c>
-      <c r="B18" s="116" t="inlineStr">
-        <is>
-          <t>Sun 10 Jan / Sat 9 Jan</t>
-        </is>
-      </c>
-      <c r="C18" s="116" t="inlineStr">
-        <is>
-          <t>7 Jan at home (04:00 start; arrive 11:50 and nap)</t>
-        </is>
-      </c>
-      <c r="D18" s="116" t="inlineStr">
-        <is>
-          <t>8 Jan iclub AMTD Sheung Wan, 2 rooms</t>
-        </is>
-      </c>
-      <c r="E18" s="116" t="inlineStr">
-        <is>
-          <t>9 Jan same, 2 MTR stops to HKU</t>
-        </is>
-      </c>
-      <c r="F18" s="116" t="inlineStr">
-        <is>
-          <t>MTR ~10–15 min, wake ~07:00</t>
-        </is>
-      </c>
-      <c r="G18" s="119" t="inlineStr">
-        <is>
-          <t>BEST</t>
-        </is>
-      </c>
-      <c r="H18" s="116" t="inlineStr">
-        <is>
-          <t>Two rooms in an 8.6-rated hotel: ₮2.55M (3 ppl) / ₮2.33M (4 ppl) vs Budget (₮11.63M / ₮14.45M total). Over the ₮12M with the coach.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="66" customHeight="1" s="56">
-      <c r="A19" s="118" t="inlineStr">
-        <is>
-          <t>Hong Kong – Funded 12M (funded regional)</t>
-        </is>
-      </c>
-      <c r="B19" s="116" t="inlineStr">
-        <is>
-          <t>Sun 10 Jan / Sat 9 Jan</t>
-        </is>
-      </c>
-      <c r="C19" s="116" t="inlineStr">
-        <is>
-          <t>7 Jan at home (04:00 start; arrive 11:50, nap)</t>
-        </is>
-      </c>
-      <c r="D19" s="116" t="inlineStr">
-        <is>
-          <t>8 Jan Best Western Plus, Sai Ying Pun, 2 rooms (2 beds each)</t>
-        </is>
-      </c>
-      <c r="E19" s="116" t="inlineStr">
-        <is>
-          <t>9 Jan same, ~540 m to HKU</t>
-        </is>
-      </c>
-      <c r="F19" s="116" t="inlineStr">
-        <is>
-          <t>Walk ~10 min, wake ~07:00</t>
-        </is>
-      </c>
-      <c r="G19" s="121" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H19" s="116" t="inlineStr">
-        <is>
-          <t>Fits ₮12M only before the 10% contingency (~₮11.7M). Separate beds and no commute; the hotel is rated 7.4–8.2, so read noise reviews. Cheaper alternative with separate beds: Good Fortune Inn (8.6, 4 twin beds) but ~35 min MTR.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="66" customHeight="1" s="56">
-      <c r="A20" s="118" t="inlineStr">
-        <is>
-          <t>EC Final – Train</t>
-        </is>
-      </c>
-      <c r="B20" s="116" t="inlineStr">
-        <is>
-          <t>Wed 27 Jan / Tue 26 Jan</t>
-        </is>
-      </c>
-      <c r="C20" s="116" t="inlineStr">
-        <is>
-          <t>24 Jan at home</t>
-        </is>
-      </c>
-      <c r="D20" s="116" t="inlineStr">
-        <is>
-          <t>25 Jan D17 2nd-class sleeper 19:10–09:15 (4-berth cabin, ~6 h) → arrive on day 1</t>
-        </is>
-      </c>
-      <c r="E20" s="116" t="inlineStr">
-        <is>
-          <t>26 Jan HanTing, 1.6 km</t>
-        </is>
-      </c>
-      <c r="F20" s="116" t="inlineStr">
-        <is>
-          <t>Walk ~20 min, wake ~07:00</t>
-        </is>
-      </c>
-      <c r="G20" s="120" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
-      <c r="H20" s="116" t="inlineStr">
-        <is>
-          <t>The sleeper is the night before the check-in / warm-up day (not the contest day), with a hotel night in between. Safer: leave Beijing 24 Jan (one more hotel night, ~₮0.35M) or take the afternoon G-train + hotel (old plan, ~+₮0.44M).</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="66" customHeight="1" s="56">
-      <c r="A21" s="118" t="inlineStr">
-        <is>
-          <t>EC Final – Fly</t>
-        </is>
-      </c>
-      <c r="B21" s="116" t="inlineStr">
-        <is>
-          <t>Wed 27 Jan / Tue 26 Jan</t>
-        </is>
-      </c>
-      <c r="C21" s="116" t="inlineStr">
-        <is>
-          <t>24 Jan at home (wake ~03:30 on 25 Jan for Aero Mongolia 06:30)</t>
-        </is>
-      </c>
-      <c r="D21" s="116" t="inlineStr">
-        <is>
-          <t>25 Jan Mehood Theater Hotel (arrive ~13:40; nap)</t>
-        </is>
-      </c>
-      <c r="E21" s="116" t="inlineStr">
-        <is>
-          <t>26 Jan same, 1.7 km</t>
-        </is>
-      </c>
-      <c r="F21" s="116" t="inlineStr">
-        <is>
-          <t>Walk ~20 min</t>
-        </is>
-      </c>
-      <c r="G21" s="121" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H21" s="116" t="inlineStr">
-        <is>
-          <t>Early start two nights before; arrives early afternoon, then two hotel nights.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="66" customHeight="1" s="56">
-      <c r="A22" s="118" t="inlineStr">
-        <is>
-          <t>Nanjing + Shenyang (older workbook A / B)</t>
-        </is>
-      </c>
-      <c r="B22" s="116" t="inlineStr">
-        <is>
-          <t>Nanjing Sun 8 Nov; Shenyang Sun 15 Nov</t>
-        </is>
-      </c>
-      <c r="C22" s="116" t="inlineStr">
-        <is>
-          <t>6 Nov Beijing hotel after MIAT lands 19:30, wake ~06:00 for the G-train</t>
-        </is>
-      </c>
-      <c r="D22" s="116" t="inlineStr">
-        <is>
-          <t>7 Nov Nanjing hotel (A 1 km, B 15 min metro)</t>
-        </is>
-      </c>
-      <c r="E22" s="116" t="inlineStr">
-        <is>
-          <t>Shenyang: Z366 sleeper 12 Nov → hotels 13 and 14 Nov</t>
-        </is>
-      </c>
-      <c r="F22" s="116" t="inlineStr">
-        <is>
-          <t>Nanjing walk / Shenyang walk</t>
-        </is>
-      </c>
-      <c r="G22" s="121" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H22" s="116" t="inlineStr">
-        <is>
-          <t>K54 home after the Shenyang contest is now a hard sleeper (soft was ¥263). Plan C (home between) uses K53 soft sleeper on 13 Nov = night before day 1 (WATCH).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" s="56"/>
-    <row r="24" s="56">
-      <c r="A24" s="122" t="inlineStr">
-        <is>
-          <t>Where the money goes (use the headroom on sleep)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="36" customHeight="1" s="56">
-      <c r="A25" s="116" t="inlineStr">
-        <is>
-          <t>One regional is funded with ₮12M (coach travels, 4 people); the other is unfunded (3 contestants pay). The funded trip has little headroom (Hong Kong does not fit), and the unfunded trip pays for every hotel night, so protect sleep with timing and location first: arrive a day early only where it is cheap (Shenyang, Nanchang), pick the hotel closest to the venue, and take the cheap-but-bad options only after the contest.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="36" customHeight="1" s="56">
-      <c r="A26" s="116" t="inlineStr">
-        <is>
-          <t>Pre-contest upgrades applied: Shenyang Budget K53 hard → soft; Hong Kong Sleep first (2 rooms near HKU). Post-contest downgrades applied: Shenyang K54 soft → hard, Shanghai D8 sleeper → seat, Nanchang D136 sleeper → seat.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="36" customHeight="1" s="56">
-      <c r="A27" s="116" t="inlineStr">
-        <is>
-          <t>Cheapest post-contest options if you want to go further: Nanchang Z182 20:01 → 08:46 hard seat (¥173.5 vs ¥271); Shanghai G808 17:25 is too early after the awards, so the D8 seat stays.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="36" customHeight="1" s="56">
-      <c r="A28" s="116" t="inlineStr">
-        <is>
-          <t>Contest-day wake-up rule of thumb: bed by 22:30–23:00, up by 06:00–06:30 for a 09:00 start; avoid alcohol and late team dinners; no phone-based all-nighters on day 1.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A26:H26"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A28:H28"/>
-    <mergeCell ref="A27:H27"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Shenyang: cross-check UB → Shenyang on Ctrip, Kiwi, Google Flights, 12go
Ctrip has Air China CA902 11:50 at ¥1,291 (Trip.com $203, Kiwi $200), so the
three sleep-first plans now budget it there (−₮38k per person). Trains match
12306. Via-Hohhot and through-ticket UB → Shenyang flights are no better.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ICPC_Single_Contest_Plans.xlsx
+++ b/ICPC_Single_Contest_Plans.xlsx
@@ -2408,7 +2408,7 @@
       </c>
       <c r="B40" s="74" t="inlineStr">
         <is>
-          <t>Funded = Hong Kong (₮12M, coach): lead with 'Hong Kong – Sleep priority' – MIAT nonstop, 2 rooms with 4 separate twin beds and private bathrooms at Good Fortune Inn (8.6, 715 reviews, ~35–40 min MTR to HKU), airport bus: ₮11.33M before the 10% contingency (₮0.67M spare), ₮12.47M with it. Walking alternative: 'Funded 12M' (Best Western Plus, ~540 m to HKU) ₮11.70M before contingency (₮0.30M spare). Unfunded = Shenyang, sleep first and cheap after: 'Shenyang – Sleep value' ₮2.73M per person (no early start, a bed each, home 16 Nov) or 'Shenyang – Overland home' ₮2.41M per person (same before the contest, night trains home via Erenhot, home 18 Nov); Budget ₮2.14M per person is cheaper but puts a sleeper the night before day 1. The HK 2026 host may not be HKU (2025 was HKUST), which favours sleeping well and staying on the MTR over a hotel next to one campus.</t>
+          <t>Funded = Hong Kong (₮12M, coach): lead with 'Hong Kong – Sleep priority' – MIAT nonstop, 2 rooms with 4 separate twin beds and private bathrooms at Good Fortune Inn (8.6, 715 reviews, ~35–40 min MTR to HKU), airport bus: ₮11.33M before the 10% contingency (₮0.67M spare), ₮12.47M with it. Walking alternative: 'Funded 12M' (Best Western Plus, ~540 m to HKU) ₮11.70M before contingency (₮0.30M spare). Unfunded = Shenyang, sleep first and cheap after: 'Shenyang – Sleep value' ₮2.69M per person (no early start, a bed each, home 16 Nov) or 'Shenyang – Overland home' ₮2.37M per person (same before the contest, night trains home via Erenhot, home 18 Nov); Budget ₮2.14M per person is cheaper but puts a sleeper the night before day 1. The HK 2026 host may not be HKU (2025 was HKUST), which favours sleeping well and staying on the MTR over a hotel next to one campus.</t>
         </is>
       </c>
     </row>
@@ -2420,7 +2420,7 @@
       </c>
       <c r="B41" s="74" t="inlineStr">
         <is>
-          <t>Cheapest sleep-safe plans per person incl. fee, taxi, insurance, eSIM and 10% contingency: Shenyang – Budget ₮2.14M per person (soft sleeper before day 1); Shenyang – Overland home ₮2.41M per person (no early start, a bed each, overland home); Shenyang – Comfort ₮2.46M per person; Nanchang – Sleeper ₮2.50M per person; Shenyang – Sleep value ₮2.73M / Sleep first ₮2.93M per person (no early start, a bed each, fly home); Shanghai – Sleeper ₮2.78M per person (Shanghai nonstop with cheap rooms ₮2.90M); Hong Kong – Budget ₮3.43M per person; EC Final – Train ₮3.14M per person. Shenyang and Nanchang are the cheap ones to pay yourselves.</t>
+          <t>Cheapest sleep-safe plans per person incl. fee, taxi, insurance, eSIM and 10% contingency: Shenyang – Budget ₮2.14M per person (soft sleeper before day 1); Shenyang – Overland home ₮2.37M per person (no early start, a bed each, overland home); Shenyang – Comfort ₮2.46M per person; Nanchang – Sleeper ₮2.50M per person; Shenyang – Sleep value ₮2.69M / Sleep first ₮2.89M per person (no early start, a bed each, fly home); Shanghai – Sleeper ₮2.78M per person (Shanghai nonstop with cheap rooms ₮2.90M); Hong Kong – Budget ₮3.43M per person; EC Final – Train ₮3.14M per person. Shenyang and Nanchang are the cheap ones to pay yourselves.</t>
         </is>
       </c>
     </row>
@@ -2444,7 +2444,7 @@
       </c>
       <c r="B43" s="74" t="inlineStr">
         <is>
-          <t>Sleep first, cheapest after (22 Oct prices): Air China 11:50 out (no 04:00 wake-up) + G153, two twin rooms for 3 nights, K28 hard seat + Air China 12:55 home. Sleep first (NEU International, 580 m, 9.7) ₮7.60M / ₮9.64M; Sleep value (Ji Hotel twins, ~15 min walk, 9.0) ₮7.00M / ₮9.04M; Overland home (Sleep value out, K1568 + 4652 night trains, jeep at Erenhot, UBTZ 275, home 18 Nov) ₮6.10M / ₮7.84M (3 / 4 ppl). Older: Comfort (MIAT 07:30, RiCH family room, K54) ₮6.18M / ₮8.04M; no sleepers: G-train Comfort ₮6.72M / ₮8.84M, G-train Budget ₮6.05M / ₮8.27M.</t>
+          <t>Sleep first, cheapest after (22 Oct prices): Air China 11:50 out (¥1,291 on Ctrip; no 04:00 wake-up) + G153, two twin rooms for 3 nights, K28 hard seat + Air China 12:55 home. Sleep first (NEU International, 580 m, 9.7) ₮7.47M / ₮9.47M; Sleep value (Ji Hotel twins, ~15 min walk, 9.0) ₮6.88M / ₮8.87M; Overland home (Sleep value out, K1568 + 4652 night trains, jeep at Erenhot, UBTZ 275, home 18 Nov) ₮5.97M / ₮7.67M (3 / 4 ppl). Older: Comfort (MIAT 07:30, RiCH family room, K54) ₮6.18M / ₮8.04M; no sleepers: G-train Comfort ₮6.72M / ₮8.84M, G-train Budget ₮6.05M / ₮8.27M.</t>
         </is>
       </c>
     </row>
@@ -2553,7 +2553,7 @@
       </c>
       <c r="B53" s="74" t="inlineStr">
         <is>
-          <t>Sources (10 Oct): Trip.com (flights and hotels, built-in browser), 12306 (official train fares), ChinaTicketOnline (timetable and sale-date check; 30–70% dearer than 12306, not used for booking), SlickTrip (MIAT / Spring fares; by 22 Oct it prices Air China, but $90–180 above Trip.com), UBTZ e-ticket (Zamyn-Uud → Ulaanbaatar train, 22 Oct).</t>
+          <t>Sources (10 Oct): Trip.com (flights and hotels, built-in browser), 12306 (official train fares), ChinaTicketOnline (timetable and sale-date check; 30–70% dearer than 12306, not used for booking), SlickTrip (MIAT / Spring fares; by 22 Oct it prices Air China, but $90–180 above Trip.com), UBTZ e-ticket (Zamyn-Uud → Ulaanbaatar train, 22 Oct), Ctrip / Kiwi / Google Flights (22 Oct cross-check of the Shenyang flights; Ctrip had the cheapest Air China fare).</t>
         </is>
       </c>
     </row>
@@ -17004,14 +17004,14 @@
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="E54:L54"/>
-    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="C44:L44"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
     <mergeCell ref="E53:L53"/>
     <mergeCell ref="B41:L41"/>
-    <mergeCell ref="C44:L44"/>
+    <mergeCell ref="B40:L40"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -18356,14 +18356,14 @@
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="E54:L54"/>
-    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="C44:L44"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
     <mergeCell ref="E53:L53"/>
     <mergeCell ref="B41:L41"/>
-    <mergeCell ref="C44:L44"/>
+    <mergeCell ref="B40:L40"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -18652,7 +18652,7 @@
       </c>
       <c r="H9" s="116" t="inlineStr">
         <is>
-          <t>No alarm before ~08:00 on any day before the contest (Air China 11:50 instead of MIAT 07:30, ~$49 pp more), three nights in the same room and a bed each (2 twin rooms, 38 m², 9.7). After the contest the cheapest: K28 hard seat + Air China 12:55. ₮2.93M per person (3 ppl).</t>
+          <t>No alarm before ~08:00 on any day before the contest (Air China 11:50 instead of MIAT 07:30, ¥195 ≈ ₮0.10M pp more on Ctrip), three nights in the same room and a bed each (2 twin rooms, 38 m², 9.7). After the contest the cheapest: K28 hard seat + Air China 12:55. ₮2.89M per person (3 ppl).</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       </c>
       <c r="H10" s="116" t="inlineStr">
         <is>
-          <t>Same timing and a bed each (2 twin rooms, King Koil mattresses, 9.0); smaller rooms and a ~15 min walk. ₮2.73M per person – ₮0.20M less than Sleep first.</t>
+          <t>Same timing and a bed each (2 twin rooms, King Koil mattresses, 9.0); smaller rooms and a ~15 min walk. ₮2.69M per person – ₮0.20M less than Sleep first.</t>
         </is>
       </c>
     </row>
@@ -18736,7 +18736,7 @@
       </c>
       <c r="H11" s="116" t="inlineStr">
         <is>
-          <t>Identical to Sleep value before the contest. After it: K1568 + 4652 hard sleepers, jeep across the border at Erenhot, UBTZ 275 platskart, home 18 Nov 09:20. ₮2.41M per person – the cheapest Shenyang plan without an early start or a sleeper before the contest.</t>
+          <t>Identical to Sleep value before the contest. After it: K1568 + 4652 hard sleepers, jeep across the border at Erenhot, UBTZ 275 platskart, home 18 Nov 09:20. ₮2.37M per person – the cheapest Shenyang plan without an early start or a sleeper before the contest.</t>
         </is>
       </c>
     </row>
@@ -20840,19 +20840,19 @@
     <mergeCell ref="E58:L58"/>
     <mergeCell ref="C45:L45"/>
     <mergeCell ref="B38:L38"/>
+    <mergeCell ref="E53:L53"/>
     <mergeCell ref="E59:L59"/>
     <mergeCell ref="E51:L51"/>
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="E54:L54"/>
-    <mergeCell ref="C44:L44"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
-    <mergeCell ref="E53:L53"/>
+    <mergeCell ref="B40:L40"/>
     <mergeCell ref="B41:L41"/>
-    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="C44:L44"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -22192,17 +22192,17 @@
     <mergeCell ref="E58:L58"/>
     <mergeCell ref="C45:L45"/>
     <mergeCell ref="B38:L38"/>
-    <mergeCell ref="E53:L53"/>
     <mergeCell ref="E59:L59"/>
     <mergeCell ref="E51:L51"/>
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="E54:L54"/>
+    <mergeCell ref="B40:L40"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
-    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="E53:L53"/>
     <mergeCell ref="B41:L41"/>
     <mergeCell ref="C44:L44"/>
   </mergeCells>
@@ -23549,14 +23549,14 @@
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="E54:L54"/>
-    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="C44:L44"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
     <mergeCell ref="E53:L53"/>
     <mergeCell ref="B41:L41"/>
-    <mergeCell ref="C44:L44"/>
+    <mergeCell ref="B40:L40"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -24901,14 +24901,14 @@
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="E54:L54"/>
-    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="C44:L44"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
     <mergeCell ref="E53:L53"/>
     <mergeCell ref="B41:L41"/>
-    <mergeCell ref="C44:L44"/>
+    <mergeCell ref="B40:L40"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -34849,7 +34849,7 @@
       <c r="K9" s="80" t="n"/>
       <c r="L9" s="80" t="n"/>
     </row>
-    <row r="10" ht="51" customHeight="1" s="56">
+    <row r="10" ht="60" customHeight="1" s="56">
       <c r="B10" s="111" t="inlineStr">
         <is>
           <t>Air China CA902 Ulaanbaatar 11:50 → Beijing Capital (PEK) 13:55, nonstop, checked bag included</t>
@@ -34864,11 +34864,11 @@
         <v>0.08680555555555555</v>
       </c>
       <c r="E10" s="85" t="n">
-        <v>203</v>
+        <v>1291</v>
       </c>
       <c r="F10" s="86" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CNY</t>
         </is>
       </c>
       <c r="G10" s="87">
@@ -34893,7 +34893,7 @@
       </c>
       <c r="L10" s="112" t="inlineStr">
         <is>
-          <t>Trip.com 22 Oct: US$203 pp. MIAT OM223 07:30 is US$170 on Trip.com / $154 on SlickTrip but means a ~04:00 wake-up; Air China lets everyone sleep normally for ~$33–49 pp more. SlickTrip prices Air China 11:50 at $316 (13 Nov) – book on Trip.com.</t>
+          <t>Ctrip 22 Oct: ¥1,291 pp incl. tax – cheapest of 5 sources (Kiwi $200, Trip.com $203, SlickTrip $316 on 13 Nov, Google Flights unpriced). MIAT OM223 07:30 is ¥1,096 on Ctrip / $167 Kiwi / $172 Google / $154 SlickTrip but means a ~04:00 wake-up. Ctrip needs a Ctrip account (Alipay or a foreign card); Trip.com $203 is the fallback.</t>
         </is>
       </c>
     </row>
@@ -34963,7 +34963,7 @@
       <c r="K12" s="80" t="n"/>
       <c r="L12" s="80" t="n"/>
     </row>
-    <row r="13" ht="63" customHeight="1" s="56">
+    <row r="13" ht="75" customHeight="1" s="56">
       <c r="B13" s="111" t="inlineStr">
         <is>
           <t>High-speed rail G153 Beijing Chaoyang 17:27 → Shenyang 20:04, 2nd class</t>
@@ -35007,7 +35007,7 @@
       </c>
       <c r="L13" s="112" t="inlineStr">
         <is>
-          <t>12306 (queried 22 Oct for 5 Nov; fares fixed): ¥369. ChinaTicketOnline confirms G153 on 12 Nov, on sale 29 Oct 10:00. Leaves 3 h 30 min after landing; if the flight is on time, change at the station to G141 16:00 → Shenyang North 18:29 (¥369). Later trains: G155 18:35 / G143 18:48 (¥369–383).</t>
+          <t>12306 (queried 22 Oct for 5 Nov; fares fixed): ¥369. ChinaTicketOnline confirms G153 on 12 Nov, on sale 29 Oct 10:00. Leaves 3 h 30 min after landing; if the flight is on time, change at the station to G141 16:00 → Shenyang North 18:29 (¥369). Later trains: G155 18:35 / G143 18:48 (¥369–383). Ctrip train list (22 Oct, for 12 Nov) shows the same fares; 12go.asia resells at ~$90 for 1st class.</t>
         </is>
       </c>
     </row>
@@ -35776,7 +35776,7 @@
       </c>
       <c r="B45" s="74" t="inlineStr">
         <is>
-          <t>Air China on Trip.com now; hotel now (free cancellation); G153 on 12306 at 10:00 on 29 Oct; K28 at 09:30 on 1 Nov.</t>
+          <t>Air China CA902 on Ctrip now (¥1,291; Trip.com $203 as fallback); hotel now (free cancellation); G153 on 12306 at 10:00 on 29 Oct; K28 at 09:30 on 1 Nov.</t>
         </is>
       </c>
     </row>
@@ -36488,7 +36488,7 @@
       <c r="K9" s="80" t="n"/>
       <c r="L9" s="80" t="n"/>
     </row>
-    <row r="10" ht="51" customHeight="1" s="56">
+    <row r="10" ht="60" customHeight="1" s="56">
       <c r="B10" s="111" t="inlineStr">
         <is>
           <t>Air China CA902 Ulaanbaatar 11:50 → Beijing Capital (PEK) 13:55, nonstop, checked bag included</t>
@@ -36503,11 +36503,11 @@
         <v>0.08680555555555555</v>
       </c>
       <c r="E10" s="85" t="n">
-        <v>203</v>
+        <v>1291</v>
       </c>
       <c r="F10" s="86" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CNY</t>
         </is>
       </c>
       <c r="G10" s="87">
@@ -36532,7 +36532,7 @@
       </c>
       <c r="L10" s="112" t="inlineStr">
         <is>
-          <t>Trip.com 22 Oct: US$203 pp. MIAT OM223 07:30 is US$170 on Trip.com / $154 on SlickTrip but means a ~04:00 wake-up; Air China lets everyone sleep normally for ~$33–49 pp more. SlickTrip prices Air China 11:50 at $316 (13 Nov) – book on Trip.com.</t>
+          <t>Ctrip 22 Oct: ¥1,291 pp incl. tax – cheapest of 5 sources (Kiwi $200, Trip.com $203, SlickTrip $316 on 13 Nov, Google Flights unpriced). MIAT OM223 07:30 is ¥1,096 on Ctrip / $167 Kiwi / $172 Google / $154 SlickTrip but means a ~04:00 wake-up. Ctrip needs a Ctrip account (Alipay or a foreign card); Trip.com $203 is the fallback.</t>
         </is>
       </c>
     </row>
@@ -36602,7 +36602,7 @@
       <c r="K12" s="80" t="n"/>
       <c r="L12" s="80" t="n"/>
     </row>
-    <row r="13" ht="63" customHeight="1" s="56">
+    <row r="13" ht="75" customHeight="1" s="56">
       <c r="B13" s="111" t="inlineStr">
         <is>
           <t>High-speed rail G153 Beijing Chaoyang 17:27 → Shenyang 20:04, 2nd class</t>
@@ -36646,7 +36646,7 @@
       </c>
       <c r="L13" s="112" t="inlineStr">
         <is>
-          <t>12306 (queried 22 Oct for 5 Nov; fares fixed): ¥369. ChinaTicketOnline confirms G153 on 12 Nov, on sale 29 Oct 10:00. Leaves 3 h 30 min after landing; if the flight is on time, change at the station to G141 16:00 → Shenyang North 18:29 (¥369). Later trains: G155 18:35 / G143 18:48 (¥369–383).</t>
+          <t>12306 (queried 22 Oct for 5 Nov; fares fixed): ¥369. ChinaTicketOnline confirms G153 on 12 Nov, on sale 29 Oct 10:00. Leaves 3 h 30 min after landing; if the flight is on time, change at the station to G141 16:00 → Shenyang North 18:29 (¥369). Later trains: G155 18:35 / G143 18:48 (¥369–383). Ctrip train list (22 Oct, for 12 Nov) shows the same fares; 12go.asia resells at ~$90 for 1st class.</t>
         </is>
       </c>
     </row>
@@ -37415,7 +37415,7 @@
       </c>
       <c r="B45" s="74" t="inlineStr">
         <is>
-          <t>Air China on Trip.com now; hotel now (free cancellation until 18:00 on 11 Nov, prepaid); G153 on 12306 at 10:00 on 29 Oct; K28 at 09:30 on 1 Nov.</t>
+          <t>Air China CA902 on Ctrip now (¥1,291; Trip.com $203 as fallback); hotel now (free cancellation until 18:00 on 11 Nov, prepaid); G153 on 12306 at 10:00 on 29 Oct; K28 at 09:30 on 1 Nov.</t>
         </is>
       </c>
     </row>
@@ -38127,7 +38127,7 @@
       <c r="K9" s="80" t="n"/>
       <c r="L9" s="80" t="n"/>
     </row>
-    <row r="10" ht="51" customHeight="1" s="56">
+    <row r="10" ht="60" customHeight="1" s="56">
       <c r="B10" s="111" t="inlineStr">
         <is>
           <t>Air China CA902 Ulaanbaatar 11:50 → Beijing Capital (PEK) 13:55, nonstop, checked bag included</t>
@@ -38142,11 +38142,11 @@
         <v>0.08680555555555555</v>
       </c>
       <c r="E10" s="85" t="n">
-        <v>203</v>
+        <v>1291</v>
       </c>
       <c r="F10" s="86" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CNY</t>
         </is>
       </c>
       <c r="G10" s="87">
@@ -38171,7 +38171,7 @@
       </c>
       <c r="L10" s="112" t="inlineStr">
         <is>
-          <t>Trip.com 22 Oct: US$203 pp. MIAT OM223 07:30 is US$170 on Trip.com / $154 on SlickTrip but means a ~04:00 wake-up; Air China lets everyone sleep normally for ~$33–49 pp more. SlickTrip prices Air China 11:50 at $316 (13 Nov) – book on Trip.com.</t>
+          <t>Ctrip 22 Oct: ¥1,291 pp incl. tax – cheapest of 5 sources (Kiwi $200, Trip.com $203, SlickTrip $316 on 13 Nov, Google Flights unpriced). MIAT OM223 07:30 is ¥1,096 on Ctrip / $167 Kiwi / $172 Google / $154 SlickTrip but means a ~04:00 wake-up. Ctrip needs a Ctrip account (Alipay or a foreign card); Trip.com $203 is the fallback.</t>
         </is>
       </c>
     </row>
@@ -38193,7 +38193,7 @@
       <c r="K11" s="80" t="n"/>
       <c r="L11" s="80" t="n"/>
     </row>
-    <row r="12" ht="63" customHeight="1" s="56">
+    <row r="12" ht="75" customHeight="1" s="56">
       <c r="B12" s="111" t="inlineStr">
         <is>
           <t>High-speed rail G153 Beijing Chaoyang 17:27 → Shenyang 20:04, 2nd class</t>
@@ -38237,7 +38237,7 @@
       </c>
       <c r="L12" s="112" t="inlineStr">
         <is>
-          <t>12306 (queried 22 Oct for 5 Nov; fares fixed): ¥369. ChinaTicketOnline confirms G153 on 12 Nov, on sale 29 Oct 10:00. Leaves 3 h 30 min after landing; if the flight is on time, change at the station to G141 16:00 → Shenyang North 18:29 (¥369). Later trains: G155 18:35 / G143 18:48 (¥369–383).</t>
+          <t>12306 (queried 22 Oct for 5 Nov; fares fixed): ¥369. ChinaTicketOnline confirms G153 on 12 Nov, on sale 29 Oct 10:00. Leaves 3 h 30 min after landing; if the flight is on time, change at the station to G141 16:00 → Shenyang North 18:29 (¥369). Later trains: G155 18:35 / G143 18:48 (¥369–383). Ctrip train list (22 Oct, for 12 Nov) shows the same fares; 12go.asia resells at ~$90 for 1st class.</t>
         </is>
       </c>
     </row>
@@ -39150,7 +39150,7 @@
       </c>
       <c r="B47" s="74" t="inlineStr">
         <is>
-          <t>Air China on Trip.com now; hotel now; G153 on 12306 at 10:00 on 29 Oct; K1568 at 09:30 on 1 Nov; 4652 at 14:00 on 2 Nov; UBTZ 275 on eticket.ubtz.mn (on sale now).</t>
+          <t>Air China CA902 on Ctrip now (¥1,291; Trip.com $203 as fallback); hotel now; G153 on 12306 at 10:00 on 29 Oct; K1568 at 09:30 on 1 Nov; 4652 at 14:00 on 2 Nov; UBTZ 275 on eticket.ubtz.mn (on sale now).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Shenyang: no-sleep-loss way out 10–13 Nov (Hohhot + Spring ₮751k pp)
Ctrip, Trip.com, SlickTrip and ChinaTicketOnline checked on 27 Oct.
Cheapest no-sleep-loss route: Air China CA758 + Spring 9C6782 via
Hohhot on 10 or 12 Nov, two tickets, ¥1,401 pp. Spring fare on the
Hohhot + Spring sheet now includes the ¥140 airport fee and fuel
surcharge (¥290 -> ¥360); the 20 kg bag fare (+¥120) is confirmed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ICPC_Single_Contest_Plans.xlsx
+++ b/ICPC_Single_Contest_Plans.xlsx
@@ -2896,7 +2896,7 @@
       </c>
       <c r="B51" s="74" t="inlineStr">
         <is>
-          <t>Sleep first, cheapest after (22 Oct prices): Air China 11:50 out (¥1,291 on Ctrip; no 04:00 wake-up) + G153, two twin rooms for 3 nights, K28 hard seat + Air China 12:55 home. Sleep first (NEU International, 580 m, 9.7) ₮7.47M / ₮9.47M; Sleep value (Ji Hotel twins, ~15 min walk, 9.0) ₮6.88M / ₮8.87M; Overland home (Sleep value out, K1568 + 4652 night trains, jeep at Erenhot, UBTZ 275, home 18 Nov) ₮5.97M / ₮7.67M (3 / 4 ppl). Older: Comfort (MIAT 07:30, RiCH family room, K54) ₮6.18M / ₮8.04M; no sleepers: G-train Comfort ₮6.72M / ₮8.84M, G-train Budget ₮6.05M / ₮8.27M. Cheap way out instead (22 Oct; sheet 'Shenyang – Way out', rest of the trip as Sleep value): Overland out (UBTZ 276 + jeep + 4654 + T301, seats) ₮3.96M / ₮5.19M, per person ₮1.70M; with berths ₮1.79M per person; Hunnu Daxing + K341 ₮2.08M; MIAT 13 Nov + K341 ₮2.10M; Hunnu Erenhot ₮2.14M; Manzhouli seats ₮2.27M (sleep OK); Hohhot red-eye ₮2.34M (WATCH). Hohhot + Spring (Air China CA758 + Spring 9C6782, two tickets, no night train, BEST) ₮6.43M / ₮8.29M, ₮2.55M per person – ₮0.15M less than Sleep value. All others are POOR for sleep: a seated night right before day 1.</t>
+          <t>Sleep first, cheapest after (22 Oct prices): Air China 11:50 out (¥1,291 on Ctrip; no 04:00 wake-up) + G153, two twin rooms for 3 nights, K28 hard seat + Air China 12:55 home. Sleep first (NEU International, 580 m, 9.7) ₮7.47M / ₮9.47M; Sleep value (Ji Hotel twins, ~15 min walk, 9.0) ₮6.88M / ₮8.87M; Overland home (Sleep value out, K1568 + 4652 night trains, jeep at Erenhot, UBTZ 275, home 18 Nov) ₮5.97M / ₮7.67M (3 / 4 ppl). Older: Comfort (MIAT 07:30, RiCH family room, K54) ₮6.18M / ₮8.04M; no sleepers: G-train Comfort ₮6.72M / ₮8.84M, G-train Budget ₮6.05M / ₮8.27M. Cheap way out instead (22 Oct; sheet 'Shenyang – Way out', rest of the trip as Sleep value): Overland out (UBTZ 276 + jeep + 4654 + T301, seats) ₮3.96M / ₮5.19M, per person ₮1.70M; with berths ₮1.79M per person; Hunnu Daxing + K341 ₮2.08M; MIAT 13 Nov + K341 ₮2.10M; Hunnu Erenhot ₮2.14M; Manzhouli seats ₮2.27M (sleep OK); Hohhot red-eye ₮2.34M (WATCH). Hohhot + Spring (Air China CA758 + Spring 9C6782, two tickets, no night train, BEST) ₮6.56M / ₮8.46M, ₮2.59M per person – ₮0.11M less than Sleep value (27 Oct: Spring ¥220 fare + ¥140 airport fee and fuel surcharge; 20 kg bag +¥120). All others are POOR for sleep: a seated night right before day 1.</t>
         </is>
       </c>
     </row>
@@ -14704,7 +14704,7 @@
     <row r="2" ht="15" customHeight="1" s="56">
       <c r="A2" s="62" t="inlineStr">
         <is>
-          <t>No early alarm and no night train, like 'Sleep value', but cheaper: Air China to Hohhot and a ¥290 Spring flight to Shenyang (two tickets); three nights in Ji Hotel twin rooms; K28 seat + Air China home.</t>
+          <t>No early alarm and no night train, like 'Sleep value', but cheaper: Air China to Hohhot and a ¥360 Spring flight to Shenyang (¥220 + taxes, two tickets); three nights in Ji Hotel twin rooms; K28 seat + Air China home.</t>
         </is>
       </c>
     </row>
@@ -14872,7 +14872,7 @@
       </c>
       <c r="L10" s="112" t="inlineStr">
         <is>
-          <t>Ctrip 22 Oct: ¥1,011 on 12 Nov (SlickTrip $268). Separate ticket from the Spring flight: a 4 h 25 min self-transfer in Hohhot (immigration, collect bags, check in again).</t>
+          <t>Ctrip 27 Oct: ¥1,011 incl. taxes on every day 10–13 Nov (Trip.com ¥1,009; 22 Oct also ¥1,011; SlickTrip $268). Separate ticket from the Spring flight: a 4 h 25 min self-transfer in Hohhot (immigration, collect bags, check in again).</t>
         </is>
       </c>
     </row>
@@ -14891,7 +14891,7 @@
         <v>0.09027777777777778</v>
       </c>
       <c r="E11" s="85" t="n">
-        <v>290</v>
+        <v>360</v>
       </c>
       <c r="F11" s="86" t="inlineStr">
         <is>
@@ -14920,7 +14920,7 @@
       </c>
       <c r="L11" s="112" t="inlineStr">
         <is>
-          <t>Ctrip 22 Oct: ¥290 (10 Nov ¥240, 11 / 13 Nov ¥400); SlickTrip $65. Only a 7 kg cabin bag included. Booked apart from CA758 – Ctrip's combined UB → SHE ticket is ¥1,561 and Kiwi's $237.</t>
+          <t>Ctrip 27 Oct: fare ¥220 (10 and 12 Nov; 11 / 13 Nov ¥400) + ¥50 airport fee + ¥90 fuel surcharge (domestic &gt; 800 km from 10 Oct 2026) = ¥360. Trip.com shows CNY 360 incl. taxes on 10 Nov (12 Nov only a CNY 520 bundle). The 22 Oct ¥290 left the taxes out. Only a 7 kg cabin bag (20×30×40 cm). Booked apart from CA758 – one ticket UB → SHE is ¥1,531 on Ctrip / ¥1,528 on Trip.com (12 Nov).</t>
         </is>
       </c>
     </row>
@@ -14936,7 +14936,7 @@
         </is>
       </c>
       <c r="D12" s="84" t="n"/>
-      <c r="E12" s="113" t="n">
+      <c r="E12" s="85" t="n">
         <v>120</v>
       </c>
       <c r="F12" s="86" t="inlineStr">
@@ -14952,7 +14952,7 @@
         <f>E12*G12*IF(F12="USD",Compare!$B$8,IF(F12="CNY",Compare!$B$9,IF(F12="HKD",Compare!$B$10,1)))</f>
         <v/>
       </c>
-      <c r="I12" s="114">
+      <c r="I12" s="89">
         <f>E12</f>
         <v/>
       </c>
@@ -14966,7 +14966,7 @@
       </c>
       <c r="L12" s="112" t="inlineStr">
         <is>
-          <t>ASSUMPTION ~¥100–150 per bag on Spring domestic routes; check ch.com when booking. Cabin bags only saves it.</t>
+          <t>Ctrip 27 Oct: the 9C6782 fare with a 20 kg checked bag is ¥340 vs ¥220 without (+¥120, same taxes). Only people who check a bag need it.</t>
         </is>
       </c>
     </row>
@@ -15789,7 +15789,7 @@
       </c>
       <c r="B45" s="74" t="inlineStr">
         <is>
-          <t>Two separate tickets: if CA758 is more than ~3 h late the ¥290 Spring ticket is lost (fallback Air China CA8179 Hohhot 08:55 next morning ¥620 + a Hohhot hotel). Spring includes only a 7 kg cabin bag (bag fee assumed). Arrive ~22:15 instead of 20:30.</t>
+          <t>Two separate tickets: if CA758 is more than ~3 h late the ¥360 Spring ticket is lost (fallback Air China CA8179 Hohhot 08:55 next morning ¥620 + a Hohhot hotel). Spring includes only a 7 kg cabin bag (a 20 kg bag fare is ¥120 more). Arrive ~22:15 instead of 20:30.</t>
         </is>
       </c>
     </row>
@@ -32878,19 +32878,19 @@
     <mergeCell ref="E58:L58"/>
     <mergeCell ref="C45:L45"/>
     <mergeCell ref="B38:L38"/>
-    <mergeCell ref="E53:L53"/>
     <mergeCell ref="E59:L59"/>
     <mergeCell ref="E51:L51"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="E54:L54"/>
+    <mergeCell ref="C44:L44"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
+    <mergeCell ref="E53:L53"/>
+    <mergeCell ref="B41:L41"/>
     <mergeCell ref="B40:L40"/>
-    <mergeCell ref="B41:L41"/>
-    <mergeCell ref="C44:L44"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -34230,19 +34230,19 @@
     <mergeCell ref="E58:L58"/>
     <mergeCell ref="C45:L45"/>
     <mergeCell ref="B38:L38"/>
-    <mergeCell ref="E53:L53"/>
     <mergeCell ref="E59:L59"/>
     <mergeCell ref="E51:L51"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="E54:L54"/>
+    <mergeCell ref="C44:L44"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
+    <mergeCell ref="E53:L53"/>
+    <mergeCell ref="B41:L41"/>
     <mergeCell ref="B40:L40"/>
-    <mergeCell ref="B41:L41"/>
-    <mergeCell ref="C44:L44"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -35582,17 +35582,17 @@
     <mergeCell ref="E58:L58"/>
     <mergeCell ref="C45:L45"/>
     <mergeCell ref="B38:L38"/>
+    <mergeCell ref="E53:L53"/>
     <mergeCell ref="E59:L59"/>
     <mergeCell ref="E51:L51"/>
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="E54:L54"/>
-    <mergeCell ref="B40:L40"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
-    <mergeCell ref="E53:L53"/>
+    <mergeCell ref="B40:L40"/>
     <mergeCell ref="B41:L41"/>
     <mergeCell ref="C44:L44"/>
   </mergeCells>
@@ -38533,14 +38533,14 @@
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="E54:L54"/>
-    <mergeCell ref="C44:L44"/>
+    <mergeCell ref="B40:L40"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
     <mergeCell ref="E53:L53"/>
     <mergeCell ref="B41:L41"/>
-    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="C44:L44"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -39880,19 +39880,19 @@
     <mergeCell ref="E58:L58"/>
     <mergeCell ref="C45:L45"/>
     <mergeCell ref="B38:L38"/>
-    <mergeCell ref="E53:L53"/>
     <mergeCell ref="E59:L59"/>
     <mergeCell ref="E51:L51"/>
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="E54:L54"/>
+    <mergeCell ref="C44:L44"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
+    <mergeCell ref="E53:L53"/>
+    <mergeCell ref="B41:L41"/>
     <mergeCell ref="B40:L40"/>
-    <mergeCell ref="B41:L41"/>
-    <mergeCell ref="C44:L44"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -41232,19 +41232,19 @@
     <mergeCell ref="E58:L58"/>
     <mergeCell ref="C45:L45"/>
     <mergeCell ref="B38:L38"/>
-    <mergeCell ref="E53:L53"/>
     <mergeCell ref="E59:L59"/>
     <mergeCell ref="E51:L51"/>
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="B39:L39"/>
     <mergeCell ref="E54:L54"/>
+    <mergeCell ref="C44:L44"/>
     <mergeCell ref="E55:L55"/>
     <mergeCell ref="E52:L52"/>
     <mergeCell ref="C46:L46"/>
     <mergeCell ref="C47:L47"/>
+    <mergeCell ref="E53:L53"/>
+    <mergeCell ref="B41:L41"/>
     <mergeCell ref="B40:L40"/>
-    <mergeCell ref="B41:L41"/>
-    <mergeCell ref="C44:L44"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>